<commit_message>
Update events: 2026-05-21 23:41 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -1769,10 +1769,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -1809,12 +1809,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>05/22/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1824,24 +1824,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>KESHA – The Freedom Tour</t>
+          <t>NIALL HORAN – Dinner Party Live On Tour</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/kesha/</t>
+          <t>https://thekiaforum.com/event/niall-horan/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>05/24/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1851,24 +1851,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>RUSH – Fifty Something</t>
+          <t>KESHA – The Freedom Tour</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rush/</t>
+          <t>https://thekiaforum.com/event/kesha/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1878,24 +1878,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
+          <t>RUSH – Fifty Something</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/ariana-grande-2/</t>
+          <t>https://thekiaforum.com/event/rush/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>06/09/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1905,24 +1905,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MADISON BEER – the locket tour</t>
+          <t>RUSH – Fifty Something</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/madison-beer/</t>
+          <t>https://thekiaforum.com/event/rush-2/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>06/11/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1932,24 +1932,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PALOMAZO NORTEÑO – CLASE MAESTRA TOUR</t>
+          <t>RUSH – Fifty Something</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/palomazo-norteno/</t>
+          <t>https://thekiaforum.com/event/rush-3/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>06/13/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1959,24 +1959,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>A$AP ROCKY – Don't Be Dumb World Tour</t>
+          <t>RUSH – Fifty Something</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/aap-rocky/</t>
+          <t>https://thekiaforum.com/event/rush-4/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>06/17/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1986,24 +1986,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ROSALÍA – LUX TOUR 2026</t>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rosalia/</t>
+          <t>https://thekiaforum.com/event/ariana-grande-2/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>06/19/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2013,24 +2013,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>HILARY DUFF – the lucky me tour</t>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/hilary-duff/</t>
+          <t>https://thekiaforum.com/event/ariana-grande/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>06/20/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2040,24 +2040,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>5 SECONDS OF SUMMER – EVERYONE’S A STAR! World Tour</t>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/5-seconds-of-summer/</t>
+          <t>https://thekiaforum.com/event/ariana-grande-3/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>06/24/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2067,24 +2067,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>YOUNG THE GIANT – Victory Garden Tour</t>
+          <t>MADISON BEER – the locket tour</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/young-the-giant/</t>
+          <t>https://thekiaforum.com/event/madison-beer/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>06/26/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2094,24 +2094,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EVANESCENCE</t>
+          <t>PALOMAZO NORTEÑO – CLASE MAESTRA TOUR</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/evanescence/</t>
+          <t>https://thekiaforum.com/event/palomazo-norteno/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>06/27/2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2121,12 +2121,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MOTIONLESS IN WHITE – The Sweat and Blood Tour</t>
+          <t>A$AP ROCKY – Don't Be Dumb World Tour</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/motionless-in-white/</t>
+          <t>https://thekiaforum.com/event/aap-rocky/</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>06/29/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2148,24 +2148,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>IVE – WORLD TOUR [SHOW WHAT I AM] IN LOS ANGELES</t>
+          <t>ROSALÍA – LUX TOUR 2026</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/ive/</t>
+          <t>https://thekiaforum.com/event/rosalia/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>07/01/2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2175,24 +2175,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>RÜFÜS DU SOL</t>
+          <t>ROSALÍA – LUX TOUR 2026</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol/</t>
+          <t>https://thekiaforum.com/event/rosalia-2/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>07/08/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2202,24 +2202,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>RÜFÜS DU SOL – with Ben Böhmer</t>
+          <t>HILARY DUFF – the lucky me tour</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol-5/</t>
+          <t>https://thekiaforum.com/event/hilary-duff/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>07/09/2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2229,24 +2229,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>MELANIE MARTINEZ – HADES: THE SACRIFICE</t>
+          <t>HILARY DUFF – the lucky me tour</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/melanie-martinez/</t>
+          <t>https://thekiaforum.com/event/hilary-duff-2/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>07/11/2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2256,24 +2256,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>OMAR COURTZ – POR SI MAÑANA NO ESTOY USA TOUR</t>
+          <t>5 SECONDS OF SUMMER – EVERYONE’S A STAR! World Tour</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/omar-courtz/</t>
+          <t>https://thekiaforum.com/event/5-seconds-of-summer/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>07/17/2026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2283,24 +2283,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CHICAGO &amp; STYX – The Windy Cities Tour - All The Hits... Your Kind of Tour</t>
+          <t>YOUNG THE GIANT – Victory Garden Tour</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/chicago-styx/</t>
+          <t>https://thekiaforum.com/event/young-the-giant/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>07/18/2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2310,24 +2310,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>JOHNNY BLUE SKIES &amp; THE DARK CLOUDS – Mutiny for the Masses 2026 Tour</t>
+          <t>EVANESCENCE</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/johnny-blue-skies-the-dark-clouds/</t>
+          <t>https://thekiaforum.com/event/evanescence/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>07/31/2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2337,24 +2337,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>SODA STEREO – ECOS TOUR</t>
+          <t>MOTIONLESS IN WHITE – The Sweat and Blood Tour</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/soda-stereo/</t>
+          <t>https://thekiaforum.com/event/motionless-in-white/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>08/01/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2364,24 +2364,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>ROBYN – The Sexistential Tour</t>
+          <t>IVE – WORLD TOUR [SHOW WHAT I AM] IN LOS ANGELES</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/robyn/</t>
+          <t>https://thekiaforum.com/event/ive/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>08/06/2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2391,24 +2391,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>LILY ALLEN – Lily Allen Performs West End Girl</t>
+          <t>RÜFÜS DU SOL</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/lily-allen/</t>
+          <t>https://thekiaforum.com/event/rufus-du-sol/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>08/07/2026</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2418,24 +2418,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>BILLY STRINGS</t>
+          <t>RÜFÜS DU SOL</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/billy-strings-3/</t>
+          <t>https://thekiaforum.com/event/rufus-du-sol-3/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>08/11/2026</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2445,24 +2445,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>DISNEY DESCENDANTS, ZOMBIES &amp; CAMP ROCK: WORLDS COLLIDE CONCERT TOUR</t>
+          <t>RÜFÜS DU SOL</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/worlds-collide-concert-tour/</t>
+          <t>https://thekiaforum.com/event/rufus-du-sol-2/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>08/12/2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2472,24 +2472,24 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
+          <t>RÜFÜS DU SOL</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/mumford-sons/</t>
+          <t>https://thekiaforum.com/event/rufus-du-sol-4/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>08/13/2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2499,24 +2499,24 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+          <t>RÜFÜS DU SOL – with Ben Böhmer</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/the-neighbourhood/</t>
+          <t>https://thekiaforum.com/event/rufus-du-sol-5/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>08/14/2026</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2526,24 +2526,24 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>SOMBR – You Are The Reason Tour</t>
+          <t>MELANIE MARTINEZ – HADES: THE SACRIFICE</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/sombr/</t>
+          <t>https://thekiaforum.com/event/melanie-martinez/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>08/21/2026</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2553,24 +2553,24 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>JUANES</t>
+          <t>OMAR COURTZ – POR SI MAÑANA NO ESTOY USA TOUR</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/juanes/</t>
+          <t>https://thekiaforum.com/event/omar-courtz/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2580,24 +2580,24 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>MONSTA X – 2026 MONSTA X WORLD TOUR [THE X : NEXUS] IN LOS ANGELES</t>
+          <t>CHICAGO &amp; STYX – The Windy Cities Tour - All The Hits... Your Kind of Tour</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/monsta-x/</t>
+          <t>https://thekiaforum.com/event/chicago-styx/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>09/11/2026</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2607,24 +2607,24 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>DOJA CAT – Tour Ma Vie World Tour</t>
+          <t>JOHNNY BLUE SKIES &amp; THE DARK CLOUDS – Mutiny for the Masses 2026 Tour</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/doja-cat/</t>
+          <t>https://thekiaforum.com/event/johnny-blue-skies-the-dark-clouds/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>09/12/2026</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2634,24 +2634,24 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>GORILLAZ – The Mountain Tour</t>
+          <t>SODA STEREO – ECOS TOUR</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/gorillaz-2/</t>
+          <t>https://thekiaforum.com/event/soda-stereo/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>09/23/2026</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2661,24 +2661,24 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>DON OMAR – The Last King World Tour</t>
+          <t>ROBYN – The Sexistential Tour</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/don-omar/</t>
+          <t>https://thekiaforum.com/event/robyn/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>09/24/2026</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2688,24 +2688,24 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>MON LAFERTE – Femme Fatale Tour</t>
+          <t>ROBYN – The Sexistential Tour</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/mon-laferte/</t>
+          <t>https://thekiaforum.com/event/robyn-2/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>09/25/2026</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2715,24 +2715,24 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>THE SMASHING PUMPKINS – The Rats In A Cage Tour</t>
+          <t>LILY ALLEN – Lily Allen Performs West End Girl</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/the-smashing-pumpkins/</t>
+          <t>https://thekiaforum.com/event/lily-allen/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>09/26/2026</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2742,24 +2742,24 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>SLAYER – Reign in Blood 40th Anniversary</t>
+          <t>BILLY STRINGS</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/slayer/</t>
+          <t>https://thekiaforum.com/event/billy-strings-3/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>09/30/2026</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2769,24 +2769,24 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>RAWAYANA – ¿Dónde es el after? World Tour</t>
+          <t>DISNEY DESCENDANTS, ZOMBIES &amp; CAMP ROCK: WORLDS COLLIDE CONCERT TOUR</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rawayana/</t>
+          <t>https://thekiaforum.com/event/worlds-collide-concert-tour/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2796,24 +2796,24 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>TEDDY SWIMS – The UGLY Tour</t>
+          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/teddy-swims/</t>
+          <t>https://thekiaforum.com/event/mumford-sons/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2823,12 +2823,417 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>NIALL HORAN – Dinner Party Live On Tour</t>
+          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/niall-horan/</t>
+          <t>https://thekiaforum.com/event/mumford-sons-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood/</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>SOMBR – You Are The Reason Tour</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/sombr/</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>10/16/2026</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>JUANES</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/juanes/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>10/20/2026</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>MONSTA X – 2026 MONSTA X WORLD TOUR [THE X : NEXUS] IN LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/monsta-x/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>10/22/2026</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>DOJA CAT – Tour Ma Vie World Tour</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/doja-cat/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>GORILLAZ – The Mountain Tour</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/gorillaz-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>11/06/2026</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>DON OMAR – The Last King World Tour</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/don-omar/</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>11/07/2026</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>MON LAFERTE – Femme Fatale Tour</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/mon-laferte/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>11/12/2026</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>THE SMASHING PUMPKINS – The Rats In A Cage Tour</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-smashing-pumpkins/</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>11/13/2026</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>SLAYER – Reign in Blood 40th Anniversary</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/slayer/</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>11/14/2026</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>SLAYER – Reign in Blood 40th Anniversary</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/slayer-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>11/15/2026</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>RAWAYANA – ¿Dónde es el after? World Tour</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rawayana/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>11/18/2026</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>TEDDY SWIMS – The UGLY Tour</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/teddy-swims/</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>12/05/2026</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood-3/</t>
         </is>
       </c>
     </row>
@@ -2872,6 +3277,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update events: 2026-05-21 23:57 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -437,11 +437,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
@@ -477,12 +477,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>06/12/2026</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Friday</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -504,12 +504,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>06/15/2026</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Monday</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -531,12 +531,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>06/18/2026</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Thursday</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -558,12 +558,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>06/21/2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Sunday</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -585,66 +585,66 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>06/25/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Book Your Flight to SoFi Stadium! – Book today with American Airlines</t>
+          <t>Türkiye vs. USA – FIFA World Cup 26™</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/american-airlines</t>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-turkiye-vs-usa</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06/25/2026</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>06/28/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>12:00 PM</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Türkiye vs. USA – FIFA World Cup 26™</t>
+          <t>Round of 32: TBD vs. TBD – FIFA World Cup 26™</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-turkiye-vs-usa</t>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-roundof32-june28</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06/28/2026</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>07/02/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -659,19 +659,19 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-roundof32-june28</t>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-roundof32-july2</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -681,78 +681,78 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Round of 32: TBD vs. TBD – FIFA World Cup 26™</t>
+          <t>Quarterfinals: TBD vs. TBD – FIFA World Cup 26™</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-roundof32-july2</t>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-quarterfinal-july10</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>08/08/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12:00 PM</t>
+          <t>5:30 PM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Quarterfinals: TBD vs. TBD – FIFA World Cup 26™</t>
+          <t>Ed Sheeran – With Myles Smith, Sigrid, Aaron Rowe</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-quarterfinal-july10</t>
+          <t>https://www.sofistadium.com/events/detail/ed-sheeran-august-8-2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>08/08/2026</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>08/14/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>5:30 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Ed Sheeran – With Myles Smith, Sigrid, Aaron Rowe</t>
+          <t>KAROL G - VIAJANDO POR EL MUNDO TROPITOUR</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/ed-sheeran-august-8-2026</t>
+          <t>https://www.sofistadium.com/events/detail/karol-g-august-14</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08/14/2026</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>08/15/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -766,33 +766,6 @@
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/karol-g-august-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>08/15/2026</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>KAROL G - VIAJANDO POR EL MUNDO TROPITOUR</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>https://www.sofistadium.com/events/detail/karol-g-august-15</t>
         </is>
@@ -811,7 +784,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3521,68 +3493,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Time</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Event Name</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>No events found</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -3616,27 +3533,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>05/21/2026</t>
+          <t>05/29/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Romeo Santos &amp; Prince Royce – Mejor Tarde Que Nunca Tour 2026</t>
+          <t>PUBLIC TOURS</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/romeosantosprinceroyce052126</t>
+          <t>https://www.rosebowlstadium.com/events/details/614/public-tours</t>
         </is>
       </c>
     </row>
@@ -3648,22 +3565,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>05/22/2026</t>
+          <t>05/29/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>11:00 AM</t>
+          <t>6:00 PM</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Crypto.com Arena VIP Tours presented by Delta Air Lines – Click ‘Buy Tickets’ to See All Available Tour Times</t>
+          <t>VIP Fan Day MexTour Live</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/cryptocom-arena-vip-tours-presented-by-delta-air-lines-1450890</t>
+          <t>https://www.rosebowlstadium.com/events/details/646/vip-fan-day-mextour-live</t>
         </is>
       </c>
     </row>
@@ -3675,22 +3592,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>05/23/2026</t>
+          <t>05/30/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>11:00 AM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Crypto.com Arena VIP Tours presented by Delta Air Lines – Click ‘Buy Tickets’ to See All Available Tour Times</t>
+          <t>Mexico vs Australia</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/crypto-com-arena-vip-tours-presented-by-delta-air-lines-1450893</t>
+          <t>https://www.rosebowlstadium.com/events/details/635/mexico-vs-australia</t>
         </is>
       </c>
     </row>
@@ -3702,49 +3619,49 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>05/24/2026</t>
+          <t>06/14/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>11:00 AM</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Crypto.com Arena VIP Tours presented by Delta Air Lines – Click ‘Buy Tickets’ to See All Available Tour Times</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/crypto-com-arena-vip-tours-presented-by-delta-air-lines-1450905</t>
+          <t>https://www.rosebowlstadium.com/events/details/601/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05/26/2026</t>
+          <t>06/26/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Crypto.com Arena VIP Tours presented by Delta Air Lines – Click ‘Buy Tickets’ to See All Available Tour Times</t>
+          <t>PUBLIC TOURS</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/crypto-com-arena-vip-tours-presented-by-delta-air-lines-1450909</t>
+          <t>https://www.rosebowlstadium.com/events/details/615/public-tours</t>
         </is>
       </c>
     </row>
@@ -3756,22 +3673,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05/29/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11:00 AM</t>
+          <t>3:00 PM</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Crypto.com Arena VIP Tours presented by Delta Air Lines – Click ‘Buy Tickets’ to See All Available Tour Times</t>
+          <t>Foodieland</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/crypto-com-arena-vip-tours-presented-by-delta-air-lines-1450912</t>
+          <t>https://www.rosebowlstadium.com/events/details/637/foodieland</t>
         </is>
       </c>
     </row>
@@ -3783,7 +3700,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05/30/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3793,12 +3710,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Crypto.com Arena VIP Tours presented by Delta Air Lines – Click ‘Buy Tickets’ to See All Available Tour Times</t>
+          <t>Foodieland</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/crypto-com-arena-vip-tours-presented-by-delta-air-lines-1450914</t>
+          <t>https://www.rosebowlstadium.com/events/details/638/foodieland</t>
         </is>
       </c>
     </row>
@@ -3810,49 +3727,805 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05/31/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11:00 AM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Crypto.com Arena VIP Tours presented by Delta Air Lines – Click ‘Buy Tickets’ to See All Available Tour Times</t>
+          <t>Foodieland</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/crypto-com-arena-vip-tours-presented-by-delta-air-lines-1450915</t>
+          <t>https://www.rosebowlstadium.com/events/details/639/foodieland</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06/02/2026</t>
+          <t>07/11/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>5:15 PM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Crypto.com Arena VIP Tours presented by Delta Air Lines – Click ‘Buy Tickets’ to See All Available Tour Times</t>
+          <t>DRUM CORPS AT THE ROSE BOWL</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/crypto-com-arena-vip-tours-presented-by-delta-air-lines-1434456</t>
+          <t>https://www.rosebowlstadium.com/events/details/644/drum-corps-at-the-rose-bowl</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>07/12/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>5:00 AM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ROSE BOWL FLEA MARKET</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/602/rose-bowl-flea-market</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>07/31/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PUBLIC TOURS</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/616/public-tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08/08/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Head in the Clouds</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/642/head-in-the-clouds</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>5:00 AM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ROSE BOWL FLEA MARKET</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/603/rose-bowl-flea-market</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>08/15/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>NOAH KAHAN - THE GREAT DIVIDE TOUR</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/633/noah-kahan-the-great-divide-tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>08/22/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Just Like Heaven</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/640/just-like-heaven</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>08/28/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>PUBLIC TOURS</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/617/public-tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>GUNS N’ ROSES</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/579/guns-n'-roses</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>09/12/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>SAN DIEGO STATE VS UCLA</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/594/san-diego-state-vs-ucla</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>09/13/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>5:00 AM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ROSE BOWL FLEA MARKET</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/604/rose-bowl-flea-market</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>09/19/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>PURDUE VS UCLA</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/595/purdue-vs-ucla</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>09/25/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>PUBLIC TOURS</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/618/public-tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>10/11/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>5:00 AM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ROSE BOWL FLEA MARKET</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/605/rose-bowl-flea-market</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>10/17/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>WISCONSIN VS UCLA</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/627/wisconsin-vs-ucla</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>MICHIGAN STATE VS UCLA</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/628/michigan-state-vs-ucla</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>10/30/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>PUBLIC TOURS</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/620/public-tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>10/31/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>NEVADA VS UCLA</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/629/nevada-vs-ucla</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>5:00 AM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ROSE BOWL FLEA MARKET</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/606/rose-bowl-flea-market</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>11/13/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>ILLINOIS VS UCLA</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/630/illinois-vs-ucla</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>11/27/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>PUBLIC TOURS</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/622/public-tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>11/28/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>USC VS UCLA</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>12/13/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>5:00 AM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>ROSE BOWL FLEA MARKET</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>12/26/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>HOLIDAY TOURS</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>12/27/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>HOLIDAY TOURS</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>12/28/2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>HOLIDAY TOURS</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>01/02/2027</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>HOLIDAY TOURS</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>01/02/2027</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>HOLIDAY TOURS (duplicate)</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/647/holiday-tours-(duplicate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>01/17/2027</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Rose Bowl Half Marathon &amp; 5K</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/626/rose-bowl-half-marathon-and-5k</t>
         </is>
       </c>
     </row>
@@ -3867,6 +4540,112 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Event Name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>05/21/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Romeo Santos &amp; Prince Royce – Mejor Tarde Que Nunca Tour 2026</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/romeosantosprinceroyce052126</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update events: 2026-05-22 00:02 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -437,14 +437,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,314 +477,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>06/12/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>USA vs. Paraguay – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-usa-paraguay</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>06/15/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>IR Iran vs. New Zealand – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-iran-new-zealand</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>06/18/2026</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Switzerland vs. Bosnia and Herzegovina – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-switzerland-vs-bosnia-and-herzegovina</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>06/21/2026</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Belgium vs. IR Iran – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-belgium-iran</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>06/25/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Türkiye vs. USA – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-turkiye-vs-usa</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>06/28/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Round of 32: TBD vs. TBD – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-roundof32-june28</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>07/02/2026</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Round of 32: TBD vs. TBD – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-roundof32-july2</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>07/10/2026</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Quarterfinals: TBD vs. TBD – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-quarterfinal-july10</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>08/08/2026</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>5:30 PM</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Ed Sheeran – With Myles Smith, Sigrid, Aaron Rowe</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/ed-sheeran-august-8-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>08/14/2026</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>KAROL G - VIAJANDO POR EL MUNDO TROPITOUR</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/karol-g-august-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>08/15/2026</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>KAROL G - VIAJANDO POR EL MUNDO TROPITOUR</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/karol-g-august-15</t>
+          <t>No events found</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3493,7 +3190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3543,142 +3240,142 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>6:00 PM</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>PUBLIC TOURS</t>
+          <t>VIP Fan Day MexTour Live</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/614/public-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/646/vip-fan-day-mextour-live</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>05/29/2026</t>
+          <t>05/30/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>VIP Fan Day MexTour Live</t>
+          <t>Mexico vs Australia</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/646/vip-fan-day-mextour-live</t>
+          <t>https://www.rosebowlstadium.com/events/details/635/mexico-vs-australia</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>05/30/2026</t>
+          <t>06/14/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mexico vs Australia</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/635/mexico-vs-australia</t>
+          <t>https://www.rosebowlstadium.com/events/details/601/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06/14/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>3:00 PM</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>Foodieland</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/601/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/637/foodieland</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06/26/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PUBLIC TOURS</t>
+          <t>Foodieland</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/615/public-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/638/foodieland</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>3:00 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -3688,7 +3385,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/637/foodieland</t>
+          <t>https://www.rosebowlstadium.com/events/details/639/foodieland</t>
         </is>
       </c>
     </row>
@@ -3700,22 +3397,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>07/11/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>5:15 PM</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Foodieland</t>
+          <t>DRUM CORPS AT THE ROSE BOWL</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/638/foodieland</t>
+          <t>https://www.rosebowlstadium.com/events/details/644/drum-corps-at-the-rose-bowl</t>
         </is>
       </c>
     </row>
@@ -3727,22 +3424,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>07/12/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Foodieland</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/639/foodieland</t>
+          <t>https://www.rosebowlstadium.com/events/details/602/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
@@ -3754,22 +3451,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>07/11/2026</t>
+          <t>08/08/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>5:15 PM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>DRUM CORPS AT THE ROSE BOWL</t>
+          <t>Head in the Clouds</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/644/drum-corps-at-the-rose-bowl</t>
+          <t>https://www.rosebowlstadium.com/events/details/642/head-in-the-clouds</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3478,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>07/12/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3796,34 +3493,34 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/602/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/603/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>07/31/2026</t>
+          <t>08/15/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>6:30 PM</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>PUBLIC TOURS</t>
+          <t>NOAH KAHAN - THE GREAT DIVIDE TOUR</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/616/public-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/633/noah-kahan-the-great-divide-tour</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3532,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>08/08/2026</t>
+          <t>08/22/2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3845,39 +3542,39 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Head in the Clouds</t>
+          <t>Just Like Heaven</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/642/head-in-the-clouds</t>
+          <t>https://www.rosebowlstadium.com/events/details/640/just-like-heaven</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>GUNS N’ ROSES</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/603/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/579/guns-n'-roses</t>
         </is>
       </c>
     </row>
@@ -3889,61 +3586,61 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>08/15/2026</t>
+          <t>09/12/2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6:30 PM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>NOAH KAHAN - THE GREAT DIVIDE TOUR</t>
+          <t>SAN DIEGO STATE VS UCLA</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/633/noah-kahan-the-great-divide-tour</t>
+          <t>https://www.rosebowlstadium.com/events/details/594/san-diego-state-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>08/22/2026</t>
+          <t>09/13/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Just Like Heaven</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/640/just-like-heaven</t>
+          <t>https://www.rosebowlstadium.com/events/details/604/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>08/28/2026</t>
+          <t>09/19/2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3953,39 +3650,39 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>PUBLIC TOURS</t>
+          <t>PURDUE VS UCLA</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/617/public-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/595/purdue-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>GUNS N’ ROSES</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/579/guns-n'-roses</t>
+          <t>https://www.rosebowlstadium.com/events/details/605/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
@@ -3997,7 +3694,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>09/12/2026</t>
+          <t>10/17/2026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -4007,39 +3704,39 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>SAN DIEGO STATE VS UCLA</t>
+          <t>WISCONSIN VS UCLA</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/594/san-diego-state-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/627/wisconsin-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>09/13/2026</t>
+          <t>10/24/2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>MICHIGAN STATE VS UCLA</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/604/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/628/michigan-state-vs-ucla</t>
         </is>
       </c>
     </row>
@@ -4051,7 +3748,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>09/19/2026</t>
+          <t>10/31/2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -4061,66 +3758,66 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>PURDUE VS UCLA</t>
+          <t>NEVADA VS UCLA</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/595/purdue-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/629/nevada-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>09/25/2026</t>
+          <t>11/08/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>PUBLIC TOURS</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/618/public-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/606/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10/11/2026</t>
+          <t>11/13/2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>6:00 PM</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>ILLINOIS VS UCLA</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/605/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/630/illinois-vs-ucla</t>
         </is>
       </c>
     </row>
@@ -4132,7 +3829,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10/17/2026</t>
+          <t>11/28/2026</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -4142,51 +3839,51 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>WISCONSIN VS UCLA</t>
+          <t>USC VS UCLA</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/627/wisconsin-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10/24/2026</t>
+          <t>12/13/2026</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>MICHIGAN STATE VS UCLA</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/628/michigan-state-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>10/30/2026</t>
+          <t>12/26/2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -4196,24 +3893,24 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>PUBLIC TOURS</t>
+          <t>HOLIDAY TOURS</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/620/public-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>10/31/2026</t>
+          <t>12/27/2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -4223,78 +3920,78 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>NEVADA VS UCLA</t>
+          <t>HOLIDAY TOURS</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/629/nevada-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>11/08/2026</t>
+          <t>12/28/2026</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>HOLIDAY TOURS</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/606/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>11/13/2026</t>
+          <t>01/02/2027</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>ILLINOIS VS UCLA</t>
+          <t>HOLIDAY TOURS</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/630/illinois-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>11/27/2026</t>
+          <t>01/02/2027</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -4304,24 +4001,24 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>PUBLIC TOURS</t>
+          <t>HOLIDAY TOURS (duplicate)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/622/public-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/647/holiday-tours-(duplicate)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>11/28/2026</t>
+          <t>01/17/2027</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -4331,199 +4028,10 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>USC VS UCLA</t>
+          <t>Rose Bowl Half Marathon &amp; 5K</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>12/13/2026</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>5:00 AM</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>ROSE BOWL FLEA MARKET</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>12/26/2026</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>HOLIDAY TOURS</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>12/27/2026</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>HOLIDAY TOURS</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>12/28/2026</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>HOLIDAY TOURS</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>01/02/2027</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>HOLIDAY TOURS</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>01/02/2027</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>HOLIDAY TOURS (duplicate)</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rosebowlstadium.com/events/details/647/holiday-tours-(duplicate)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>01/17/2027</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Rose Bowl Half Marathon &amp; 5K</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>https://www.rosebowlstadium.com/events/details/626/rose-bowl-half-marathon-and-5k</t>
         </is>
@@ -4561,13 +4069,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update events: 2026-05-22 00:04 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -437,14 +437,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,11 +477,314 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/12/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>USA vs. Paraguay – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-usa-paraguay</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>06/15/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>IR Iran vs. New Zealand – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-iran-new-zealand</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>06/18/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Switzerland vs. Bosnia and Herzegovina – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-switzerland-vs-bosnia-and-herzegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>06/21/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Belgium vs. IR Iran – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-belgium-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06/25/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Türkiye vs. USA – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-turkiye-vs-usa</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06/28/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Round of 32: TBD vs. TBD – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-roundof32-june28</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07/02/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Round of 32: TBD vs. TBD – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-roundof32-july2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Quarterfinals: TBD vs. TBD – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-quarterfinal-july10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08/08/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ed Sheeran – With Myles Smith, Sigrid, Aaron Rowe</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/ed-sheeran-august-8-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08/14/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>KAROL G - VIAJANDO POR EL MUNDO TROPITOUR</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/karol-g-august-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08/15/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>KAROL G - VIAJANDO POR EL MUNDO TROPITOUR</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/karol-g-august-15</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update events: 2026-05-25 20:16 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -1741,7 +1741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1781,12 +1781,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>05/22/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1796,24 +1796,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NIALL HORAN – Dinner Party Live On Tour</t>
+          <t>RUSH – Fifty Something</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/niall-horan/</t>
+          <t>https://thekiaforum.com/event/rush/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>05/24/2026</t>
+          <t>06/09/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1823,24 +1823,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>KESHA – The Freedom Tour</t>
+          <t>RUSH – Fifty Something</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/kesha/</t>
+          <t>https://thekiaforum.com/event/rush-2/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>06/11/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1855,19 +1855,19 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rush/</t>
+          <t>https://thekiaforum.com/event/rush-3/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06/09/2026</t>
+          <t>06/13/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1882,19 +1882,19 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rush-2/</t>
+          <t>https://thekiaforum.com/event/rush-4/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06/11/2026</t>
+          <t>06/17/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1904,24 +1904,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>RUSH – Fifty Something</t>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rush-3/</t>
+          <t>https://thekiaforum.com/event/ariana-grande-2/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06/13/2026</t>
+          <t>06/19/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1931,24 +1931,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>RUSH – Fifty Something</t>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rush-4/</t>
+          <t>https://thekiaforum.com/event/ariana-grande/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06/17/2026</t>
+          <t>06/20/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1963,19 +1963,19 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/ariana-grande-2/</t>
+          <t>https://thekiaforum.com/event/ariana-grande-3/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06/19/2026</t>
+          <t>06/24/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1985,24 +1985,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
+          <t>MADISON BEER – the locket tour</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/ariana-grande/</t>
+          <t>https://thekiaforum.com/event/madison-beer/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06/20/2026</t>
+          <t>06/26/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2012,24 +2012,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
+          <t>PALOMAZO NORTEÑO – CLASE MAESTRA TOUR</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/ariana-grande-3/</t>
+          <t>https://thekiaforum.com/event/palomazo-norteno/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06/24/2026</t>
+          <t>06/27/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2039,24 +2039,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MADISON BEER – the locket tour</t>
+          <t>A$AP ROCKY – Don't Be Dumb World Tour</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/madison-beer/</t>
+          <t>https://thekiaforum.com/event/aap-rocky/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06/26/2026</t>
+          <t>06/29/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2066,24 +2066,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>PALOMAZO NORTEÑO – CLASE MAESTRA TOUR</t>
+          <t>ROSALÍA – LUX TOUR 2026</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/palomazo-norteno/</t>
+          <t>https://thekiaforum.com/event/rosalia/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06/27/2026</t>
+          <t>07/01/2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2093,24 +2093,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>A$AP ROCKY – Don't Be Dumb World Tour</t>
+          <t>ROSALÍA – LUX TOUR 2026</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/aap-rocky/</t>
+          <t>https://thekiaforum.com/event/rosalia-2/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06/29/2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2120,24 +2120,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ROSALÍA – LUX TOUR 2026</t>
+          <t>HILARY DUFF – the lucky me tour</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rosalia/</t>
+          <t>https://thekiaforum.com/event/hilary-duff/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>07/01/2026</t>
+          <t>07/09/2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2147,24 +2147,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>ROSALÍA – LUX TOUR 2026</t>
+          <t>HILARY DUFF – the lucky me tour</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rosalia-2/</t>
+          <t>https://thekiaforum.com/event/hilary-duff-2/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07/08/2026</t>
+          <t>07/11/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2174,24 +2174,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>HILARY DUFF – the lucky me tour</t>
+          <t>5 SECONDS OF SUMMER – EVERYONE’S A STAR! World Tour</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/hilary-duff/</t>
+          <t>https://thekiaforum.com/event/5-seconds-of-summer/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>07/17/2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2201,12 +2201,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>HILARY DUFF – the lucky me tour</t>
+          <t>YOUNG THE GIANT – Victory Garden Tour</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/hilary-duff-2/</t>
+          <t>https://thekiaforum.com/event/young-the-giant/</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07/11/2026</t>
+          <t>07/18/2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2228,12 +2228,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>5 SECONDS OF SUMMER – EVERYONE’S A STAR! World Tour</t>
+          <t>EVANESCENCE</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/5-seconds-of-summer/</t>
+          <t>https://thekiaforum.com/event/evanescence/</t>
         </is>
       </c>
     </row>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07/17/2026</t>
+          <t>07/31/2026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2255,12 +2255,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>YOUNG THE GIANT – Victory Garden Tour</t>
+          <t>MOTIONLESS IN WHITE – The Sweat and Blood Tour</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/young-the-giant/</t>
+          <t>https://thekiaforum.com/event/motionless-in-white/</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07/18/2026</t>
+          <t>08/01/2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2282,24 +2282,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>EVANESCENCE</t>
+          <t>IVE – WORLD TOUR [SHOW WHAT I AM] IN LOS ANGELES</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/evanescence/</t>
+          <t>https://thekiaforum.com/event/ive/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07/31/2026</t>
+          <t>08/06/2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2309,24 +2309,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MOTIONLESS IN WHITE – The Sweat and Blood Tour</t>
+          <t>RÜFÜS DU SOL</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/motionless-in-white/</t>
+          <t>https://thekiaforum.com/event/rufus-du-sol/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>08/01/2026</t>
+          <t>08/07/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2336,24 +2336,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>IVE – WORLD TOUR [SHOW WHAT I AM] IN LOS ANGELES</t>
+          <t>RÜFÜS DU SOL</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/ive/</t>
+          <t>https://thekiaforum.com/event/rufus-du-sol-3/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>08/06/2026</t>
+          <t>08/11/2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2368,19 +2368,19 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol/</t>
+          <t>https://thekiaforum.com/event/rufus-du-sol-2/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>08/07/2026</t>
+          <t>08/12/2026</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2395,19 +2395,19 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol-3/</t>
+          <t>https://thekiaforum.com/event/rufus-du-sol-4/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>08/11/2026</t>
+          <t>08/13/2026</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2417,24 +2417,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>RÜFÜS DU SOL</t>
+          <t>RÜFÜS DU SOL – with Ben Böhmer</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol-2/</t>
+          <t>https://thekiaforum.com/event/rufus-du-sol-5/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>08/12/2026</t>
+          <t>08/14/2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2444,24 +2444,24 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>RÜFÜS DU SOL</t>
+          <t>MELANIE MARTINEZ – HADES: THE SACRIFICE</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol-4/</t>
+          <t>https://thekiaforum.com/event/melanie-martinez/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>08/13/2026</t>
+          <t>08/21/2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2471,24 +2471,24 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>RÜFÜS DU SOL – with Ben Böhmer</t>
+          <t>OMAR COURTZ – POR SI MAÑANA NO ESTOY USA TOUR</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol-5/</t>
+          <t>https://thekiaforum.com/event/omar-courtz/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>08/14/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2498,12 +2498,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>MELANIE MARTINEZ – HADES: THE SACRIFICE</t>
+          <t>CHICAGO &amp; STYX – The Windy Cities Tour - All The Hits... Your Kind of Tour</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/melanie-martinez/</t>
+          <t>https://thekiaforum.com/event/chicago-styx/</t>
         </is>
       </c>
     </row>
@@ -2515,7 +2515,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>08/21/2026</t>
+          <t>09/11/2026</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2525,24 +2525,24 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>OMAR COURTZ – POR SI MAÑANA NO ESTOY USA TOUR</t>
+          <t>JOHNNY BLUE SKIES &amp; THE DARK CLOUDS – Mutiny for the Masses 2026 Tour</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/omar-courtz/</t>
+          <t>https://thekiaforum.com/event/johnny-blue-skies-the-dark-clouds/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>09/06/2026</t>
+          <t>09/12/2026</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2552,24 +2552,24 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>CHICAGO &amp; STYX – The Windy Cities Tour - All The Hits... Your Kind of Tour</t>
+          <t>SODA STEREO – ECOS TOUR</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/chicago-styx/</t>
+          <t>https://thekiaforum.com/event/soda-stereo/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>09/11/2026</t>
+          <t>09/23/2026</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2579,24 +2579,24 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>JOHNNY BLUE SKIES &amp; THE DARK CLOUDS – Mutiny for the Masses 2026 Tour</t>
+          <t>ROBYN – The Sexistential Tour</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/johnny-blue-skies-the-dark-clouds/</t>
+          <t>https://thekiaforum.com/event/robyn/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>09/12/2026</t>
+          <t>09/24/2026</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2606,24 +2606,24 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>SODA STEREO – ECOS TOUR</t>
+          <t>ROBYN – The Sexistential Tour</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/soda-stereo/</t>
+          <t>https://thekiaforum.com/event/robyn-2/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>09/23/2026</t>
+          <t>09/25/2026</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2633,24 +2633,24 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>ROBYN – The Sexistential Tour</t>
+          <t>LILY ALLEN – Lily Allen Performs West End Girl</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/robyn/</t>
+          <t>https://thekiaforum.com/event/lily-allen/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>09/24/2026</t>
+          <t>09/26/2026</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2660,24 +2660,24 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>ROBYN – The Sexistential Tour</t>
+          <t>BILLY STRINGS</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/robyn-2/</t>
+          <t>https://thekiaforum.com/event/billy-strings-3/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>09/25/2026</t>
+          <t>09/30/2026</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2687,24 +2687,24 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>LILY ALLEN – Lily Allen Performs West End Girl</t>
+          <t>DISNEY DESCENDANTS, ZOMBIES &amp; CAMP ROCK: WORLDS COLLIDE CONCERT TOUR</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/lily-allen/</t>
+          <t>https://thekiaforum.com/event/worlds-collide-concert-tour/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>09/26/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2714,12 +2714,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>BILLY STRINGS</t>
+          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/billy-strings-3/</t>
+          <t>https://thekiaforum.com/event/mumford-sons/</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>09/30/2026</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2741,24 +2741,24 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>DISNEY DESCENDANTS, ZOMBIES &amp; CAMP ROCK: WORLDS COLLIDE CONCERT TOUR</t>
+          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/worlds-collide-concert-tour/</t>
+          <t>https://thekiaforum.com/event/mumford-sons-2/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>10/06/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2768,24 +2768,24 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/mumford-sons/</t>
+          <t>https://thekiaforum.com/event/the-neighbourhood/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2795,12 +2795,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
+          <t>SOMBR – You Are The Reason Tour</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/mumford-sons-2/</t>
+          <t>https://thekiaforum.com/event/sombr/</t>
         </is>
       </c>
     </row>
@@ -2812,7 +2812,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>10/16/2026</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2822,24 +2822,24 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+          <t>JUANES</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/the-neighbourhood/</t>
+          <t>https://thekiaforum.com/event/juanes/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>10/20/2026</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2849,24 +2849,24 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>SOMBR – You Are The Reason Tour</t>
+          <t>MONSTA X – 2026 MONSTA X WORLD TOUR [THE X : NEXUS] IN LOS ANGELES</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/sombr/</t>
+          <t>https://thekiaforum.com/event/monsta-x/</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>10/16/2026</t>
+          <t>10/22/2026</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2876,24 +2876,24 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>JUANES</t>
+          <t>DOJA CAT – Tour Ma Vie World Tour</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/juanes/</t>
+          <t>https://thekiaforum.com/event/doja-cat/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>10/20/2026</t>
+          <t>10/24/2026</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2903,24 +2903,24 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>MONSTA X – 2026 MONSTA X WORLD TOUR [THE X : NEXUS] IN LOS ANGELES</t>
+          <t>GORILLAZ – The Mountain Tour</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/monsta-x/</t>
+          <t>https://thekiaforum.com/event/gorillaz-2/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>10/22/2026</t>
+          <t>11/06/2026</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2930,12 +2930,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>DOJA CAT – Tour Ma Vie World Tour</t>
+          <t>DON OMAR – The Last King World Tour</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/doja-cat/</t>
+          <t>https://thekiaforum.com/event/don-omar/</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>10/24/2026</t>
+          <t>11/07/2026</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2957,24 +2957,24 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>GORILLAZ – The Mountain Tour</t>
+          <t>MON LAFERTE – Femme Fatale Tour</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/gorillaz-2/</t>
+          <t>https://thekiaforum.com/event/mon-laferte/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>11/06/2026</t>
+          <t>11/12/2026</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2984,24 +2984,24 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>DON OMAR – The Last King World Tour</t>
+          <t>THE SMASHING PUMPKINS – The Rats In A Cage Tour</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/don-omar/</t>
+          <t>https://thekiaforum.com/event/the-smashing-pumpkins/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>11/07/2026</t>
+          <t>11/13/2026</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3011,24 +3011,24 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>MON LAFERTE – Femme Fatale Tour</t>
+          <t>SLAYER – Reign in Blood 40th Anniversary</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/mon-laferte/</t>
+          <t>https://thekiaforum.com/event/slayer/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>11/12/2026</t>
+          <t>11/14/2026</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3038,24 +3038,24 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>THE SMASHING PUMPKINS – The Rats In A Cage Tour</t>
+          <t>SLAYER – Reign in Blood 40th Anniversary</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/the-smashing-pumpkins/</t>
+          <t>https://thekiaforum.com/event/slayer-2/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>11/13/2026</t>
+          <t>11/15/2026</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3065,24 +3065,24 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>SLAYER – Reign in Blood 40th Anniversary</t>
+          <t>RAWAYANA – ¿Dónde es el after? World Tour</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/slayer/</t>
+          <t>https://thekiaforum.com/event/rawayana/</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>11/14/2026</t>
+          <t>11/18/2026</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3092,24 +3092,24 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>SLAYER – Reign in Blood 40th Anniversary</t>
+          <t>TEDDY SWIMS – The UGLY Tour</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/slayer-2/</t>
+          <t>https://thekiaforum.com/event/teddy-swims/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>11/15/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3119,24 +3119,24 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>RAWAYANA – ¿Dónde es el after? World Tour</t>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rawayana/</t>
+          <t>https://thekiaforum.com/event/the-neighbourhood-2/</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>11/18/2026</t>
+          <t>12/05/2026</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3146,24 +3146,24 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>TEDDY SWIMS – The UGLY Tour</t>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/teddy-swims/</t>
+          <t>https://thekiaforum.com/event/the-neighbourhood-3/</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>05/22/2027</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3173,39 +3173,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+          <t>NIALL HORAN – Dinner Party Live On Tour</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/the-neighbourhood-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>12/05/2026</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/the-neighbourhood-3/</t>
+          <t>https://thekiaforum.com/event/niall-horan/</t>
         </is>
       </c>
     </row>
@@ -3263,7 +3236,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3281,7 +3253,7 @@
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="37" customWidth="1" min="4" max="4"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -3315,12 +3287,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>05/23/2026</t>
+          <t>07/17/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3330,24 +3302,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>LA Galaxy vs Houston Dynamo FC</t>
+          <t>LA Galaxy vs LAFC</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-houston-dynamo-fc</t>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-lafc</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>07/17/2026</t>
+          <t>07/22/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3357,24 +3329,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>LA Galaxy vs LAFC</t>
+          <t>LA Galaxy vs St. Louis CITY SC</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-lafc</t>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-st-louis-city-sc</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>07/22/2026</t>
+          <t>07/25/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3384,12 +3356,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>LA Galaxy vs St. Louis CITY SC</t>
+          <t>Campeón de Campeones 2026</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-st-louis-city-sc</t>
+          <t>https://www.dignityhealthsportspark.com/events/detail/campeon-de-campeones-2026</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3373,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>07/25/2026</t>
+          <t>08/01/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3411,24 +3383,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Campeón de Campeones 2026</t>
+          <t>LA Galaxy vs FC Dallas</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/campeon-de-campeones-2026</t>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-fc-dallas</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>08/01/2026</t>
+          <t>08/19/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3438,24 +3410,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>LA Galaxy vs FC Dallas</t>
+          <t>LA Galaxy vs San Jose Earthquakes</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-fc-dallas</t>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-san-jose-earthquakes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>08/19/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3465,12 +3437,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>LA Galaxy vs San Jose Earthquakes</t>
+          <t>LA Galaxy vs New England Revolution</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-san-jose-earthquakes</t>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-new-england-revolution</t>
         </is>
       </c>
     </row>
@@ -4383,10 +4355,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -4423,33 +4395,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>05/21/2026</t>
+          <t>06/02/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Romeo Santos &amp; Prince Royce – Mejor Tarde Que Nunca Tour 2026</t>
+          <t>Los Angeles Sparks vs Las Vegas Aces – Commissioner's Cup</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/romeosantosprinceroyce052126</t>
+          <t>https://www.cryptoarena.com/events/detail/sparksaces060226</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Dallas Wings – Commissioner's Cup</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparkswings060526</t>
         </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4808,7 +4808,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>05/23/2026</t>
+          <t>05/30/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4818,12 +4818,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Golden State Judo</t>
+          <t>Society of Nuclear Medicine and Molecular Imaging Annual Meeting 2026</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.laconventioncenter.com/events/detail/golden-state-judo</t>
+          <t>https://www.laconventioncenter.com/events/detail/society-of-nuclear-medicine-and-molecular-imaging-annual-meeting-2026</t>
         </is>
       </c>
     </row>
@@ -4835,7 +4835,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>05/30/2026</t>
+          <t>06/06/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4845,24 +4845,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Society of Nuclear Medicine and Molecular Imaging Annual Meeting 2026</t>
+          <t>FITTED x COD - LOS ANGELES</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.laconventioncenter.com/events/detail/society-of-nuclear-medicine-and-molecular-imaging-annual-meeting-2026</t>
+          <t>https://www.laconventioncenter.com/events/detail/fitted-cod-los-angeles</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06/06/2026</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4872,24 +4872,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>FITTED x COD - LOS ANGELES</t>
+          <t>AWS Summit Los Angeles 2026</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.laconventioncenter.com/events/detail/fitted-cod-los-angeles</t>
+          <t>https://www.laconventioncenter.com/events/detail/aws-summit-los-angeles-2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>06/13/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4899,12 +4899,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>AWS Summit Los Angeles 2026</t>
+          <t>LA Card Show</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.laconventioncenter.com/events/detail/aws-summit-los-angeles-2026</t>
+          <t>https://www.laconventioncenter.com/events/detail/la-card-show</t>
         </is>
       </c>
     </row>
@@ -4926,12 +4926,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>LA Card Show</t>
+          <t>HorrorCon Los Angeles</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.laconventioncenter.com/events/detail/la-card-show</t>
+          <t>https://www.laconventioncenter.com/events/detail/horrorcon-los-angeles-2026</t>
         </is>
       </c>
     </row>
@@ -4953,12 +4953,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>HorrorCon Los Angeles</t>
+          <t>CoreTCG x One Piece Regionals</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.laconventioncenter.com/events/detail/horrorcon-los-angeles-2026</t>
+          <t>https://www.laconventioncenter.com/events/detail/coretcg-one-piece-regionals</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update events: 2026-05-26 17:49 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -437,10 +437,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -771,415 +771,57 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E33"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="56" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Time</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Event Name</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3888?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270112</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>01/13/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3889?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270113</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>01/16/2026</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3890?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270116</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>01/17/2026</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3891?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270117</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>01/20/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3913?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270120</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>01/21/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3914?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270121</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>01/24/2026</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3915?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270124</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>01/25/2026</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3916?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270125</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>01/28/2026</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3917?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270128</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>01/29/2026</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3918?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270129</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>02/26/2026</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>MORAT</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3967?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=morat_270226</t>
-        </is>
-      </c>
-    </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06/13/2026</t>
+          <t>08/16/2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
+          <t>KAROL G - VIAJANDO POR EL MUNDO TROPITOUR</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3671?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260613</t>
+          <t>https://www.sofistadium.com/events/detail/karol-g-august-16</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06/14/2026</t>
+          <t>08/20/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
+          <t>Chargers vs 49ers – Preseason</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3672?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260614</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-49ers-preseason-2026</t>
         </is>
       </c>
     </row>
@@ -1191,142 +833,142 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06/20/2026</t>
+          <t>08/22/2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>12:30 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>BIG3</t>
+          <t>Rams vs. Saints – Preseason</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3898?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=big3_260620</t>
+          <t>https://www.sofistadium.com/events/detail/rams-saints-preseason-2026</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07/11/2026</t>
+          <t>08/27/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>6:30 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>JOJI: SOLARIS</t>
+          <t>Chargers vs Rams – Preseason</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3506?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260711</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-rams-preseason-2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07/12/2026</t>
+          <t>09/01/2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>6:30 PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>JOJI: SOLARIS</t>
+          <t>BTS – BTS WORLD TOUR ‘ARIRANG’ IN LOS ANGELES</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3513?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260712</t>
+          <t>https://www.sofistadium.com/events/detail/bts-september-1-2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07/17/2026</t>
+          <t>09/02/2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Forrest Frank</t>
+          <t>BTS – BTS WORLD TOUR ‘ARIRANG’ IN LOS ANGELES</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3285?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=forrest_frank_260717</t>
+          <t>https://www.sofistadium.com/events/detail/bts-september-2-2026</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07/27/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>4:30 PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>WWE Monday Night RAW</t>
+          <t>BTS – BTS WORLD TOUR ‘ARIRANG’ IN LOS ANGELES</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3937?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=wwe_monday_night_raw_260727</t>
+          <t>https://www.sofistadium.com/events/detail/bts-september-5-2026</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>08/07/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1336,12 +978,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Grupo Frontera</t>
+          <t>BTS – BTS WORLD TOUR ‘ARIRANG’ IN LOS ANGELES</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3520?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=grupo_frontera_260807</t>
+          <t>https://www.sofistadium.com/events/detail/bts-september-6-2026</t>
         </is>
       </c>
     </row>
@@ -1353,157 +995,157 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>09/13/2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>1:25 PM</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Lionel Richie and Earth, Wind &amp; Fire</t>
+          <t>Chargers vs. Cardinals – Week 1</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3449?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=lionel_richie_earth_wind_fire_260809</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-cardinals-2026</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>08/15/2026</t>
+          <t>09/20/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>1:05 PM</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Yeat</t>
+          <t>Chargers vs. Raiders – Week 2</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3699?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=yeat_260815</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-raiders-2026</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>08/21/2026</t>
+          <t>09/21/2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>5:15 PM</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Ne-Yo &amp; Akon</t>
+          <t>Rams vs. Giants – Week 2</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3454?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=ne-yo_akon_260821</t>
+          <t>https://www.sofistadium.com/events/detail/rams-giants-2026</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>09/25/2026</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>J. Cole</t>
+          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3492?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
+          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-25</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>09/26/2026</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>J. Cole</t>
+          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3498?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
+          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-26</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>09/30/2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>World of Warcraft®: 20 Years of Music</t>
+          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3683?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=world_of_warcraft_260910</t>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-september-30</t>
         </is>
       </c>
     </row>
@@ -1515,22 +1157,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>09/18/2026</t>
+          <t>10/02/2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>8:30 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Maná</t>
+          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260918</t>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-2</t>
         </is>
       </c>
     </row>
@@ -1542,130 +1184,130 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>09/19/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>8:30 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Maná</t>
+          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260919</t>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-3</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>aespa LIVE TOUR – SYNK : COMPLæXITY – in Los Angeles</t>
+          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3850?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=aespa_live_tour_261003</t>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-6</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>TLC and Salt-N-Pepa</t>
+          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3613?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=tlc_salt-n-pepa_261010</t>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-7</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10/17/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>1:05 PM</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Young Miko</t>
+          <t>Chargers vs. Broncos – Week 5</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3707?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=young_miko_261017</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-broncos-2026</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>10/24/2026</t>
+          <t>10/12/2026</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>5:15 PM</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Pokémon Night Out</t>
+          <t>Rams vs. Bills – Week 5</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3674?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=pokemon_night_out_261024</t>
+          <t>https://www.sofistadium.com/events/detail/rams-bills-2026</t>
         </is>
       </c>
     </row>
@@ -1677,22 +1319,346 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>10/18/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1:05 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Rams vs. Cardinals – Week 6</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/rams-cardinals-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>11/01/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1:05 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Rams vs. Chargers – Week 8</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/rams-chargers-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1:05 PM</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Chargers vs. Texans – Week 9</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chargers-texans-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>11/15/2026</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-november-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>11/22/2026</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Three Days Grace</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3149?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=three_days_grace_261122</t>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1:05 PM</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Chargers vs. Jets – Week 11</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chargers-jets-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>11/25/2026</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>5:00 PM</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Rams vs. Packers – Week 12</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/rams-packers-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>11/29/2026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>5:20 PM</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Chargers vs. Patriots – Week 12</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chargers-patriots-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>12/03/2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>5:15 PM</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Rams vs. Chiefs – Week 13</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/rams-chiefs-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>12/17/2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>5:15 PM</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Chargers vs. 49ers – Week 15</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chargers-49ers-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>12/20/2026</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1:25 PM</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Rams vs. Cowboys – Week 15</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/rams-cowboys-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Chargers vs. Chiefs – Week 17</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chargers-chiefs-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Rams vs. Seahawks – Week 18</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/rams-seahawks-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Super Bowl LXI</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/super-bowl-lxi</t>
         </is>
       </c>
     </row>
@@ -1730,6 +1696,992 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Event Name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3888?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270112</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>01/13/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3889?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270113</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>01/16/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3890?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270116</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>01/17/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3891?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270117</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>01/20/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3913?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270120</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>01/21/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3914?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270121</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>01/24/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3915?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270124</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>01/25/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3916?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270125</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>01/28/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3917?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270128</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>01/29/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3918?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270129</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>02/26/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MORAT</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3967?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=morat_270226</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06/13/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3671?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260613</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06/14/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3672?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260614</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06/20/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>12:30 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>BIG3</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3898?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=big3_260620</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>JOJI: SOLARIS</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3506?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260711</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07/12/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>JOJI: SOLARIS</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3513?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260712</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Forrest Frank</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3285?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=forrest_frank_260717</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07/27/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>4:30 PM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>WWE Monday Night RAW</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3937?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=wwe_monday_night_raw_260727</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Grupo Frontera</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3520?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=grupo_frontera_260807</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Lionel Richie and Earth, Wind &amp; Fire</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3449?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=lionel_richie_earth_wind_fire_260809</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08/15/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Yeat</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3699?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=yeat_260815</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08/21/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ne-Yo &amp; Akon</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3454?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=ne-yo_akon_260821</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>09/03/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>J. Cole</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3492?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>J. Cole</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3498?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>World of Warcraft®: 20 Years of Music</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3683?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=world_of_warcraft_260910</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>09/18/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>8:30 PM</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Maná</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260918</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>09/19/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>8:30 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Maná</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260919</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09/24/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Kehlani</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/4033?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=kehlani_260924</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>aespa LIVE TOUR – SYNK : COMPLæXITY – in Los Angeles</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3850?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=aespa_live_tour_261003</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>TLC and Salt-N-Pepa</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3613?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=tlc_salt-n-pepa_261010</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>10/17/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Young Miko</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3707?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=young_miko_261017</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Pokémon Night Out</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3674?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=pokemon_night_out_261024</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>11/22/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Three Days Grace</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3149?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=three_days_grace_261122</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1741,7 +2693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2699,12 +3651,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>10/06/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2714,24 +3666,24 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
+          <t>KLANGKUENSTLER – OUTWORLD – Klangkuenstler All Night Long</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/mumford-sons/</t>
+          <t>https://thekiaforum.com/event/klangkuenstler/</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2746,19 +3698,19 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/mumford-sons-2/</t>
+          <t>https://thekiaforum.com/event/mumford-sons/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2768,24 +3720,24 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/the-neighbourhood/</t>
+          <t>https://thekiaforum.com/event/mumford-sons-2/</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2795,24 +3747,24 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>SOMBR – You Are The Reason Tour</t>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/sombr/</t>
+          <t>https://thekiaforum.com/event/the-neighbourhood/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>10/16/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2822,24 +3774,24 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>JUANES</t>
+          <t>SOMBR – You Are The Reason Tour</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/juanes/</t>
+          <t>https://thekiaforum.com/event/sombr/</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>10/20/2026</t>
+          <t>10/16/2026</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2849,24 +3801,24 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>MONSTA X – 2026 MONSTA X WORLD TOUR [THE X : NEXUS] IN LOS ANGELES</t>
+          <t>JUANES</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/monsta-x/</t>
+          <t>https://thekiaforum.com/event/juanes/</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>10/22/2026</t>
+          <t>10/20/2026</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2876,24 +3828,24 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>DOJA CAT – Tour Ma Vie World Tour</t>
+          <t>MONSTA X – 2026 MONSTA X WORLD TOUR [THE X : NEXUS] IN LOS ANGELES</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/doja-cat/</t>
+          <t>https://thekiaforum.com/event/monsta-x/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>10/24/2026</t>
+          <t>10/22/2026</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2903,24 +3855,24 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>GORILLAZ – The Mountain Tour</t>
+          <t>DOJA CAT – Tour Ma Vie World Tour</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/gorillaz-2/</t>
+          <t>https://thekiaforum.com/event/doja-cat/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>11/06/2026</t>
+          <t>10/24/2026</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2930,24 +3882,24 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>DON OMAR – The Last King World Tour</t>
+          <t>GORILLAZ – The Mountain Tour</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/don-omar/</t>
+          <t>https://thekiaforum.com/event/gorillaz-2/</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>11/07/2026</t>
+          <t>11/06/2026</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2957,24 +3909,24 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>MON LAFERTE – Femme Fatale Tour</t>
+          <t>DON OMAR – The Last King World Tour</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/mon-laferte/</t>
+          <t>https://thekiaforum.com/event/don-omar/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>11/12/2026</t>
+          <t>11/07/2026</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2984,24 +3936,24 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>THE SMASHING PUMPKINS – The Rats In A Cage Tour</t>
+          <t>MON LAFERTE – Femme Fatale Tour</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/the-smashing-pumpkins/</t>
+          <t>https://thekiaforum.com/event/mon-laferte/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>11/13/2026</t>
+          <t>11/12/2026</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3011,24 +3963,24 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>SLAYER – Reign in Blood 40th Anniversary</t>
+          <t>THE SMASHING PUMPKINS – The Rats In A Cage Tour</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/slayer/</t>
+          <t>https://thekiaforum.com/event/the-smashing-pumpkins/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>11/14/2026</t>
+          <t>11/13/2026</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3043,19 +3995,19 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/slayer-2/</t>
+          <t>https://thekiaforum.com/event/slayer/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>11/15/2026</t>
+          <t>11/14/2026</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3065,24 +4017,24 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>RAWAYANA – ¿Dónde es el after? World Tour</t>
+          <t>SLAYER – Reign in Blood 40th Anniversary</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/rawayana/</t>
+          <t>https://thekiaforum.com/event/slayer-2/</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>11/18/2026</t>
+          <t>11/15/2026</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3092,24 +4044,24 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>TEDDY SWIMS – The UGLY Tour</t>
+          <t>RAWAYANA – ¿Dónde es el after? World Tour</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/teddy-swims/</t>
+          <t>https://thekiaforum.com/event/rawayana/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>11/18/2026</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3119,24 +4071,24 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+          <t>TEDDY SWIMS – The UGLY Tour</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/the-neighbourhood-2/</t>
+          <t>https://thekiaforum.com/event/teddy-swims/</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>12/05/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3151,7 +4103,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/the-neighbourhood-3/</t>
+          <t>https://thekiaforum.com/event/the-neighbourhood-2/</t>
         </is>
       </c>
     </row>
@@ -3163,20 +4115,47 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
+          <t>12/05/2026</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
           <t>05/22/2027</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
         <is>
           <t>NIALL HORAN – Dinner Party Live On Tour</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>https://thekiaforum.com/event/niall-horan/</t>
         </is>
@@ -3236,6 +4215,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update events: 2026-05-26 18:00 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1092,573 +1092,6 @@
       <c r="E24" s="2" t="inlineStr">
         <is>
           <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>09/26/2026</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>09/30/2026</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-september-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>10/02/2026</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>10/03/2026</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>10/06/2026</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-6</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>10/07/2026</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-7</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>10/11/2026</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>1:05 PM</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Chargers vs. Broncos – Week 5</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-broncos-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>10/12/2026</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>5:15 PM</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Rams vs. Bills – Week 5</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-bills-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>10/18/2026</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>1:05 PM</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Rams vs. Cardinals – Week 6</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-cardinals-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>11/01/2026</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>1:05 PM</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Rams vs. Chargers – Week 8</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-chargers-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>11/08/2026</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>1:05 PM</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Chargers vs. Texans – Week 9</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-texans-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>11/15/2026</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-november-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>11/22/2026</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>1:05 PM</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Chargers vs. Jets – Week 11</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-jets-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>11/25/2026</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Rams vs. Packers – Week 12</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-packers-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>11/29/2026</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>5:20 PM</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Chargers vs. Patriots – Week 12</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-patriots-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>12/03/2026</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>5:15 PM</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Rams vs. Chiefs – Week 13</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-chiefs-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>12/17/2026</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>5:15 PM</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Chargers vs. 49ers – Week 15</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-49ers-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>12/20/2026</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>1:25 PM</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Rams vs. Cowboys – Week 15</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-cowboys-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Chargers vs. Chiefs – Week 17</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-chiefs-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Rams vs. Seahawks – Week 18</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-seahawks-2027</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Super Bowl LXI</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/super-bowl-lxi</t>
         </is>
       </c>
     </row>
@@ -1687,27 +1120,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4277,7 +3689,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -4304,7 +3716,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -4331,7 +3743,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -4358,7 +3770,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -4385,7 +3797,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -4412,7 +3824,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -5143,7 +4555,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -5170,7 +4582,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -5197,7 +4609,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -5224,7 +4636,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -5251,7 +4663,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -5491,7 +4903,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -5518,7 +4930,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -5545,7 +4957,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -5572,7 +4984,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -5599,7 +5011,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -5626,7 +5038,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -5653,7 +5065,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -5680,7 +5092,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -5707,7 +5119,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -5793,7 +5205,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -5820,7 +5232,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -5847,7 +5259,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -5874,7 +5286,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -5901,7 +5313,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -5928,7 +5340,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">

</xml_diff>

<commit_message>
Update events: 2026-05-26 18:57 UTC
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -878,13 +878,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F208"/>
+  <dimension ref="A1:F163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
@@ -971,7 +971,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1023,7 +1023,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>05/18/2026</t>
@@ -1031,7 +1035,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1095,7 +1099,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1127,7 +1131,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1159,7 +1163,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1223,7 +1227,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1403,7 +1407,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>05/08/2026</t>
@@ -1411,7 +1419,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1495,7 +1503,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>05/03/2026</t>
@@ -1503,7 +1515,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1523,7 +1535,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>05/03/2026</t>
@@ -1531,7 +1547,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1563,7 +1579,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1583,7 +1599,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>04/27/2026</t>
@@ -1591,7 +1611,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1655,7 +1675,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1675,7 +1695,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>04/22/2026</t>
@@ -1683,7 +1707,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1715,7 +1739,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1767,7 +1791,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr">
         <is>
           <t>04/16/2026</t>
@@ -1775,7 +1803,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1807,7 +1835,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1987,7 +2015,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
       <c r="C36" t="inlineStr">
         <is>
           <t>04/11/2026</t>
@@ -1995,7 +2027,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2027,7 +2059,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2143,7 +2175,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
       <c r="C41" t="inlineStr">
         <is>
           <t>04/08/2026</t>
@@ -2151,7 +2187,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2439,7 +2475,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2503,7 +2539,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2567,7 +2603,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2715,7 +2751,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
       <c r="C59" t="inlineStr">
         <is>
           <t>03/28/2026</t>
@@ -2723,7 +2763,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2775,7 +2815,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
       <c r="C61" t="inlineStr">
         <is>
           <t>03/27/2026</t>
@@ -2783,7 +2827,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2815,7 +2859,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2879,7 +2923,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2943,7 +2987,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3103,7 +3147,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3359,7 +3403,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3583,7 +3627,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -3647,7 +3691,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -3711,7 +3755,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -3743,7 +3787,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -3795,7 +3839,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr"/>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
       <c r="C93" t="inlineStr">
         <is>
           <t>03/06/2026</t>
@@ -3803,7 +3851,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -3887,7 +3935,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr"/>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
       <c r="C96" t="inlineStr">
         <is>
           <t>03/04/2026</t>
@@ -3895,7 +3947,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -3947,7 +3999,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr"/>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
       <c r="C98" t="inlineStr">
         <is>
           <t>03/03/2026</t>
@@ -3955,7 +4011,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -4199,7 +4255,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr"/>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
       <c r="C106" t="inlineStr">
         <is>
           <t>02/28/2026</t>
@@ -4207,7 +4267,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -4227,7 +4287,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr"/>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
       <c r="C107" t="inlineStr">
         <is>
           <t>02/28/2026</t>
@@ -4235,7 +4299,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -4267,7 +4331,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -4299,7 +4363,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -4523,7 +4587,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -4587,7 +4651,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -4735,7 +4799,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr"/>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
       <c r="C123" t="inlineStr">
         <is>
           <t>02/22/2026</t>
@@ -4743,7 +4811,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -4967,7 +5035,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -5127,7 +5195,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -5159,7 +5227,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -5191,7 +5259,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -5255,7 +5323,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -5319,7 +5387,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -5383,7 +5451,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -5415,7 +5483,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -5435,7 +5503,11 @@
           <t>Crypto.com Arena</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr"/>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
       <c r="C145" t="inlineStr">
         <is>
           <t>02/13/2026</t>
@@ -5443,7 +5515,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -5475,7 +5547,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -5527,7 +5599,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr"/>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
       <c r="C148" t="inlineStr">
         <is>
           <t>02/12/2026</t>
@@ -5535,7 +5611,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -5823,7 +5899,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -5855,7 +5931,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -5887,7 +5963,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -5907,7 +5983,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B160" t="inlineStr"/>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
       <c r="C160" t="inlineStr">
         <is>
           <t>01/31/2026</t>
@@ -5915,7 +5995,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
@@ -5947,7 +6027,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -5967,7 +6047,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr"/>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
       <c r="C162" t="inlineStr">
         <is>
           <t>01/07/2026</t>
@@ -5975,7 +6059,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
@@ -5995,7 +6079,11 @@
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B163" t="inlineStr"/>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
       <c r="C163" t="inlineStr">
         <is>
           <t>01/06/2026</t>
@@ -6003,7 +6091,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Time TBA</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -6014,1386 +6102,6 @@
       <c r="F163" s="2" t="inlineStr">
         <is>
           <t>https://www.laconventioncenter.com/events/detail/la-art-show-2027</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>Intuit Dome</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>11/22/2025</t>
-        </is>
-      </c>
-      <c r="D164" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="E164" t="inlineStr">
-        <is>
-          <t>Three Days Grace</t>
-        </is>
-      </c>
-      <c r="F164" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3149?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=three_days_grace_261122</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>L.A. Memorial Coliseum</t>
-        </is>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>Mon</t>
-        </is>
-      </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>11/02/2025</t>
-        </is>
-      </c>
-      <c r="D165" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E165" t="inlineStr">
-        <is>
-          <t>Maryland vs USC</t>
-        </is>
-      </c>
-      <c r="F165" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/maryland-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>10/22/2025</t>
-        </is>
-      </c>
-      <c r="D166" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E166" t="inlineStr">
-        <is>
-          <t>DOJA CAT</t>
-        </is>
-      </c>
-      <c r="F166" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/doja-cat/</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>LA Convention Center</t>
-        </is>
-      </c>
-      <c r="B167" t="inlineStr"/>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>10/17/2025</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E167" t="inlineStr">
-        <is>
-          <t>American Academy of Otolaryngology: 2026 AAO OTO EXPO</t>
-        </is>
-      </c>
-      <c r="F167" s="2" t="inlineStr">
-        <is>
-          <t>https://www.laconventioncenter.com/events/detail/american-academy-of-otolaryngology-2026-aao-oto-expo</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>10/09/2025</t>
-        </is>
-      </c>
-      <c r="D168" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E168" t="inlineStr">
-        <is>
-          <t>THE NEIGHBOURHOOD</t>
-        </is>
-      </c>
-      <c r="F168" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/the-neighbourhood/</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>LA Convention Center</t>
-        </is>
-      </c>
-      <c r="B169" t="inlineStr"/>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>10/09/2025</t>
-        </is>
-      </c>
-      <c r="D169" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E169" t="inlineStr">
-        <is>
-          <t>SCG CON Los Angeles 2026</t>
-        </is>
-      </c>
-      <c r="F169" s="2" t="inlineStr">
-        <is>
-          <t>https://www.laconventioncenter.com/events/detail/scg-con-los-angeles-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>L.A. Memorial Coliseum</t>
-        </is>
-      </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>10/03/2025</t>
-        </is>
-      </c>
-      <c r="D170" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E170" t="inlineStr">
-        <is>
-          <t>Washington vs USC</t>
-        </is>
-      </c>
-      <c r="F170" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/washington-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>L.A. Memorial Coliseum</t>
-        </is>
-      </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>10/03/2025</t>
-        </is>
-      </c>
-      <c r="D171" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E171" t="inlineStr">
-        <is>
-          <t>Ohio State vs USC</t>
-        </is>
-      </c>
-      <c r="F171" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/ohio-state-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>LA Convention Center</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr"/>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>09/23/2025</t>
-        </is>
-      </c>
-      <c r="D172" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E172" t="inlineStr">
-        <is>
-          <t>National Black MBA Annual Conference &amp; Exposition</t>
-        </is>
-      </c>
-      <c r="F172" s="2" t="inlineStr">
-        <is>
-          <t>https://www.laconventioncenter.com/events/detail/national-black-mba-association-conference-exposition</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>Intuit Dome</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>09/19/2025</t>
-        </is>
-      </c>
-      <c r="D173" t="inlineStr">
-        <is>
-          <t>8:30 PM</t>
-        </is>
-      </c>
-      <c r="E173" t="inlineStr">
-        <is>
-          <t>Maná</t>
-        </is>
-      </c>
-      <c r="F173" s="2" t="inlineStr">
-        <is>
-          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260919</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>Intuit Dome</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>09/18/2025</t>
-        </is>
-      </c>
-      <c r="D174" t="inlineStr">
-        <is>
-          <t>8:30 PM</t>
-        </is>
-      </c>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>Maná</t>
-        </is>
-      </c>
-      <c r="F174" s="2" t="inlineStr">
-        <is>
-          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260918</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>LA Convention Center</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr"/>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>09/16/2025</t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E175" t="inlineStr">
-        <is>
-          <t>ASLA 2026 Conference on Landscape Architecture</t>
-        </is>
-      </c>
-      <c r="F175" s="2" t="inlineStr">
-        <is>
-          <t>https://www.laconventioncenter.com/events/detail/asla-2026-conference-on-landscape-architecture</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>09/06/2025</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E176" t="inlineStr">
-        <is>
-          <t>CHICAGO &amp; STYX</t>
-        </is>
-      </c>
-      <c r="F176" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/chicago-styx/</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>L.A. Memorial Coliseum</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>09/05/2025</t>
-        </is>
-      </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E177" t="inlineStr">
-        <is>
-          <t>Fresno State vs USC</t>
-        </is>
-      </c>
-      <c r="F177" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/fresno-state-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>L.A. Memorial Coliseum</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>09/02/2025</t>
-        </is>
-      </c>
-      <c r="D178" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E178" t="inlineStr">
-        <is>
-          <t>Oregon vs USC</t>
-        </is>
-      </c>
-      <c r="F178" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/oregon-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>L.A. Memorial Coliseum</t>
-        </is>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>Tue</t>
-        </is>
-      </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>09/01/2025</t>
-        </is>
-      </c>
-      <c r="D179" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E179" t="inlineStr">
-        <is>
-          <t>Louisiana vs USC</t>
-        </is>
-      </c>
-      <c r="F179" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/louisiana-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>Intuit Dome</t>
-        </is>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>08/21/2025</t>
-        </is>
-      </c>
-      <c r="D180" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="E180" t="inlineStr">
-        <is>
-          <t>Ne-Yo &amp; Akon</t>
-        </is>
-      </c>
-      <c r="F180" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3454?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=ne-yo_akon_260821</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>08/15/2025</t>
-        </is>
-      </c>
-      <c r="D181" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E181" t="inlineStr">
-        <is>
-          <t>MEGHAN TRAINOR</t>
-        </is>
-      </c>
-      <c r="F181" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/meghan-trainor/</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>LA Convention Center</t>
-        </is>
-      </c>
-      <c r="B182" t="inlineStr"/>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>08/15/2025</t>
-        </is>
-      </c>
-      <c r="D182" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E182" t="inlineStr">
-        <is>
-          <t>APWU Biennial Convention 2026</t>
-        </is>
-      </c>
-      <c r="F182" s="2" t="inlineStr">
-        <is>
-          <t>https://www.laconventioncenter.com/events/detail/apwu-biennial-convention-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>Intuit Dome</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>08/09/2025</t>
-        </is>
-      </c>
-      <c r="D183" t="inlineStr">
-        <is>
-          <t>7:30 PM</t>
-        </is>
-      </c>
-      <c r="E183" t="inlineStr">
-        <is>
-          <t>Lionel Richie and Earth, Wind &amp; Fire</t>
-        </is>
-      </c>
-      <c r="F183" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3449?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=lionel_richie_earth_wind_fire_260809</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>LA Convention Center</t>
-        </is>
-      </c>
-      <c r="B184" t="inlineStr"/>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>08/08/2025</t>
-        </is>
-      </c>
-      <c r="D184" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E184" t="inlineStr">
-        <is>
-          <t>El Sembrador Ministries - Metanoia Los Angeles</t>
-        </is>
-      </c>
-      <c r="F184" s="2" t="inlineStr">
-        <is>
-          <t>https://www.laconventioncenter.com/events/detail/el-sembrador-ministries-metanoia-los-angeles</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>Crypto.com Arena</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr"/>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>08/07/2025</t>
-        </is>
-      </c>
-      <c r="D185" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E185" t="inlineStr">
-        <is>
-          <t>Megan Moroney</t>
-        </is>
-      </c>
-      <c r="F185" s="2" t="inlineStr">
-        <is>
-          <t>https://www.cryptoarena.com/events/detail/megan-moroney-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>LA Convention Center</t>
-        </is>
-      </c>
-      <c r="B186" t="inlineStr"/>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>08/03/2025</t>
-        </is>
-      </c>
-      <c r="D186" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E186" t="inlineStr">
-        <is>
-          <t>NALC 74th Biennial Convention</t>
-        </is>
-      </c>
-      <c r="F186" s="2" t="inlineStr">
-        <is>
-          <t>https://www.laconventioncenter.com/events/detail/nalc-74th-biennial-convention</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>L.A. Memorial Coliseum</t>
-        </is>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>08/02/2025</t>
-        </is>
-      </c>
-      <c r="D187" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E187" t="inlineStr">
-        <is>
-          <t>TBD vs USC</t>
-        </is>
-      </c>
-      <c r="F187" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/tbd-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>LA Convention Center</t>
-        </is>
-      </c>
-      <c r="B188" t="inlineStr"/>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>08/01/2025</t>
-        </is>
-      </c>
-      <c r="D188" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E188" t="inlineStr">
-        <is>
-          <t>Collect-A-Con Los Angeles</t>
-        </is>
-      </c>
-      <c r="F188" s="2" t="inlineStr">
-        <is>
-          <t>https://www.laconventioncenter.com/events/detail/collect-a-con-los-angeles-august-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C189" t="inlineStr">
-        <is>
-          <t>07/18/2025</t>
-        </is>
-      </c>
-      <c r="D189" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E189" t="inlineStr">
-        <is>
-          <t>EVANESCENCE</t>
-        </is>
-      </c>
-      <c r="F189" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/evanescence/</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>Intuit Dome</t>
-        </is>
-      </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>07/17/2025</t>
-        </is>
-      </c>
-      <c r="D190" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="E190" t="inlineStr">
-        <is>
-          <t>Forrest Frank</t>
-        </is>
-      </c>
-      <c r="F190" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3285?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=forrest_frank_260717</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>Crypto.com Arena</t>
-        </is>
-      </c>
-      <c r="B191" t="inlineStr"/>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>07/14/2025</t>
-        </is>
-      </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E191" t="inlineStr">
-        <is>
-          <t>Olivia Dean</t>
-        </is>
-      </c>
-      <c r="F191" s="2" t="inlineStr">
-        <is>
-          <t>https://www.cryptoarena.com/events/detail/oliviadean26</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C192" t="inlineStr">
-        <is>
-          <t>07/11/2025</t>
-        </is>
-      </c>
-      <c r="D192" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E192" t="inlineStr">
-        <is>
-          <t>5 SECONDS OF SUMMER</t>
-        </is>
-      </c>
-      <c r="F192" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/5-seconds-of-summer/</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>LA Convention Center</t>
-        </is>
-      </c>
-      <c r="B193" t="inlineStr"/>
-      <c r="C193" t="inlineStr">
-        <is>
-          <t>07/02/2025</t>
-        </is>
-      </c>
-      <c r="D193" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E193" t="inlineStr">
-        <is>
-          <t>Anime Expo 2026</t>
-        </is>
-      </c>
-      <c r="F193" s="2" t="inlineStr">
-        <is>
-          <t>https://www.laconventioncenter.com/events/detail/anime-expo-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="C194" t="inlineStr">
-        <is>
-          <t>07/01/2025</t>
-        </is>
-      </c>
-      <c r="D194" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E194" t="inlineStr">
-        <is>
-          <t>ROSALÍA</t>
-        </is>
-      </c>
-      <c r="F194" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rosalia-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>Mon</t>
-        </is>
-      </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>06/29/2025</t>
-        </is>
-      </c>
-      <c r="D195" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E195" t="inlineStr">
-        <is>
-          <t>ROSALÍA</t>
-        </is>
-      </c>
-      <c r="F195" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rosalia/</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B196" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C196" t="inlineStr">
-        <is>
-          <t>06/27/2025</t>
-        </is>
-      </c>
-      <c r="D196" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E196" t="inlineStr">
-        <is>
-          <t>A$AP ROCKY</t>
-        </is>
-      </c>
-      <c r="F196" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/aap-rocky/</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B197" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="C197" t="inlineStr">
-        <is>
-          <t>06/24/2025</t>
-        </is>
-      </c>
-      <c r="D197" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E197" t="inlineStr">
-        <is>
-          <t>MADISON BEER</t>
-        </is>
-      </c>
-      <c r="F197" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/madison-beer/</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>06/20/2025</t>
-        </is>
-      </c>
-      <c r="D198" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E198" t="inlineStr">
-        <is>
-          <t>ARIANA GRANDE</t>
-        </is>
-      </c>
-      <c r="F198" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/ariana-grande-3/</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B199" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="C199" t="inlineStr">
-        <is>
-          <t>06/19/2025</t>
-        </is>
-      </c>
-      <c r="D199" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E199" t="inlineStr">
-        <is>
-          <t>ARIANA GRANDE</t>
-        </is>
-      </c>
-      <c r="F199" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/ariana-grande/</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>LA Convention Center</t>
-        </is>
-      </c>
-      <c r="B200" t="inlineStr"/>
-      <c r="C200" t="inlineStr">
-        <is>
-          <t>06/19/2025</t>
-        </is>
-      </c>
-      <c r="D200" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E200" t="inlineStr">
-        <is>
-          <t>SoCal Cup: The Showcase</t>
-        </is>
-      </c>
-      <c r="F200" s="2" t="inlineStr">
-        <is>
-          <t>https://www.laconventioncenter.com/events/detail/socal-cup-the-showcase-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="C201" t="inlineStr">
-        <is>
-          <t>06/17/2025</t>
-        </is>
-      </c>
-      <c r="D201" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E201" t="inlineStr">
-        <is>
-          <t>ARIANA GRANDE</t>
-        </is>
-      </c>
-      <c r="F201" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/ariana-grande-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B202" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C202" t="inlineStr">
-        <is>
-          <t>06/13/2025</t>
-        </is>
-      </c>
-      <c r="D202" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E202" t="inlineStr">
-        <is>
-          <t>RUSH</t>
-        </is>
-      </c>
-      <c r="F202" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rush-4/</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>Crypto.com Arena</t>
-        </is>
-      </c>
-      <c r="B203" t="inlineStr"/>
-      <c r="C203" t="inlineStr">
-        <is>
-          <t>06/13/2025</t>
-        </is>
-      </c>
-      <c r="D203" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E203" t="inlineStr">
-        <is>
-          <t>Ariana Grande</t>
-        </is>
-      </c>
-      <c r="F203" s="2" t="inlineStr">
-        <is>
-          <t>https://www.cryptoarena.com/events/detail/arianagrande26</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>LA Convention Center</t>
-        </is>
-      </c>
-      <c r="B204" t="inlineStr"/>
-      <c r="C204" t="inlineStr">
-        <is>
-          <t>06/13/2025</t>
-        </is>
-      </c>
-      <c r="D204" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E204" t="inlineStr">
-        <is>
-          <t>Security and Safety Expo</t>
-        </is>
-      </c>
-      <c r="F204" s="2" t="inlineStr">
-        <is>
-          <t>https://www.laconventioncenter.com/events/detail/security-and-safety-expo</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>LA Convention Center</t>
-        </is>
-      </c>
-      <c r="B205" t="inlineStr"/>
-      <c r="C205" t="inlineStr">
-        <is>
-          <t>06/13/2025</t>
-        </is>
-      </c>
-      <c r="D205" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E205" t="inlineStr">
-        <is>
-          <t>HorrorCon Los Angeles</t>
-        </is>
-      </c>
-      <c r="F205" s="2" t="inlineStr">
-        <is>
-          <t>https://www.laconventioncenter.com/events/detail/horrorcon-los-angeles-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="C206" t="inlineStr">
-        <is>
-          <t>06/11/2025</t>
-        </is>
-      </c>
-      <c r="D206" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E206" t="inlineStr">
-        <is>
-          <t>RUSH</t>
-        </is>
-      </c>
-      <c r="F206" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rush-3/</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>Tue</t>
-        </is>
-      </c>
-      <c r="C207" t="inlineStr">
-        <is>
-          <t>06/09/2025</t>
-        </is>
-      </c>
-      <c r="D207" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E207" t="inlineStr">
-        <is>
-          <t>RUSH</t>
-        </is>
-      </c>
-      <c r="F207" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rush-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>Kia Forum</t>
-        </is>
-      </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C208" t="inlineStr">
-        <is>
-          <t>06/07/2025</t>
-        </is>
-      </c>
-      <c r="D208" t="inlineStr">
-        <is>
-          <t>Time TBA</t>
-        </is>
-      </c>
-      <c r="E208" t="inlineStr">
-        <is>
-          <t>RUSH</t>
-        </is>
-      </c>
-      <c r="F208" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rush/</t>
         </is>
       </c>
     </row>
@@ -7561,51 +6269,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F161" r:id="rId160"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F162" r:id="rId161"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F163" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F164" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F165" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F166" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F167" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F168" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F169" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F170" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F171" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F172" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F173" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F174" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F175" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F176" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F177" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F178" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F179" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F180" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F181" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F182" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F183" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F184" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F185" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F186" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F187" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F188" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F189" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F190" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F191" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F192" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F193" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F194" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F195" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F196" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F197" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F198" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F199" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F200" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F201" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F202" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F203" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F204" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F205" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F206" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F207" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F208" r:id="rId207"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update events: 2026-05-26 19:01 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SoFi Stadium" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intuit Dome" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kia Forum" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dignity Health Sports Park" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rose Bowl Stadium" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto.com Arena" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L.A. Memorial Coliseum" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LA Convention Center" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Past Events" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="SoFi Stadium" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Intuit Dome" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Kia Forum" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dignity Health Sports Park" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Rose Bowl Stadium" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Crypto.com Arena" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="L.A. Memorial Coliseum" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="LA Convention Center" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Past Events" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -438,14 +438,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,11 +478,650 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/12/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>USA vs. Paraguay – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-usa-paraguay</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>06/15/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>IR Iran vs. New Zealand – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-iran-new-zealand</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>06/18/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Switzerland vs. Bosnia and Herzegovina – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-switzerland-vs-bosnia-and-herzegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>06/21/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Belgium vs. IR Iran – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-belgium-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06/25/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Türkiye vs. USA – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-turkiye-vs-usa</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06/28/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Round of 32: TBD vs. TBD – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-roundof32-june28</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07/02/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Round of 32: TBD vs. TBD – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-roundof32-july2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Quarterfinals: TBD vs. TBD – FIFA World Cup 26™</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-quarterfinal-july10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08/08/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ed Sheeran – With Myles Smith, Sigrid, Aaron Rowe</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/ed-sheeran-august-8-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08/14/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>KAROL G - VIAJANDO POR EL MUNDO TROPITOUR</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/karol-g-august-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08/15/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>KAROL G - VIAJANDO POR EL MUNDO TROPITOUR</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/karol-g-august-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08/16/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>KAROL G - VIAJANDO POR EL MUNDO TROPITOUR</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/karol-g-august-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>08/20/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Chargers vs 49ers – Preseason</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chargers-49ers-preseason-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>08/22/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Rams vs. Saints – Preseason</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/rams-saints-preseason-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>08/27/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Chargers vs Rams – Preseason</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chargers-rams-preseason-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>BTS – BTS WORLD TOUR ‘ARIRANG’ IN LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/bts-september-1-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>09/02/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>BTS – BTS WORLD TOUR ‘ARIRANG’ IN LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/bts-september-2-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>BTS – BTS WORLD TOUR ‘ARIRANG’ IN LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/bts-september-5-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>09/06/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>BTS – BTS WORLD TOUR ‘ARIRANG’ IN LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/bts-september-6-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>09/13/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1:25 PM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Chargers vs. Cardinals – Week 1</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chargers-cardinals-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>09/20/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1:05 PM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Chargers vs. Raiders – Week 2</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chargers-raiders-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>09/21/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>5:15 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Rams vs. Giants – Week 2</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/rams-giants-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>09/25/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-25</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -493,14 +1132,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -533,11 +1172,930 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3888?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270112</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>01/13/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3889?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270113</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>01/16/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3890?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270116</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>01/17/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3891?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270117</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>01/20/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3913?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270120</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>01/21/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3914?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270121</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>01/24/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3915?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270124</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>01/25/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3916?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270125</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>01/28/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3917?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270128</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>01/29/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3918?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270129</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>02/26/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MORAT</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3967?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=morat_270226</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06/13/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3671?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260613</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06/14/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3672?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260614</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06/20/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>12:30 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>BIG3</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3898?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=big3_260620</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>JOJI: SOLARIS</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3506?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260711</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07/12/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>JOJI: SOLARIS</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3513?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260712</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Forrest Frank</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3285?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=forrest_frank_260717</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07/27/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>4:30 PM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>WWE Monday Night RAW</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3937?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=wwe_monday_night_raw_260727</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Grupo Frontera</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3520?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=grupo_frontera_260807</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Lionel Richie and Earth, Wind &amp; Fire</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3449?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=lionel_richie_earth_wind_fire_260809</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08/15/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Yeat</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3699?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=yeat_260815</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08/21/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ne-Yo &amp; Akon</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3454?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=ne-yo_akon_260821</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>09/03/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>J. Cole</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3492?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>J. Cole</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3498?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>World of Warcraft®: 20 Years of Music</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3683?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=world_of_warcraft_260910</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>09/18/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>8:30 PM</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Maná</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260918</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>09/19/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>8:30 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Maná</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260919</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09/24/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Kehlani</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/4033?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=kehlani_260924</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>aespa LIVE TOUR – SYNK : COMPLæXITY – in Los Angeles</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3850?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=aespa_live_tour_261003</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>TLC and Salt-N-Pepa</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3613?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=tlc_salt-n-pepa_261010</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>10/17/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Young Miko</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3707?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=young_miko_261017</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Pokémon Night Out</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3674?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=pokemon_night_out_261024</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>11/22/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Three Days Grace</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3149?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=three_days_grace_261122</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -548,14 +2106,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -588,11 +2146,1490 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>06/09/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>06/13/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush-4/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06/17/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ariana-grande-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06/19/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ariana-grande/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06/20/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ariana-grande-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06/24/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>MADISON BEER – the locket tour</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/madison-beer/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06/26/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PALOMAZO NORTEÑO – CLASE MAESTRA TOUR</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/palomazo-norteno/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06/27/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>A$AP ROCKY – Don't Be Dumb World Tour</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/aap-rocky/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06/29/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ROSALÍA – LUX TOUR 2026</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rosalia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ROSALÍA – LUX TOUR 2026</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rosalia-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>HILARY DUFF – the lucky me tour</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/hilary-duff/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>HILARY DUFF – the lucky me tour</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/hilary-duff-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>5 SECONDS OF SUMMER – EVERYONE’S A STAR! World Tour</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/5-seconds-of-summer/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>YOUNG THE GIANT – Victory Garden Tour</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/young-the-giant/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07/18/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>EVANESCENCE</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/evanescence/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07/31/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MOTIONLESS IN WHITE – The Sweat and Blood Tour</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/motionless-in-white/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>IVE – WORLD TOUR [SHOW WHAT I AM] IN LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ive/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>08/12/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-4/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>08/13/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL – with Ben Böhmer</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-5/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>08/14/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>MELANIE MARTINEZ – HADES: THE SACRIFICE</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/melanie-martinez/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>08/21/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>OMAR COURTZ – POR SI MAÑANA NO ESTOY USA TOUR</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/omar-courtz/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>09/06/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CHICAGO &amp; STYX – The Windy Cities Tour - All The Hits... Your Kind of Tour</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/chicago-styx/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09/11/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>JOHNNY BLUE SKIES &amp; THE DARK CLOUDS – Mutiny for the Masses 2026 Tour</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/johnny-blue-skies-the-dark-clouds/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>09/12/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SODA STEREO – ECOS TOUR</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/soda-stereo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>09/23/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>ROBYN – The Sexistential Tour</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/robyn/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>09/24/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>ROBYN – The Sexistential Tour</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/robyn-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>09/25/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>LILY ALLEN – Lily Allen Performs West End Girl</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/lily-allen/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>09/26/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>BILLY STRINGS</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/billy-strings-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>09/30/2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>DISNEY DESCENDANTS, ZOMBIES &amp; CAMP ROCK: WORLDS COLLIDE CONCERT TOUR</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/worlds-collide-concert-tour/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>KLANGKUENSTLER – OUTWORLD – Klangkuenstler All Night Long</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/klangkuenstler/</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/mumford-sons/</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/mumford-sons-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>SOMBR – You Are The Reason Tour</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/sombr/</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>10/16/2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>JUANES</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/juanes/</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>10/20/2026</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>MONSTA X – 2026 MONSTA X WORLD TOUR [THE X : NEXUS] IN LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/monsta-x/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>10/22/2026</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>DOJA CAT – Tour Ma Vie World Tour</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/doja-cat/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>GORILLAZ – The Mountain Tour</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/gorillaz-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>11/06/2026</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>DON OMAR – The Last King World Tour</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/don-omar/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>11/07/2026</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>MON LAFERTE – Femme Fatale Tour</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/mon-laferte/</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>11/12/2026</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>THE SMASHING PUMPKINS – The Rats In A Cage Tour</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-smashing-pumpkins/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>11/13/2026</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>SLAYER – Reign in Blood 40th Anniversary</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/slayer/</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>11/14/2026</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>SLAYER – Reign in Blood 40th Anniversary</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/slayer-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>11/15/2026</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>RAWAYANA – ¿Dónde es el after? World Tour</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rawayana/</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>11/18/2026</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>TEDDY SWIMS – The UGLY Tour</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/teddy-swims/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>12/05/2026</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>05/22/2027</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>NIALL HORAN – Dinner Party Live On Tour</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/niall-horan/</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -603,14 +3640,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -643,11 +3680,174 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs LAFC</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-lafc</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>07/22/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs St. Louis CITY SC</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-st-louis-city-sc</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>07/25/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Campeón de Campeones 2026</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/campeon-de-campeones-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs FC Dallas</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-fc-dallas</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>08/19/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs San Jose Earthquakes</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-san-jose-earthquakes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs New England Revolution</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-new-england-revolution</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -658,14 +3858,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -698,11 +3898,846 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>05/29/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>VIP Fan Day MexTour Live</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/646/vip-fan-day-mextour-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>05/30/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Mexico vs Australia</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/635/mexico-vs-australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>06/14/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>5:00 AM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ROSE BOWL FLEA MARKET</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/601/rose-bowl-flea-market</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Foodieland</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/637/foodieland</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Foodieland</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/638/foodieland</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Foodieland</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/639/foodieland</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>5:15 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DRUM CORPS AT THE ROSE BOWL</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/644/drum-corps-at-the-rose-bowl</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>07/12/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>5:00 AM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ROSE BOWL FLEA MARKET</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/602/rose-bowl-flea-market</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08/08/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Head in the Clouds</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/642/head-in-the-clouds</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>5:00 AM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ROSE BOWL FLEA MARKET</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/603/rose-bowl-flea-market</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08/15/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>NOAH KAHAN - THE GREAT DIVIDE TOUR</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/633/noah-kahan-the-great-divide-tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08/22/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Just Like Heaven</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/640/just-like-heaven</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>GUNS N’ ROSES</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/579/guns-n'-roses</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>09/12/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>SAN DIEGO STATE VS UCLA</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/594/san-diego-state-vs-ucla</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09/13/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>5:00 AM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ROSE BOWL FLEA MARKET</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/604/rose-bowl-flea-market</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>09/19/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>PURDUE VS UCLA</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/595/purdue-vs-ucla</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10/11/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>5:00 AM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ROSE BOWL FLEA MARKET</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/605/rose-bowl-flea-market</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10/17/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>WISCONSIN VS UCLA</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/627/wisconsin-vs-ucla</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MICHIGAN STATE VS UCLA</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/628/michigan-state-vs-ucla</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>10/31/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>NEVADA VS UCLA</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/629/nevada-vs-ucla</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>5:00 AM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>ROSE BOWL FLEA MARKET</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/606/rose-bowl-flea-market</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>11/13/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ILLINOIS VS UCLA</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/630/illinois-vs-ucla</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>11/28/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>USC VS UCLA</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>12/13/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>5:00 AM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ROSE BOWL FLEA MARKET</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>12/26/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>HOLIDAY TOURS</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>12/27/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>HOLIDAY TOURS</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>12/28/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>HOLIDAY TOURS</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>01/02/2027</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>HOLIDAY TOURS</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>01/02/2027</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>HOLIDAY TOURS (duplicate)</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/647/holiday-tours-(duplicate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>01/17/2027</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Rose Bowl Half Marathon &amp; 5K</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/626/rose-bowl-half-marathon-and-5k</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -713,14 +4748,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -753,11 +4788,62 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/02/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Las Vegas Aces – Commissioner's Cup</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksaces060226</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Dallas Wings – Commissioner's Cup</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparkswings060526</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -768,14 +4854,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -808,11 +4894,258 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FIFA Fan Festival™ Los Angeles</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/fifa-fan-festival-los-angeles/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>America250 July 4 Concert</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/america250-july-4-concert/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>08/29/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>San Jose State vs USC</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/sanjosestate-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Fresno State vs USC</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/fresno-state-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>09/12/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Louisiana vs USC</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/louisiana-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>09/26/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Oregon vs USC</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/oregon-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Washington vs USC</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/washington-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10/31/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ohio State vs USC</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/ohio-state-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>11/21/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Maryland vs USC</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/maryland-vs-usc-2026/</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update events: 2026-05-26 19:14 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1093,6 +1093,573 @@
       <c r="E24" s="2" t="inlineStr">
         <is>
           <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>09/26/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>09/30/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-september-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>10/02/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-7</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>10/11/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1:05 PM</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Chargers vs. Broncos – Week 5</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chargers-broncos-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>10/12/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>5:15 PM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Rams vs. Bills – Week 5</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/rams-bills-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>10/18/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1:05 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Rams vs. Cardinals – Week 6</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/rams-cardinals-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>11/01/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1:05 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Rams vs. Chargers – Week 8</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/rams-chargers-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1:05 PM</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Chargers vs. Texans – Week 9</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chargers-texans-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>11/15/2026</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-november-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>11/22/2026</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1:05 PM</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Chargers vs. Jets – Week 11</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chargers-jets-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>11/25/2026</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>5:00 PM</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Rams vs. Packers – Week 12</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/rams-packers-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>11/29/2026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>5:20 PM</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Chargers vs. Patriots – Week 12</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chargers-patriots-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>12/03/2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>5:15 PM</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Rams vs. Chiefs – Week 13</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/rams-chiefs-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>12/17/2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>5:15 PM</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Chargers vs. 49ers – Week 15</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chargers-49ers-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>12/20/2026</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1:25 PM</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Rams vs. Cowboys – Week 15</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/rams-cowboys-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Chargers vs. Chiefs – Week 17</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/chargers-chiefs-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Rams vs. Seahawks – Week 18</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/rams-seahawks-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Super Bowl LXI</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sofistadium.com/events/detail/super-bowl-lxi</t>
         </is>
       </c>
     </row>
@@ -1121,6 +1688,27 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5211,11 +5799,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F163"/>
+  <dimension ref="A1:F174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
@@ -8777,17 +9365,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Dignity Health Sports Park</t>
+          <t>Intuit Dome</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Wed</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>02/25/2026</t>
+          <t>02/26/2026</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -8797,19 +9385,19 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>LA Galaxy vs Sporting San Miguelito</t>
+          <t>MORAT</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-sporting-san-miguelito</t>
+          <t>https://www.intuitdome.com/events/event-schedule/3967?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=morat_270226</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Crypto.com Arena</t>
+          <t>Dignity Health Sports Park</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -8824,17 +9412,17 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>7:00PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Vegas Golden Knights vs Los Angeles Kings</t>
+          <t>LA Galaxy vs Sporting San Miguelito</t>
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/kingsknights022526</t>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-sporting-san-miguelito</t>
         </is>
       </c>
     </row>
@@ -8846,66 +9434,66 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Tue</t>
+          <t>Wed</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>02/24/2026</t>
+          <t>02/25/2026</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>7:30PM</t>
+          <t>7:00PM</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Orlando Magic vs Los Angeles Lakers</t>
+          <t>Vegas Golden Knights vs Los Angeles Kings</t>
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/lakersmagic022426</t>
+          <t>https://www.cryptoarena.com/events/detail/kingsknights022526</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Intuit Dome</t>
+          <t>Crypto.com Arena</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Tue</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>02/23/2026</t>
+          <t>02/24/2026</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>7:30PM</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>GHOST: Skeletour World Tour 2026</t>
+          <t>Orlando Magic vs Los Angeles Lakers</t>
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/2964?utm_source=eventschedule&amp;utm_medium=IDwebsite&amp;utm_campaign=IDevents25&amp;utm_content=ghost_260223</t>
+          <t>https://www.cryptoarena.com/events/detail/lakersmagic022426</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Kia Forum</t>
+          <t>Intuit Dome</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -8920,56 +9508,56 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>LADY GAGA</t>
+          <t>GHOST: Skeletour World Tour 2026</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/lady-gaga-8/</t>
+          <t>https://www.intuitdome.com/events/event-schedule/2964?utm_source=eventschedule&amp;utm_medium=IDwebsite&amp;utm_campaign=IDevents25&amp;utm_content=ghost_260223</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Intuit Dome</t>
+          <t>Kia Forum</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Sun</t>
+          <t>Mon</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>02/22/2026</t>
+          <t>02/23/2026</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Orlando Magic vs LA Clippers</t>
+          <t>LADY GAGA</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>https://intuitdome.com/events/event-schedule/2688?type=games&amp;utm_source=eventschedule&amp;utm_medium=IDwebsite&amp;utm_campaign=SGT_2526&amp;utm_content=SGT_2526_260222</t>
+          <t>https://thekiaforum.com/event/lady-gaga-8/</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Kia Forum</t>
+          <t>Intuit Dome</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -8984,24 +9572,24 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>6:00 PM</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>LADY GAGA</t>
+          <t>Orlando Magic vs LA Clippers</t>
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/lady-gaga-7/</t>
+          <t>https://intuitdome.com/events/event-schedule/2688?type=games&amp;utm_source=eventschedule&amp;utm_medium=IDwebsite&amp;utm_campaign=SGT_2526&amp;utm_content=SGT_2526_260222</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Dignity Health Sports Park</t>
+          <t>Kia Forum</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -9016,24 +9604,24 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>4:00 PM</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>LA Galaxy vs New York City FC</t>
+          <t>LADY GAGA</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-new-york-city-fc</t>
+          <t>https://thekiaforum.com/event/lady-gaga-7/</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Rose Bowl Stadium</t>
+          <t>Dignity Health Sports Park</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -9048,17 +9636,17 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>4:00 PM</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Mega Night at Pokémon GO Tour: Kalos – Los Angeles</t>
+          <t>LA Galaxy vs New York City FC</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/585/mega-night-at-pokemon-go-tour:-kalos-los-angeles</t>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-new-york-city-fc</t>
         </is>
       </c>
     </row>
@@ -9080,24 +9668,24 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>6:00 PM</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Pokémon GO Tour: Kalos – Los Angeles</t>
+          <t>Mega Night at Pokémon GO Tour: Kalos – Los Angeles</t>
         </is>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/588/pokemon-go-tour:-kalos-los-angeles</t>
+          <t>https://www.rosebowlstadium.com/events/details/585/mega-night-at-pokemon-go-tour:-kalos-los-angeles</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Crypto.com Arena</t>
+          <t>Rose Bowl Stadium</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -9112,24 +9700,24 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>3:30PM</t>
+          <t>9:00 AM</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Boston Celtics vs Los Angeles Lakers</t>
+          <t>Pokémon GO Tour: Kalos – Los Angeles</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/lakersceltics022226</t>
+          <t>https://www.rosebowlstadium.com/events/details/588/pokemon-go-tour:-kalos-los-angeles</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>LA Convention Center</t>
+          <t>Crypto.com Arena</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -9144,56 +9732,56 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>3:30PM</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>ViVE 2026</t>
+          <t>Boston Celtics vs Los Angeles Lakers</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>https://www.laconventioncenter.com/events/detail/vive-2026</t>
+          <t>https://www.cryptoarena.com/events/detail/lakersceltics022226</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>SoFi Stadium</t>
+          <t>LA Convention Center</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Sun</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>02/21/2026</t>
+          <t>02/22/2026</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>8 PM</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Los Bukis</t>
+          <t>ViVE 2026</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/los-bukis-february-21-2026</t>
+          <t>https://www.laconventioncenter.com/events/detail/vive-2026</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Intuit Dome</t>
+          <t>SoFi Stadium</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -9208,24 +9796,24 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>8 PM</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Los Tigres del Norte</t>
+          <t>Los Bukis</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/2912?utm_source=eventschedule&amp;utm_medium=IDwebsite&amp;utm_campaign=IDevents25&amp;utm_content=los_tigres_del_norte_260221</t>
+          <t>https://www.sofistadium.com/events/detail/los-bukis-february-21-2026</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Rose Bowl Stadium</t>
+          <t>Intuit Dome</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -9240,17 +9828,17 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Mega Night at Pokémon GO Tour: Kalos – Los Angeles</t>
+          <t>Los Tigres del Norte</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/584/mega-night-at-pokemon-go-tour:-kalos-los-angeles</t>
+          <t>https://www.intuitdome.com/events/event-schedule/2912?utm_source=eventschedule&amp;utm_medium=IDwebsite&amp;utm_campaign=IDevents25&amp;utm_content=los_tigres_del_norte_260221</t>
         </is>
       </c>
     </row>
@@ -9272,56 +9860,56 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>6:00 PM</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Pokémon GO Tour: Kalos – Los Angeles</t>
+          <t>Mega Night at Pokémon GO Tour: Kalos – Los Angeles</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/587/pokemon-go-tour:-kalos-los-angeles</t>
+          <t>https://www.rosebowlstadium.com/events/details/584/mega-night-at-pokemon-go-tour:-kalos-los-angeles</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>SoFi Stadium</t>
+          <t>Rose Bowl Stadium</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Fri</t>
+          <t>Sat</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>02/20/2026</t>
+          <t>02/21/2026</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>8 PM</t>
+          <t>9:00 AM</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Los Bukis</t>
+          <t>Pokémon GO Tour: Kalos – Los Angeles</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/los-bukis-2026</t>
+          <t>https://www.rosebowlstadium.com/events/details/587/pokemon-go-tour:-kalos-los-angeles</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Intuit Dome</t>
+          <t>SoFi Stadium</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -9336,24 +9924,24 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>8 PM</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Harlem Globetrotters</t>
+          <t>Los Bukis</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/2904</t>
+          <t>https://www.sofistadium.com/events/detail/los-bukis-2026</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Kia Forum</t>
+          <t>Intuit Dome</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -9368,24 +9956,24 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>SABATON</t>
+          <t>Harlem Globetrotters</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/sabaton/</t>
+          <t>https://www.intuitdome.com/events/event-schedule/2904</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Rose Bowl Stadium</t>
+          <t>Kia Forum</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -9400,17 +9988,17 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Mega Night at Pokémon GO Tour: Kalos – Los Angeles</t>
+          <t>SABATON</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/583/mega-night-at-pokemon-go-tour:-kalos-los-angeles</t>
+          <t>https://thekiaforum.com/event/sabaton/</t>
         </is>
       </c>
     </row>
@@ -9432,24 +10020,24 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>6:00 PM</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Pokémon GO Tour: Kalos – Los Angeles</t>
+          <t>Mega Night at Pokémon GO Tour: Kalos – Los Angeles</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/586/pokemon-go-tour:-kalos-los-angeles</t>
+          <t>https://www.rosebowlstadium.com/events/details/583/mega-night-at-pokemon-go-tour:-kalos-los-angeles</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Crypto.com Arena</t>
+          <t>Rose Bowl Stadium</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -9464,56 +10052,56 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>7:00PM</t>
+          <t>9:00 AM</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Los Angeles Clippers vs Los Angeles Lakers</t>
+          <t>Pokémon GO Tour: Kalos – Los Angeles</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/lakersclippers022026</t>
+          <t>https://www.rosebowlstadium.com/events/details/586/pokemon-go-tour:-kalos-los-angeles</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Intuit Dome</t>
+          <t>Crypto.com Arena</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Thu</t>
+          <t>Fri</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>02/19/2026</t>
+          <t>02/20/2026</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>7:00PM</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Denver Nuggets vs LA Clippers</t>
+          <t>Los Angeles Clippers vs Los Angeles Lakers</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>https://intuitdome.com/events/event-schedule/2687?type=games&amp;utm_source=eventschedule&amp;utm_medium=IDwebsite&amp;utm_campaign=SGT_2526&amp;utm_content=SGT_2526_260219</t>
+          <t>https://www.cryptoarena.com/events/detail/lakersclippers022026</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Kia Forum</t>
+          <t>Intuit Dome</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -9528,17 +10116,17 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>7:30 PM</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>LADY GAGA</t>
+          <t>Denver Nuggets vs LA Clippers</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/lady-gaga-5/</t>
+          <t>https://intuitdome.com/events/event-schedule/2687?type=games&amp;utm_source=eventschedule&amp;utm_medium=IDwebsite&amp;utm_campaign=SGT_2526&amp;utm_content=SGT_2526_260219</t>
         </is>
       </c>
     </row>
@@ -9550,12 +10138,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Wed</t>
+          <t>Thu</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>02/18/2026</t>
+          <t>02/19/2026</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -9570,7 +10158,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/lady-gaga-6/</t>
+          <t>https://thekiaforum.com/event/lady-gaga-5/</t>
         </is>
       </c>
     </row>
@@ -9582,12 +10170,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Wed</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>02/16/2026</t>
+          <t>02/18/2026</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -9597,51 +10185,51 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>CARDI B</t>
+          <t>LADY GAGA</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/cardi-b-2/</t>
+          <t>https://thekiaforum.com/event/lady-gaga-6/</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Intuit Dome</t>
+          <t>Kia Forum</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Sun</t>
+          <t>Mon</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>02/15/2026</t>
+          <t>02/16/2026</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>2:00 PM</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>75th NBA All-Star Game</t>
+          <t>CARDI B</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3002?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=All_Star26&amp;utm_content=all_star_game_260215</t>
+          <t>https://thekiaforum.com/event/cardi-b-2/</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Kia Forum</t>
+          <t>Intuit Dome</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -9656,56 +10244,56 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>2:00 PM</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>CARDI B</t>
+          <t>75th NBA All-Star Game</t>
         </is>
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/cardi-b/</t>
+          <t>https://www.intuitdome.com/events/event-schedule/3002?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=All_Star26&amp;utm_content=all_star_game_260215</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Intuit Dome</t>
+          <t>Kia Forum</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Sun</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>02/14/2026</t>
+          <t>02/15/2026</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>2:00 PM</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>All-Star Saturday</t>
+          <t>CARDI B</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3003?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=All_Star26&amp;utm_content=all_star_saturday_260214</t>
+          <t>https://thekiaforum.com/event/cardi-b/</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Kia Forum</t>
+          <t>Intuit Dome</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -9720,56 +10308,56 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>2:00 PM</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>DJ CASSIDY'S PASS THE MIC LIVE!</t>
+          <t>All-Star Saturday</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/dj-cassidys-pass-the-mic-live/</t>
+          <t>https://www.intuitdome.com/events/event-schedule/3003?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=All_Star26&amp;utm_content=all_star_saturday_260214</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Intuit Dome</t>
+          <t>Kia Forum</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Fri</t>
+          <t>Sat</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>02/13/2026</t>
+          <t>02/14/2026</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Castrol Rising Stars</t>
+          <t>DJ CASSIDY'S PASS THE MIC LIVE!</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3004?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=All_Star26&amp;utm_content=castrol_rising_stars_260213</t>
+          <t>https://thekiaforum.com/event/dj-cassidys-pass-the-mic-live/</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Kia Forum</t>
+          <t>Intuit Dome</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -9784,17 +10372,17 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>6:00 PM</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>HBCU CLASSIC PRESENTED BY AT&amp;T</t>
+          <t>Castrol Rising Stars</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/hbcu-classic-presented-by-att/</t>
+          <t>https://www.intuitdome.com/events/event-schedule/3004?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=All_Star26&amp;utm_content=castrol_rising_stars_260213</t>
         </is>
       </c>
     </row>
@@ -9821,19 +10409,19 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>RUFFLES CELEBRITY GAME</t>
+          <t>HBCU CLASSIC PRESENTED BY AT&amp;T</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/ruffles-celebrity-game/</t>
+          <t>https://thekiaforum.com/event/hbcu-classic-presented-by-att/</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Crypto.com Arena</t>
+          <t>Kia Forum</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -9853,29 +10441,29 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Banda MS de Sergio Lizarraga</t>
+          <t>RUFFLES CELEBRITY GAME</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/bandams021326</t>
+          <t>https://thekiaforum.com/event/ruffles-celebrity-game/</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Kia Forum</t>
+          <t>Crypto.com Arena</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Thu</t>
+          <t>Fri</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>02/12/2026</t>
+          <t>02/13/2026</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -9885,19 +10473,19 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>NBA ALL-STAR PITCH COMPETITION</t>
+          <t>Banda MS de Sergio Lizarraga</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/nba-all-star-pitch-competition/</t>
+          <t>https://www.cryptoarena.com/events/detail/bandams021326</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Crypto.com Arena</t>
+          <t>Kia Forum</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -9912,24 +10500,24 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>7:00PM</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Dallas Mavericks vs Los Angeles Lakers</t>
+          <t>NBA ALL-STAR PITCH COMPETITION</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/lakersmavs021226</t>
+          <t>https://thekiaforum.com/event/nba-all-star-pitch-competition/</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>LA Convention Center</t>
+          <t>Crypto.com Arena</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -9944,49 +10532,49 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>7:00PM</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>NBA Crossover: The Ultimate Fan Experience</t>
+          <t>Dallas Mavericks vs Los Angeles Lakers</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>https://www.laconventioncenter.com/events/detail/nba-crossover-ultimate-fan-experience</t>
+          <t>https://www.cryptoarena.com/events/detail/lakersmavs021226</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Crypto.com Arena</t>
+          <t>LA Convention Center</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Tue</t>
+          <t>Thu</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>02/12/2026</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>7:30PM</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>San Antonio Spurs vs Los Angeles Lakers</t>
+          <t>NBA Crossover: The Ultimate Fan Experience</t>
         </is>
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/lakersspurs021026</t>
+          <t>https://www.laconventioncenter.com/events/detail/nba-crossover-ultimate-fan-experience</t>
         </is>
       </c>
     </row>
@@ -9998,91 +10586,91 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Tue</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>7:00PM</t>
+          <t>7:30PM</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Oklahoma City Thunder vs Los Angeles Lakers</t>
+          <t>San Antonio Spurs vs Los Angeles Lakers</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/lakersthuner020926</t>
+          <t>https://www.cryptoarena.com/events/detail/lakersspurs021026</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Rose Bowl Stadium</t>
+          <t>Crypto.com Arena</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Sun</t>
+          <t>Mon</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>02/08/2026</t>
+          <t>02/09/2026</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>7:00PM</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>Oklahoma City Thunder vs Los Angeles Lakers</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/597/rose-bowl-flea-market</t>
+          <t>https://www.cryptoarena.com/events/detail/lakersthuner020926</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Crypto.com Arena</t>
+          <t>Rose Bowl Stadium</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Sun</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>02/07/2026</t>
+          <t>02/08/2026</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>5:30PM</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Golden State Warriors vs Los Angeles Lakers</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/lakerswarriors020726</t>
+          <t>https://www.rosebowlstadium.com/events/details/597/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
@@ -10094,66 +10682,66 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Thu</t>
+          <t>Sat</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>7:00PM</t>
+          <t>5:30PM</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Philadelphia 76ers vs Los Angeles Lakers</t>
+          <t>Golden State Warriors vs Los Angeles Lakers</t>
         </is>
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/lakers76ers020526</t>
+          <t>https://www.cryptoarena.com/events/detail/lakerswarriors020726</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Intuit Dome</t>
+          <t>Crypto.com Arena</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Wed</t>
+          <t>Thu</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>7:00PM</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Cleveland Cavaliers vs LA Clippers</t>
+          <t>Philadelphia 76ers vs Los Angeles Lakers</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>https://intuitdome.com/events/event-schedule/2662?type=games&amp;utm_source=eventschedule&amp;utm_medium=IDwebsite&amp;utm_campaign=SGT_2526&amp;utm_content=SGT_2526_260204</t>
+          <t>https://www.cryptoarena.com/events/detail/lakers76ers020526</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Crypto.com Arena</t>
+          <t>Intuit Dome</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -10168,56 +10756,56 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>7:00PM</t>
+          <t>7:30 PM</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Seattle Kraken vs Los Angeles Kings</t>
+          <t>Cleveland Cavaliers vs LA Clippers</t>
         </is>
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>https://www.cryptoarena.com/events/detail/kingskraken020426</t>
+          <t>https://intuitdome.com/events/event-schedule/2662?type=games&amp;utm_source=eventschedule&amp;utm_medium=IDwebsite&amp;utm_campaign=SGT_2526&amp;utm_content=SGT_2526_260204</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Intuit Dome</t>
+          <t>Crypto.com Arena</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Wed</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>02/02/2026</t>
+          <t>02/04/2026</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>7:00PM</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Philadelphia 76ers vs LA Clippers</t>
+          <t>Seattle Kraken vs Los Angeles Kings</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>https://intuitdome.com/events/event-schedule/2686?type=games&amp;utm_source=eventschedule&amp;utm_medium=IDwebsite&amp;utm_campaign=SGT_2526&amp;utm_content=SGT_2526_260202</t>
+          <t>https://www.cryptoarena.com/events/detail/kingskraken020426</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>L.A. Memorial Coliseum</t>
+          <t>Intuit Dome</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -10232,17 +10820,17 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>LAFC vs Inter Miami CF</t>
+          <t>Philadelphia 76ers vs LA Clippers</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>https://www.lacoliseum.com/events/lafc-vs-intermiami-2026/</t>
+          <t>https://intuitdome.com/events/event-schedule/2686?type=games&amp;utm_source=eventschedule&amp;utm_medium=IDwebsite&amp;utm_campaign=SGT_2526&amp;utm_content=SGT_2526_260202</t>
         </is>
       </c>
     </row>
@@ -10269,29 +10857,29 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Night of Hope</t>
+          <t>LAFC vs Inter Miami CF</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>https://www.lacoliseum.com/events/night-of-hope/</t>
+          <t>https://www.lacoliseum.com/events/lafc-vs-intermiami-2026/</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Kia Forum</t>
+          <t>L.A. Memorial Coliseum</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Mon</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>01/31/2026</t>
+          <t>02/02/2026</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -10301,19 +10889,19 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>NEW EDITION</t>
+          <t>Night of Hope</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>https://thekiaforum.com/event/new-edition/</t>
+          <t>https://www.lacoliseum.com/events/night-of-hope/</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>LA Convention Center</t>
+          <t>Kia Forum</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -10333,12 +10921,12 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>IBJJF Jiu Jitsu Championship</t>
+          <t>NEW EDITION</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>https://www.laconventioncenter.com/events/detail/ibjjf-jiu-jitsu-championship</t>
+          <t>https://thekiaforum.com/event/new-edition/</t>
         </is>
       </c>
     </row>
@@ -10365,12 +10953,12 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Grand Archive Phantom Monarch Regional Championships</t>
+          <t>IBJJF Jiu Jitsu Championship</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>https://www.laconventioncenter.com/events/detail/grand-archive-phantom-monarch-regional-championships</t>
+          <t>https://www.laconventioncenter.com/events/detail/ibjjf-jiu-jitsu-championship</t>
         </is>
       </c>
     </row>
@@ -10382,12 +10970,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Wed</t>
+          <t>Sat</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>01/31/2026</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -10397,42 +10985,394 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Modern Language Association Annual Convention 2027</t>
+          <t>Grand Archive Phantom Monarch Regional Championships</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>https://www.laconventioncenter.com/events/detail/modern-language-association-annual-convention-2027</t>
+          <t>https://www.laconventioncenter.com/events/detail/grand-archive-phantom-monarch-regional-championships</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
+          <t>Intuit Dome</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>01/29/2026</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3918?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270129</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Intuit Dome</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>01/28/2026</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3917?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270128</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Intuit Dome</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>01/25/2026</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3916?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270125</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Intuit Dome</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>01/24/2026</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3915?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270124</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Intuit Dome</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>01/21/2026</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3914?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270121</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Intuit Dome</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>01/20/2026</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3913?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270120</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Intuit Dome</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>01/17/2026</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3891?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270117</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Intuit Dome</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>01/16/2026</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3890?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270116</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Intuit Dome</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>01/13/2026</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3889?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270113</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Intuit Dome</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3888?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270112</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
           <t>LA Convention Center</t>
         </is>
       </c>
-      <c r="B163" t="inlineStr">
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Modern Language Association Annual Convention 2027</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/modern-language-association-annual-convention-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>LA Convention Center</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr">
+      <c r="C174" t="inlineStr">
         <is>
           <t>01/06/2026</t>
         </is>
       </c>
-      <c r="D163" t="inlineStr">
+      <c r="D174" t="inlineStr">
         <is>
           <t>TBA</t>
         </is>
       </c>
-      <c r="E163" t="inlineStr">
+      <c r="E174" t="inlineStr">
         <is>
           <t>LA Art Show 2027</t>
         </is>
       </c>
-      <c r="F163" s="2" t="inlineStr">
+      <c r="F174" s="2" t="inlineStr">
         <is>
           <t>https://www.laconventioncenter.com/events/detail/la-art-show-2027</t>
         </is>
@@ -10602,6 +11542,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F161" r:id="rId160"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F162" r:id="rId161"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F168" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F170" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F171" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F173" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F174" r:id="rId173"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update events: 2026-05-26 21:42 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -1585,12 +1585,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>02/14/2027</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1600,12 +1600,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Chargers vs. Chiefs – Week 17</t>
+          <t>Super Bowl LXI</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-chiefs-2026</t>
+          <t>https://www.sofistadium.com/events/detail/super-bowl-lxi</t>
         </is>
       </c>
     </row>
@@ -1627,12 +1627,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Rams vs. Seahawks – Week 18</t>
+          <t>Chargers vs. Chiefs – Week 17</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-seahawks-2027</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-chiefs-2026</t>
         </is>
       </c>
     </row>
@@ -1654,12 +1654,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Super Bowl LXI</t>
+          <t>Rams vs. Seahawks – Week 18</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/super-bowl-lxi</t>
+          <t>https://www.sofistadium.com/events/detail/rams-seahawks-2027</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update events: 2026-05-26 22:22 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -1585,12 +1585,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>02/14/2027</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1600,12 +1600,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Super Bowl LXI</t>
+          <t>Chargers vs. Chiefs – Week 17</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/super-bowl-lxi</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-chiefs-2026</t>
         </is>
       </c>
     </row>
@@ -1627,24 +1627,24 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Chargers vs. Chiefs – Week 17</t>
+          <t>Rams vs. Seahawks – Week 18</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-chiefs-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-seahawks-2027</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>02/14/2027</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1654,12 +1654,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Rams vs. Seahawks – Week 18</t>
+          <t>Super Bowl LXI</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-seahawks-2027</t>
+          <t>https://www.sofistadium.com/events/detail/super-bowl-lxi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update events: 2026-05-26 22:31 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -1585,12 +1585,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1612,12 +1612,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -5336,14 +5336,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5376,62 +5376,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>06/02/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Los Angeles Sparks vs Las Vegas Aces – Commissioner's Cup</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.cryptoarena.com/events/detail/sparksaces060226</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Los Angeles Sparks vs Dallas Wings – Commissioner's Cup</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.cryptoarena.com/events/detail/sparkswings060526</t>
+          <t>No events found</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5744,14 +5693,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5784,11 +5733,1126 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>05/30/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Society of Nuclear Medicine and Molecular Imaging Annual Meeting 2026</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/society-of-nuclear-medicine-and-molecular-imaging-annual-meeting-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FITTED x COD - LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/fitted-cod-los-angeles</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>AWS Summit Los Angeles 2026</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/aws-summit-los-angeles-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>06/13/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>LA Card Show</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/la-card-show</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06/13/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>HorrorCon Los Angeles</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/horrorcon-los-angeles-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06/13/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CoreTCG x One Piece Regionals</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/coretcg-one-piece-regionals</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06/13/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Tonight's Conversation: LIVE &amp; UNCUT Los Angeles</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/tonights-conversation-live-uncut-los-angeles</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06/19/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SoCal Cup: The Showcase</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/socal-cup-the-showcase-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>07/02/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Anime Expo 2026</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/anime-expo-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Gothic Market Los Angeles 2026</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/gothic-market-los-angeles-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>SPOCOM Los Angeles 2026</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/spocom-los-angeles-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Los Angeles Summer International Open IBJJF Jiu-Jitsu Championship</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/los-angeles-summer-international-open-ibjjf-jiu-jitsu-championship</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Collect-A-Con Los Angeles</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/collect-a-con-los-angeles-august-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>08/03/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>NALC 74th Biennial Convention</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/nalc-74th-biennial-convention</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>08/08/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>El Sembrador Ministries - Metanoia Los Angeles</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/el-sembrador-ministries-metanoia-los-angeles</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>08/13/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>KCON LA 2026</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/kcon-la-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>08/15/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>APWU Biennial Convention 2026</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/apwu-biennial-convention-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>08/22/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Smith Chason College Los Angeles Campus Graduation 2026</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/smith-chason-college-los-angeles-campus-graduation-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>09/16/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ASLA 2026 Conference on Landscape Architecture</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/asla-2026-conference-on-landscape-architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>09/19/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Got Sole Los Angeles</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/got-sole-los-angeles</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>09/20/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>California Bridal &amp; Wedding Expo</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/california-bridal-wedding-expo-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>09/20/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Wekfest LA 2026</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/wekfest-la-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>09/23/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>National Black MBA Annual Conference &amp; Exposition</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/national-black-mba-association-conference-exposition</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>09/25/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Riftbound Regional Qualifier</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/riftbound-regional-qualifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>38th Annual SCANPH Conference</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/38th-annual-scanph-conference</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Net Zero Conference 2026</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/net-zero-conference-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>SCG CON Los Angeles 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/scg-con-los-angeles-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>10/17/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>American Academy of Otolaryngology: 2026 AAO OTO EXPO</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/american-academy-of-otolaryngology-2026-aao-oto-expo</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10/30/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>L.A. Comic Con 2026</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/la-comic-con-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>11/04/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Build Expo 2026</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/build-expo-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>12/12/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Spirit Royale Cheer | Marquee Championship Los Angeles</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/spirit-royale-cheer-marquee-los-angeles</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>12/18/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Copa Toque Futsal Festival</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/copa-toque-festival-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>12/19/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Collect-A-Con Los Angeles</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/collect-a-con-los-angeles-december-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>01/06/2027</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>LA Art Show 2027</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/la-art-show-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>01/07/2027</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Modern Language Association Annual Convention 2027</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/modern-language-association-annual-convention-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>01/23/2027</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>The Fit Expo Los Angeles 2027</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/the-fit-expo-los-angeles-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>02/23/2027</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>MakeUp + LUXE PACK in Los Angeles 2027</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/makeup-luxe-pack-in-los-angeles-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>04/01/2027</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Star Wars Celebration 2027</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/star-wars-celebration-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>04/15/2027</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>ACP Internal Medicine Meeting 2027</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/acp-internal-medicine-meeting-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>05/01/2027</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>American Association of Thoracic Surgery Annual Meeting</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.laconventioncenter.com/events/detail/aats-annual-mtg-2027</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update events: 2026-05-26 22:40 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -5336,14 +5336,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5376,11 +5376,62 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/02/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Las Vegas Aces – Commissioner's Cup</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksaces060226</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Dallas Wings – Commissioner's Cup</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparkswings060526</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix past events venue filter using row.hidden for reliable hiding
Switches from style.display manipulation to the hidden attribute so
Bootstrap's display:none !important takes effect regardless of table CSS.
Also re-applies filter after Tablesort reorders rows, and wraps Tablesort
init in try-catch to prevent a sort error from blocking the filter listener.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="SoFi Stadium" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Intuit Dome" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Kia Forum" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Dignity Health Sports Park" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rose Bowl Stadium" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Crypto.com Arena" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="L.A. Memorial Coliseum" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="LA Convention Center" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Past Events" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SoFi Stadium" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intuit Dome" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kia Forum" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dignity Health Sports Park" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rose Bowl Stadium" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto.com Arena" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L.A. Memorial Coliseum" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LA Convention Center" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Past Events" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1720,14 +1720,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="56" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1760,930 +1760,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3888?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270112</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>01/13/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3889?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270113</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>01/16/2026</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3890?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270116</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>01/17/2026</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3891?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270117</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>01/20/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3913?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270120</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>01/21/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3914?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270121</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>01/24/2026</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3915?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270124</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>01/25/2026</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3916?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270125</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>01/28/2026</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3917?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270128</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>01/29/2026</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3918?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270129</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>02/26/2026</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>MORAT</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3967?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=morat_270226</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>06/13/2026</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>7:30 PM</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3671?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260613</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>06/14/2026</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>7:30 PM</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3672?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260614</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>06/20/2026</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>12:30 PM</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>BIG3</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3898?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=big3_260620</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>07/11/2026</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>6:30 PM</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>JOJI: SOLARIS</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3506?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260711</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>07/12/2026</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>6:30 PM</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>JOJI: SOLARIS</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3513?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260712</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>07/17/2026</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Forrest Frank</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3285?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=forrest_frank_260717</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>07/27/2026</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>4:30 PM</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>WWE Monday Night RAW</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3937?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=wwe_monday_night_raw_260727</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Grupo Frontera</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3520?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=grupo_frontera_260807</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>7:30 PM</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Lionel Richie and Earth, Wind &amp; Fire</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3449?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=lionel_richie_earth_wind_fire_260809</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>08/15/2026</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Yeat</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3699?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=yeat_260815</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>08/21/2026</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Ne-Yo &amp; Akon</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3454?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=ne-yo_akon_260821</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>09/03/2026</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>J. Cole</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3492?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>09/04/2026</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>J. Cole</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3498?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>World of Warcraft®: 20 Years of Music</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3683?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=world_of_warcraft_260910</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>09/18/2026</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>8:30 PM</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Maná</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260918</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>09/19/2026</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>8:30 PM</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Maná</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260919</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>09/24/2026</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>6:30 PM</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Kehlani</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/4033?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=kehlani_260924</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>10/03/2026</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>aespa LIVE TOUR – SYNK : COMPLæXITY – in Los Angeles</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3850?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=aespa_live_tour_261003</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>10/10/2026</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>7:30 PM</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>TLC and Salt-N-Pepa</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3613?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=tlc_salt-n-pepa_261010</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>10/17/2026</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Young Miko</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3707?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=young_miko_261017</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>10/24/2026</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>7:30 PM</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Pokémon Night Out</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3674?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=pokemon_night_out_261024</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>11/22/2026</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Three Days Grace</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3149?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=three_days_grace_261122</t>
+          <t>No events found</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2694,14 +1775,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2734,1490 +1815,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>06/07/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>RUSH – Fifty Something</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rush/</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>06/09/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>RUSH – Fifty Something</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rush-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>06/11/2026</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>RUSH – Fifty Something</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rush-3/</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>06/13/2026</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>RUSH – Fifty Something</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rush-4/</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>06/17/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/ariana-grande-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>06/19/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/ariana-grande/</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>06/20/2026</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/ariana-grande-3/</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>06/24/2026</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>MADISON BEER – the locket tour</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/madison-beer/</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>06/26/2026</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>PALOMAZO NORTEÑO – CLASE MAESTRA TOUR</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/palomazo-norteno/</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>06/27/2026</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>A$AP ROCKY – Don't Be Dumb World Tour</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/aap-rocky/</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>06/29/2026</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>ROSALÍA – LUX TOUR 2026</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rosalia/</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>07/01/2026</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>ROSALÍA – LUX TOUR 2026</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rosalia-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>07/08/2026</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>HILARY DUFF – the lucky me tour</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/hilary-duff/</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>07/09/2026</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>HILARY DUFF – the lucky me tour</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/hilary-duff-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>07/11/2026</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>5 SECONDS OF SUMMER – EVERYONE’S A STAR! World Tour</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/5-seconds-of-summer/</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>07/17/2026</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>YOUNG THE GIANT – Victory Garden Tour</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/young-the-giant/</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>07/18/2026</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>EVANESCENCE</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/evanescence/</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>07/31/2026</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>MOTIONLESS IN WHITE – The Sweat and Blood Tour</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/motionless-in-white/</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>08/01/2026</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>IVE – WORLD TOUR [SHOW WHAT I AM] IN LOS ANGELES</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/ive/</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>08/06/2026</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>RÜFÜS DU SOL</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol/</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>RÜFÜS DU SOL</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol-3/</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>08/11/2026</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>RÜFÜS DU SOL</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>08/12/2026</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>RÜFÜS DU SOL</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol-4/</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>08/13/2026</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>RÜFÜS DU SOL – with Ben Böhmer</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol-5/</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>08/14/2026</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>MELANIE MARTINEZ – HADES: THE SACRIFICE</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/melanie-martinez/</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>08/21/2026</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>OMAR COURTZ – POR SI MAÑANA NO ESTOY USA TOUR</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/omar-courtz/</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>09/06/2026</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>CHICAGO &amp; STYX – The Windy Cities Tour - All The Hits... Your Kind of Tour</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/chicago-styx/</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>09/11/2026</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>JOHNNY BLUE SKIES &amp; THE DARK CLOUDS – Mutiny for the Masses 2026 Tour</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/johnny-blue-skies-the-dark-clouds/</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>09/12/2026</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>SODA STEREO – ECOS TOUR</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/soda-stereo/</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>09/23/2026</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>ROBYN – The Sexistential Tour</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/robyn/</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>09/24/2026</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>ROBYN – The Sexistential Tour</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/robyn-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>09/25/2026</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>LILY ALLEN – Lily Allen Performs West End Girl</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/lily-allen/</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>09/26/2026</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>BILLY STRINGS</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/billy-strings-3/</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>09/30/2026</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>DISNEY DESCENDANTS, ZOMBIES &amp; CAMP ROCK: WORLDS COLLIDE CONCERT TOUR</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/worlds-collide-concert-tour/</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>10/03/2026</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>KLANGKUENSTLER – OUTWORLD – Klangkuenstler All Night Long</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/klangkuenstler/</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>10/06/2026</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/mumford-sons/</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>10/07/2026</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/mumford-sons-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>10/09/2026</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/the-neighbourhood/</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>10/10/2026</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>SOMBR – You Are The Reason Tour</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/sombr/</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>10/16/2026</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>JUANES</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/juanes/</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>10/20/2026</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>MONSTA X – 2026 MONSTA X WORLD TOUR [THE X : NEXUS] IN LOS ANGELES</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/monsta-x/</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>10/22/2026</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>DOJA CAT – Tour Ma Vie World Tour</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/doja-cat/</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>10/24/2026</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>GORILLAZ – The Mountain Tour</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/gorillaz-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>11/06/2026</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>DON OMAR – The Last King World Tour</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/don-omar/</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>11/07/2026</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>MON LAFERTE – Femme Fatale Tour</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/mon-laferte/</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>11/12/2026</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>THE SMASHING PUMPKINS – The Rats In A Cage Tour</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/the-smashing-pumpkins/</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>11/13/2026</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>SLAYER – Reign in Blood 40th Anniversary</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/slayer/</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>11/14/2026</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>SLAYER – Reign in Blood 40th Anniversary</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/slayer-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>11/15/2026</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>RAWAYANA – ¿Dónde es el after? World Tour</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rawayana/</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>11/18/2026</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>TEDDY SWIMS – The UGLY Tour</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/teddy-swims/</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/the-neighbourhood-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>12/05/2026</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/the-neighbourhood-3/</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>05/22/2027</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>NIALL HORAN – Dinner Party Live On Tour</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/niall-horan/</t>
+          <t>No events found</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4228,14 +1830,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="39" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4268,174 +1870,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>07/17/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>LA Galaxy vs LAFC</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-lafc</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>07/22/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>LA Galaxy vs St. Louis CITY SC</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-st-louis-city-sc</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>07/25/2026</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Campeón de Campeones 2026</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/campeon-de-campeones-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>08/01/2026</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>LA Galaxy vs FC Dallas</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-fc-dallas</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>08/19/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>LA Galaxy vs San Jose Earthquakes</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-san-jose-earthquakes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>09/05/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>LA Galaxy vs New England Revolution</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-new-england-revolution</t>
+          <t>No events found</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5336,14 +2775,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5376,62 +2815,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>06/02/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Los Angeles Sparks vs Las Vegas Aces – Commissioner's Cup</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.cryptoarena.com/events/detail/sparksaces060226</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Los Angeles Sparks vs Dallas Wings – Commissioner's Cup</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.cryptoarena.com/events/detail/sparkswings060526</t>
+          <t>No events found</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5442,14 +2830,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5482,258 +2870,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>06/11/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>FIFA Fan Festival™ Los Angeles</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/fifa-fan-festival-los-angeles/</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>07/04/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>America250 July 4 Concert</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/america250-july-4-concert/</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>08/29/2026</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>San Jose State vs USC</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/sanjosestate-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>09/04/2026</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Fresno State vs USC</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/fresno-state-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>09/12/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Louisiana vs USC</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/louisiana-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>09/26/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Oregon vs USC</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/oregon-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>10/03/2026</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Washington vs USC</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/washington-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>10/31/2026</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Ohio State vs USC</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/ohio-state-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>11/21/2026</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Maryland vs USC</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/maryland-vs-usc-2026/</t>
+          <t>No events found</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update events: 2026-05-26 23:13 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SoFi Stadium" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intuit Dome" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kia Forum" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dignity Health Sports Park" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rose Bowl Stadium" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto.com Arena" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L.A. Memorial Coliseum" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LA Convention Center" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Past Events" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="SoFi Stadium" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Intuit Dome" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Kia Forum" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dignity Health Sports Park" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Rose Bowl Stadium" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Crypto.com Arena" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="L.A. Memorial Coliseum" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="LA Convention Center" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Past Events" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1720,14 +1720,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1760,11 +1760,930 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3888?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270112</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>01/13/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3889?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270113</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>01/16/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3890?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270116</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>01/17/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3891?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270117</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>01/20/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3913?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270120</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>01/21/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3914?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270121</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>01/24/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3915?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270124</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>01/25/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3916?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270125</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>01/28/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3917?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270128</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>01/29/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3918?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270129</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>02/26/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MORAT</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3967?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=morat_270226</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06/13/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3671?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260613</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06/14/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3672?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260614</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06/20/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>12:30 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>BIG3</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3898?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=big3_260620</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>JOJI: SOLARIS</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3506?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260711</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07/12/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>JOJI: SOLARIS</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3513?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260712</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Forrest Frank</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3285?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=forrest_frank_260717</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07/27/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>4:30 PM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>WWE Monday Night RAW</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3937?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=wwe_monday_night_raw_260727</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Grupo Frontera</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3520?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=grupo_frontera_260807</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Lionel Richie and Earth, Wind &amp; Fire</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3449?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=lionel_richie_earth_wind_fire_260809</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08/15/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Yeat</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3699?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=yeat_260815</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08/21/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ne-Yo &amp; Akon</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3454?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=ne-yo_akon_260821</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>09/03/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>J. Cole</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3492?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>J. Cole</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3498?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>World of Warcraft®: 20 Years of Music</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3683?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=world_of_warcraft_260910</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>09/18/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>8:30 PM</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Maná</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260918</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>09/19/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>8:30 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Maná</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260919</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09/24/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Kehlani</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/4033?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=kehlani_260924</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>aespa LIVE TOUR – SYNK : COMPLæXITY – in Los Angeles</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3850?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=aespa_live_tour_261003</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>TLC and Salt-N-Pepa</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3613?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=tlc_salt-n-pepa_261010</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>10/17/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Young Miko</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3707?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=young_miko_261017</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Pokémon Night Out</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3674?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=pokemon_night_out_261024</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>11/22/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Three Days Grace</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3149?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=three_days_grace_261122</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1775,14 +2694,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1815,11 +2734,1490 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>06/09/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>06/13/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush-4/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06/17/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ariana-grande-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06/19/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ariana-grande/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06/20/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ariana-grande-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06/24/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>MADISON BEER – the locket tour</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/madison-beer/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06/26/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PALOMAZO NORTEÑO – CLASE MAESTRA TOUR</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/palomazo-norteno/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06/27/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>A$AP ROCKY – Don't Be Dumb World Tour</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/aap-rocky/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06/29/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ROSALÍA – LUX TOUR 2026</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rosalia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ROSALÍA – LUX TOUR 2026</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rosalia-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>HILARY DUFF – the lucky me tour</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/hilary-duff/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>HILARY DUFF – the lucky me tour</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/hilary-duff-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>5 SECONDS OF SUMMER – EVERYONE’S A STAR! World Tour</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/5-seconds-of-summer/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>YOUNG THE GIANT – Victory Garden Tour</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/young-the-giant/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07/18/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>EVANESCENCE</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/evanescence/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07/31/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MOTIONLESS IN WHITE – The Sweat and Blood Tour</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/motionless-in-white/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>IVE – WORLD TOUR [SHOW WHAT I AM] IN LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ive/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>08/12/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-4/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>08/13/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL – with Ben Böhmer</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-5/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>08/14/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>MELANIE MARTINEZ – HADES: THE SACRIFICE</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/melanie-martinez/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>08/21/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>OMAR COURTZ – POR SI MAÑANA NO ESTOY USA TOUR</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/omar-courtz/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>09/06/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CHICAGO &amp; STYX – The Windy Cities Tour - All The Hits... Your Kind of Tour</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/chicago-styx/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09/11/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>JOHNNY BLUE SKIES &amp; THE DARK CLOUDS – Mutiny for the Masses 2026 Tour</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/johnny-blue-skies-the-dark-clouds/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>09/12/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SODA STEREO – ECOS TOUR</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/soda-stereo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>09/23/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>ROBYN – The Sexistential Tour</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/robyn/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>09/24/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>ROBYN – The Sexistential Tour</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/robyn-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>09/25/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>LILY ALLEN – Lily Allen Performs West End Girl</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/lily-allen/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>09/26/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>BILLY STRINGS</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/billy-strings-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>09/30/2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>DISNEY DESCENDANTS, ZOMBIES &amp; CAMP ROCK: WORLDS COLLIDE CONCERT TOUR</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/worlds-collide-concert-tour/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>KLANGKUENSTLER – OUTWORLD – Klangkuenstler All Night Long</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/klangkuenstler/</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/mumford-sons/</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/mumford-sons-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>SOMBR – You Are The Reason Tour</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/sombr/</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>10/16/2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>JUANES</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/juanes/</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>10/20/2026</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>MONSTA X – 2026 MONSTA X WORLD TOUR [THE X : NEXUS] IN LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/monsta-x/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>10/22/2026</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>DOJA CAT – Tour Ma Vie World Tour</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/doja-cat/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>GORILLAZ – The Mountain Tour</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/gorillaz-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>11/06/2026</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>DON OMAR – The Last King World Tour</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/don-omar/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>11/07/2026</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>MON LAFERTE – Femme Fatale Tour</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/mon-laferte/</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>11/12/2026</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>THE SMASHING PUMPKINS – The Rats In A Cage Tour</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-smashing-pumpkins/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>11/13/2026</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>SLAYER – Reign in Blood 40th Anniversary</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/slayer/</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>11/14/2026</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>SLAYER – Reign in Blood 40th Anniversary</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/slayer-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>11/15/2026</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>RAWAYANA – ¿Dónde es el after? World Tour</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rawayana/</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>11/18/2026</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>TEDDY SWIMS – The UGLY Tour</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/teddy-swims/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>12/05/2026</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>05/22/2027</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>NIALL HORAN – Dinner Party Live On Tour</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/niall-horan/</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1830,14 +4228,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1870,11 +4268,174 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs LAFC</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-lafc</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>07/22/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs St. Louis CITY SC</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-st-louis-city-sc</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>07/25/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Campeón de Campeones 2026</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/campeon-de-campeones-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs FC Dallas</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-fc-dallas</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>08/19/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs San Jose Earthquakes</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-san-jose-earthquakes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs New England Revolution</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-new-england-revolution</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2775,14 +5336,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2815,11 +5376,90 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/02/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Las Vegas Aces – Commissioner's Cup</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksaces060226</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Dallas Wings – Commissioner's Cup</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparkswings060526</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Alex Warren: Finding Family on the Road – With special guests Nat &amp; Alex Wolff</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/alexwarren060626</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2830,14 +5470,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2870,11 +5510,258 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FIFA Fan Festival™ Los Angeles</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/fifa-fan-festival-los-angeles/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>America250 July 4 Concert</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/america250-july-4-concert/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>08/29/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>San Jose State vs USC</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/sanjosestate-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Fresno State vs USC</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/fresno-state-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>09/12/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Louisiana vs USC</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/louisiana-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>09/26/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Oregon vs USC</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/oregon-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Washington vs USC</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/washington-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10/31/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ohio State vs USC</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/ohio-state-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>11/21/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Maryland vs USC</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/maryland-vs-usc-2026/</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update events: 2026-05-28 21:45 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -16,7 +16,8 @@
     <sheet name="L.A. Memorial Coliseum" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="LA Convention Center" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Dodger Stadium" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Past Events" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Hollywood Bowl" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Past Events" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1721,6 +1722,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Event Name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>No events found</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Update events: 2026-05-28 21:51 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -1722,14 +1722,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1762,11 +1762,2834 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>05/30/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Pitbull – Lil Jon</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4278/2026-05-30/pitbull</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>06/04/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>The Human League – Soft Cell, Alison Moyet</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4283/2026-06-04/the-human-league</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>37th Mariachi USA with Fireworks</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4274/2026-06-06/37th-mariachi-usa-with-fireworks</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Paul Simon</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4359/2026-06-07/paul-simon</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Rod Stewart – Richard Marx</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4258/2026-06-10/rod-stewart</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06/13/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Blue Note Jazz Festival – Day One: Saturday</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4273/2026-06-13/blue-note-jazz-festival</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06/14/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Blue Note Jazz Festival – Day Two: Sunday</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4291/2026-06-14/blue-note-jazz-festival</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06/19/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Chance the Rapper – A Juneteenth Celebration</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4292/2026-06-19/chance-the-rapper</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06/20/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Opening Night at the Bowl: The Best of Broadway</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4247/2026-06-20/opening-night-at-the-bowl-the-best-of-broadway</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06/21/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Reggae Night XXIV – Ziggy Marley, Burning Spear, Zuri Marley, KCRW Festival</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4293/2026-06-21/reggae-night-xxiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06/24/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>The Tabernacle Choir at Temple Square: Songs of Hope Benefit Concert</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4838/2026-06-24/the-tabernacle-choir-at-temple-square-songs-of-hope-benefit-concert</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06/25/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>The Tabernacle Choir at Temple Square: Songs of Hope Benefit Concert</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4839/2026-06-25/the-tabernacle-choir-at-temple-square-songs-of-hope-benefit-concert</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06/27/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>A Roots Picnic Experience – A Great Night in Hip-Hop</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4248/2026-06-27/a-roots-picnic-experience</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07/02/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>July Fourth Fireworks Spectacular with The Beach Boys – with Special Guest John Stamos</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4249/2026-07-02/july-fourth-fireworks-spectacular-with-the-beach-boys</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>July Fourth Fireworks Spectacular with The Beach Boys – with Special Guest John Stamos</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4250/2026-07-03/july-fourth-fireworks-spectacular-with-the-beach-boys</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>July Fourth Fireworks Spectacular with The Beach Boys – with Special Guest John Stamos</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4251/2026-07-04/july-fourth-fireworks-spectacular-with-the-beach-boys</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Herb Alpert &amp; The Tijuana Brass &amp; Other Delights</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4294/2026-07-05/herb-alpert-the-tijuana-brass-other-delights</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Wilkins Conducts Bernstein &amp; Ellington</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4295/2026-07-08/wilkins-conducts-bernstein-ellington</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>The Classical World Cup</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4296/2026-07-09/the-classical-world-cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Music from the Films of Wes Anderson</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4288/2026-07-10/music-from-the-films-of-wes-anderson</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Music from the Films of Wes Anderson</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4289/2026-07-11/music-from-the-films-of-wes-anderson</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>07/12/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Music from the Films of Wes Anderson – KCRW Festival</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4534/2026-07-12/music-from-the-films-of-wes-anderson</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>07/14/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Tchaikovsky &amp; Beethoven</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4297/2026-07-14/tchaikovsky-beethoven</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>07/15/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Salsa Spectacular: Nathy Peluso &amp; Grupo Niche</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4298/2026-07-15/salsa-spectacular-nathy-peluso-grupo-niche</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>07/16/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Mozart &amp; Brahms</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4299/2026-07-16/mozart-brahms</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Let the Sunshine In: The Music of ’69</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4300/2026-07-17/let-the-sunshine-in-the-music-of-69</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>07/18/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Blues Traveler • Gin Blossoms – Spin Doctors</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4301/2026-07-18/blues-traveler-gin-blossoms</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>07/19/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Bob Moses and Cannons: Afterglow Tour – Oxis, KCRW Festival</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4302/2026-07-19/bob-moses-and-cannons-afterglow-tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>07/21/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Joe Hisaishi Film Music Concert – Featuring Studio Ghibli &amp; More</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4303/2026-07-21/joe-hisaishi-film-music-concert</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>07/22/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Joe Hisaishi Film Music Concert – Featuring Studio Ghibli &amp; More</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4304/2026-07-22/joe-hisaishi-film-music-concert</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>07/23/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Joe Hisaishi Film Music Concert – Featuring Studio Ghibli &amp; More</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4305/2026-07-23/joe-hisaishi-film-music-concert</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>07/24/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Smokey Robinson &amp; Gladys Knight: Just the Two of Us</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4259/2026-07-24/smokey-robinson-gladys-knight-just-the-two-of-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>07/25/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Smokey Robinson &amp; Gladys Knight: Just the Two of Us</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4260/2026-07-25/smokey-robinson-gladys-knight-just-the-two-of-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>07/26/2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Boris Brejcha with the Hollywood Bowl Orchestra – KCRW Festival</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4308/2026-07-26/boris-brejcha-with-the-hollywood-bowl-orchestra</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>07/28/2026</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Rhapsody in Blue&amp; Shostakovich</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4309/2026-07-28/rhapsody-in-blue-shostakovich</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>07/29/2026</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Tower of Power and Preservation Hall Jazz Band</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4310/2026-07-29/tower-of-power-and-preservation-hall-jazz-band</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>07/30/2026</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Pictures at an Exhibition</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4311/2026-07-30/pictures-at-an-exhibition</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>07/31/2026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Tchaikovsky Spectacular with Fireworks</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4312/2026-07-31/tchaikovsky-spectacular-with-fireworks</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Tchaikovsky Spectacular with Fireworks</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4313/2026-08-01/tchaikovsky-spectacular-with-fireworks</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>08/02/2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>St. Vincent with the Hollywood Bowl Orchestra – Anoushka Shankar, KCRW Festival</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4314/2026-08-02/st-vincent-with-the-hollywood-bowl-orchestra</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>08/04/2026</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Mendelssohn &amp; Haydn</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4315/2026-08-04/mendelssohn-haydn</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>ZZ Top – with Special Guest Cheap Trick</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4354/2026-08-05/zz-top</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Brahms &amp; Bizet</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4316/2026-08-06/brahms-bizet</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Counting Crows</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4317/2026-08-07/counting-crows</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>08/08/2026</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Counting Crows</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4349/2026-08-08/counting-crows</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>How to Train Your Dragonin Concert</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4319/2026-08-09/how-to-train-your-dragon-in-concert</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>John Mellencamp</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4277/2026-08-10/john-mellencamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Mozart Under the Stars</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4320/2026-08-11/mozart-under-the-stars</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>08/13/2026</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Santana – The Doobie Brothers</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4364/2026-08-13/santana</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>08/14/2026</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Al Green – The Womack Sisters</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4321/2026-08-14/al-green</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>08/15/2026</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Top Gun: Maverickin Concert</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4353/2026-08-15/top-gun-maverick-in-concert</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>08/16/2026</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>YOASOBI</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4844/2026-08-16/yoasobi</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>08/17/2026</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>The Black Crowes &amp; Tedeschi Trucks Band – Whiskey Myers</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4352/2026-08-17/the-black-crowes-tedeschi-trucks-band</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>08/18/2026</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Gershwin, Bernstein &amp; More</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4323/2026-08-18/gershwin-bernstein-more</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>08/19/2026</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Herbie Hancock Celebrates Miles Davis</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4324/2026-08-19/herbie-hancock-celebrates-miles-davis</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>08/20/2026</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Celebrating Gustavo at the Bowl: Beethoven 9</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4325/2026-08-20/celebrating-gustavo-at-the-bowl-beethoven-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>08/21/2026</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Celebrating Gustavo at the Bowl: Dudamel's Playlist</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4326/2026-08-21/celebrating-gustavo-at-the-bowl-dudamels-playlist</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>08/22/2026</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Celebrating Gustavo at the Bowl: Foo Fighters with the LA Phil and YOLA</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4287/2026-08-22/celebrating-gustavo-at-the-bowl-foo-fighters-with-the-la-phil-and-yola</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>08/23/2026</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Celebrating Gustavo at the Bowl: A Musical Legacy</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4361/2026-08-23/celebrating-gustavo-at-the-bowl-a-musical-legacy</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>08/25/2026</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Beethoven’s Fifth</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4330/2026-08-25/beethovens-fifth</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>08/27/2026</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Rachmaninoff &amp; Adams</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4327/2026-08-27/rachmaninoff-adams</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>08/28/2026</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>David Byrne: Who is the Sky?</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4328/2026-08-28/david-byrne-who-is-the-sky</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>08/29/2026</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>David Byrne: Who is the Sky?</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4329/2026-08-29/david-byrne-who-is-the-sky</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>08/30/2026</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Smooth Summer Jazz – The Commodores • Boney James, Sheila E.</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4252/2026-08-30/smooth-summer-jazz</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>08/31/2026</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>MUSE – Portugal. The Man, The Temper Trap</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4837/2026-08-31/muse</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Dvořák &amp; Bruch</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4331/2026-09-01/dvorak-bruch</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>09/03/2026</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Amadeusin Concert</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4332/2026-09-03/amadeus-in-concert</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Maestro of the Movies:A Tribute to John Williams</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4333/2026-09-04/maestro-of-the-movies-a-tribute-to-john-williams</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Maestro of the Movies:A Tribute to John Williams</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4334/2026-09-05/maestro-of-the-movies-a-tribute-to-john-williams</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>09/06/2026</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Maestro of the Movies:A Tribute to John Williams</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4335/2026-09-06/maestro-of-the-movies-a-tribute-to-john-williams</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>09/08/2026</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Los Angeles Ballet at the Bowl</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4336/2026-09-08/los-angeles-ballet-at-the-bowl</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Buddy Guy 90 – with Special Guests Christone “Kingfish” Ingram and his Delta Jam</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4337/2026-09-09/buddy-guy-90</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Ravel, Debussy &amp; Saint-Saëns</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4338/2026-09-10/ravel-debussy-saint-saens</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>09/11/2026</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Fireworks Finale:OneRepublic</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4339/2026-09-11/fireworks-finale-onerepublic</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>09/12/2026</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Fireworks Finale:OneRepublic</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4340/2026-09-12/fireworks-finale-onerepublic</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>09/13/2026</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Lucy Dacus with the Hollywood Bowl Orchestra – Cat Power, KCRW Festival</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4341/2026-09-13/lucy-dacus-with-the-hollywood-bowl-orchestra</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>09/15/2026</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Andrea Bocelli</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4356/2026-09-15/andrea-bocelli</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>09/16/2026</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Andrea Bocelli</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4357/2026-09-16/andrea-bocelli</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>09/18/2026</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Orville Peck</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4355/2026-09-18/orville-peck</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>09/19/2026</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Squeeze – with special guest ADAM ANT, and The English Beat</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4343/2026-09-19/squeeze</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>09/20/2026</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Gregory Alan Isakov with the Hollywood Bowl Orchestra – José González</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4344/2026-09-20/gregory-alan-isakov-with-the-hollywood-bowl-orchestra</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>09/23/2026</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Jazz at Lincoln Center Orchestra with Wynton Marsalis – John Coltrane 100th Celebration with Lakecia Benjamin</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4345/2026-09-23/jazz-at-lincoln-center-orchestra-with-wynton-marsalis</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>09/24/2026</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Jon Bellion</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4509/2026-09-24/jon-bellion</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>09/25/2026</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>The Concert:A Tribute to ABBA – MenAlive</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4254/2026-09-25/the-concert-a-tribute-to-abba</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>09/26/2026</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Rodgers &amp; Hammerstein’s The Sound of Music Sing-A-Long</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4342/2026-09-26/rodgers-hammersteins-the-sound-of-music-sing-a-long</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>09/27/2026</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Jon Batiste</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4346/2026-09-27/jon-batiste</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>09/29/2026</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Lauren Halsey'semajendatwith Erykah Badu – and DJ Pee .Wee (Anderson .Paak), and Charles Gaines Collective with Black Nile</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4843/2026-09-29/lauren-halseys-emajendat-with-erykah-badu</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>09/30/2026</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Rubén Blades &amp; Roberto Delgado Big Band: Fotografías Tour – Silvana Estrada</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4347/2026-09-30/ruben-blades-roberto-delgado-big-band-fotografias-tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>“The Hayley Williams Show”</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4885/2026-10-05/the-hayley-williams-show</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>“The Hayley Williams Show”</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4888/2026-10-06/the-hayley-williams-show</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Empire of the Sun – Polo &amp; Pan, Midnight Gen</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4537/2026-10-08/empire-of-the-sun</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Mac DeMarco</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4363/2026-10-09/mac-demarco</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Jack Johnson – Hermanos Gutiérrez</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4256/2026-10-10/jack-johnson</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>10/11/2026</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Jack Johnson – Hermanos Gutiérrez</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4257/2026-10-11/jack-johnson</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>10/15/2026</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Cynthia Erivo</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4891/2026-10-15/cynthia-erivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>10/17/2026</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>SmartLess Live with Jason Bateman, Sean Hayes, &amp; Will Arnett</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4841/2026-10-17/smartless-live-with-jason-bateman-sean-hayes-will-arnett</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>10/21/2026</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>My Chemical Romance</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4231/2026-10-21/my-chemical-romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>10/23/2026</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>My Chemical Romance</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4232/2026-10-23/my-chemical-romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>My Chemical Romance</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4233/2026-10-24/my-chemical-romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>10/30/2026</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>My Chemical Romance – The Used</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4263/2026-10-30/my-chemical-romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>10/31/2026</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>My Chemical Romance – Thrice</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodbowl.com/events/performances/4264/2026-10-31/my-chemical-romance</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E102" r:id="rId101"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update events: 2026-05-29 21:29 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SoFi Stadium" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intuit Dome" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kia Forum" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dignity Health Sports Park" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rose Bowl Stadium" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto.com Arena" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L.A. Memorial Coliseum" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LA Convention Center" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dodger Stadium" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hollywood Bowl" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Past Events" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="SoFi Stadium" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Intuit Dome" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Kia Forum" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dignity Health Sports Park" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Rose Bowl Stadium" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Crypto.com Arena" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="L.A. Memorial Coliseum" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="LA Convention Center" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Dodger Stadium" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Hollywood Bowl" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Past Events" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11289,14 +11289,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11329,11 +11329,930 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3888?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270112</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>01/13/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3889?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270113</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>01/16/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3890?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270116</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>01/17/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3891?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270117</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>01/20/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3913?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270120</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>01/21/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3914?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270121</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>01/24/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3915?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270124</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>01/25/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3916?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270125</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>01/28/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3917?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270128</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>01/29/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3918?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270129</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>02/26/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MORAT</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3967?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=morat_270226</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06/13/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3671?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260613</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06/14/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3672?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260614</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06/20/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>12:30 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>BIG3</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3898?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=big3_260620</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>JOJI: SOLARIS</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3506?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260711</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07/12/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>JOJI: SOLARIS</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3513?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260712</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Forrest Frank</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3285?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=forrest_frank_260717</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07/27/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>4:30 PM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>WWE Monday Night RAW</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3937?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=wwe_monday_night_raw_260727</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Grupo Frontera</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3520?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=grupo_frontera_260807</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Lionel Richie and Earth, Wind &amp; Fire</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3449?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=lionel_richie_earth_wind_fire_260809</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08/15/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Yeat</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3699?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=yeat_260815</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08/21/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ne-Yo &amp; Akon</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3454?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=ne-yo_akon_260821</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>09/03/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>J. Cole</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3492?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>J. Cole</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3498?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>World of Warcraft®: 20 Years of Music</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3683?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=world_of_warcraft_260910</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>09/18/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>8:30 PM</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Maná</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260918</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>09/19/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>8:30 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Maná</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260919</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09/24/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Kehlani</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/4033?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=kehlani_260924</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>aespa LIVE TOUR – SYNK : COMPLæXITY – in Los Angeles</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3850?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=aespa_live_tour_261003</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>TLC and Salt-N-Pepa</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3613?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=tlc_salt-n-pepa_261010</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>10/17/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Young Miko</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3707?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=young_miko_261017</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Pokémon Night Out</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3674?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=pokemon_night_out_261024</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>11/22/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Three Days Grace</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3149?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=three_days_grace_261122</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11344,14 +12263,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11384,11 +12303,1602 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>06/09/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>06/13/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush-4/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06/17/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ariana-grande-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06/19/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ariana-grande/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06/20/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ariana-grande-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06/24/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>MADISON BEER – the locket tour</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/madison-beer/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06/26/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PALOMAZO NORTEÑO – CLASE MAESTRA TOUR</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/palomazo-norteno/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06/27/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>A$AP ROCKY – Don't Be Dumb World Tour</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/aap-rocky/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06/29/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ROSALÍA – LUX TOUR 2026</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rosalia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ROSALÍA – LUX TOUR 2026</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rosalia-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>HILARY DUFF – the lucky me tour</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/hilary-duff/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>HILARY DUFF – the lucky me tour</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/hilary-duff-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>5 SECONDS OF SUMMER – EVERYONE’S A STAR! World Tour</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/5-seconds-of-summer/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>YOUNG THE GIANT – Victory Garden Tour</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/young-the-giant/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07/18/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>EVANESCENCE</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/evanescence/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07/31/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MOTIONLESS IN WHITE – The Sweat and Blood Tour</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/motionless-in-white/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>IVE – WORLD TOUR [SHOW WHAT I AM] IN LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ive/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>08/12/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-4/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>08/13/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL – with Ben Böhmer</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-5/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>08/14/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>MELANIE MARTINEZ – HADES: THE SACRIFICE</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/melanie-martinez/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>08/21/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>OMAR COURTZ – POR SI MAÑANA NO ESTOY USA TOUR</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/omar-courtz/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>09/06/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CHICAGO &amp; STYX – The Windy Cities Tour - All The Hits... Your Kind of Tour</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/chicago-styx/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09/11/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>JOHNNY BLUE SKIES &amp; THE DARK CLOUDS – Mutiny for the Masses 2026 Tour</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/johnny-blue-skies-the-dark-clouds/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>09/12/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SODA STEREO – ECOS TOUR</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/soda-stereo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>09/23/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>ROBYN – The Sexistential Tour</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/robyn/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>09/24/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>ROBYN – The Sexistential Tour</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/robyn-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>09/25/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>LILY ALLEN – Lily Allen Performs West End Girl</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/lily-allen/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>09/26/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>BILLY STRINGS</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/billy-strings-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>09/30/2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>DISNEY DESCENDANTS, ZOMBIES &amp; CAMP ROCK: WORLDS COLLIDE CONCERT TOUR</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/worlds-collide-concert-tour/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>KLANGKUENSTLER – OUTWORLD – Klangkuenstler All Night Long</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/klangkuenstler/</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/mumford-sons/</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/mumford-sons-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>SOMBR – You Are The Reason Tour</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/sombr/</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>10/16/2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>JUANES</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/juanes/</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>10/20/2026</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>MONSTA X – 2026 MONSTA X WORLD TOUR [THE X : NEXUS] IN LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/monsta-x/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>10/22/2026</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>DOJA CAT – Tour Ma Vie World Tour</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/doja-cat/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>GORILLAZ – The Mountain Tour</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/gorillaz-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>11/06/2026</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>DON OMAR – The Last King World Tour</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/don-omar/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>11/07/2026</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>MON LAFERTE – Femme Fatale Tour</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/mon-laferte/</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>11/12/2026</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>THE SMASHING PUMPKINS – The Rats In A Cage Tour</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-smashing-pumpkins/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>11/13/2026</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>SLAYER – Reign in Blood 40th Anniversary</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/slayer/</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>11/14/2026</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>SLAYER – Reign in Blood 40th Anniversary</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/slayer-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>11/15/2026</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>RAWAYANA – ¿Dónde es el after? World Tour</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rawayana/</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>11/18/2026</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>TEDDY SWIMS – The UGLY Tour</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/teddy-swims/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>12/05/2026</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>12/14/2026</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>GRACIE ABRAMS – The Look at My Life Tour</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/gracie-abrams-5/</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>12/18/2026</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>GRACIE ABRAMS – The Look at My Life Tour</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/gracie-abrams-6/</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>12/19/2026</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>GRACIE ABRAMS – The Look at My Life Tour</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/gracie-abrams-4/</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>12/20/2026</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>GRACIE ABRAMS – The Look at My Life Tour</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/gracie-abrams-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>05/22/2027</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>NIALL HORAN – Dinner Party Live On Tour</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/niall-horan/</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId57"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11399,14 +13909,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11439,11 +13949,174 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs LAFC</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-lafc</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>07/22/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs St. Louis CITY SC</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-st-louis-city-sc</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>07/25/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Campeón de Campeones 2026</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/campeon-de-campeones-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs FC Dallas</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-fc-dallas</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>08/19/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs San Jose Earthquakes</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-san-jose-earthquakes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs New England Revolution</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-new-england-revolution</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12344,14 +15017,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12384,11 +15057,90 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/02/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Las Vegas Aces – Commissioner's Cup</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksaces060226</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Dallas Wings – Commissioner's Cup</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparkswings060526</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Alex Warren: Finding Family on the Road – With special guests Nat &amp; Alex Wolff</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/alexwarren060626</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12399,14 +15151,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12439,11 +15191,258 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FIFA Fan Festival™ Los Angeles</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/fifa-fan-festival-los-angeles/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>America250 July 4 Concert</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/america250-july-4-concert/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>08/29/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>San Jose State vs USC</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/sanjosestate-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Fresno State vs USC</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/fresno-state-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>09/12/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Louisiana vs USC</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/louisiana-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>09/26/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Oregon vs USC</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/oregon-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Washington vs USC</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/washington-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10/31/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ohio State vs USC</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/ohio-state-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>11/21/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Maryland vs USC</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/maryland-vs-usc-2026/</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13652,14 +16651,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13692,11 +16691,1490 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>05/29/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:15 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>vs. Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823946</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>05/30/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>vs. Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823945</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>05/31/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1:10 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>vs. Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823944</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>vs. Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823943</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>vs. Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823942</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1:10 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>vs. Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823941</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06/15/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>vs. Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823938</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06/16/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>vs. Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823939</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06/17/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>12:10 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>vs. Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823940</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06/19/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>vs. Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823936</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06/20/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>vs. Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823937</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06/21/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1:10 PM</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>vs. Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823934</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>07/02/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>vs. San Diego Padres</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823935</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>vs. San Diego Padres</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823933</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>vs. San Diego Padres</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823932</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>4:20 PM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>vs. San Diego Padres</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823931</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07/06/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>vs. Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823930</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07/07/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>vs. Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823929</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>vs. Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823928</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>vs. Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823927</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>6:10 PM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>vs. Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823926</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>07/12/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1:10 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>vs. Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823925</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>07/28/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>vs. Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823923</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>07/29/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>vs. Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823924</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>07/30/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>vs. Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823921</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>07/31/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>vs. Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823922</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>6:10 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>vs. Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823920</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>08/02/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>4:20 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>vs. Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823919</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>vs. Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823918</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>vs. Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823917</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>08/12/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>vs. Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823916</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>08/13/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>vs. Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823915</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>08/14/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>vs. Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823913</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>08/15/2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>4:15 PM</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>vs. Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823914</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>08/16/2026</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1:10 PM</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>vs. Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>08/21/2026</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>vs. Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823911</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>08/22/2026</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>6:10 PM</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>vs. Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823910</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>08/23/2026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1:10 PM</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>vs. Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823909</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>vs. St. Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823908</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>09/02/2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>vs. St. Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823906</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>09/03/2026</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>vs. St. Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823907</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>vs. Washington Nationals</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823905</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>6:10 PM</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>vs. Washington Nationals</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823904</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>09/06/2026</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>vs. Washington Nationals</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823903</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>09/07/2026</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>6:10 PM</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>vs. Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823902</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>09/08/2026</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>vs. Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823901</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>vs. Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823900</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>09/18/2026</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>vs. San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823898</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>09/19/2026</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>6:10 PM</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>vs. San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823899</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>09/20/2026</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>1:10 PM</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>vs. San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823896</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>09/22/2026</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>vs. San Diego Padres</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823897</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>09/23/2026</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>vs. San Diego Padres</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823894</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>09/24/2026</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>vs. San Diego Padres</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823895</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix sidebar width: widen to 220px and allow venue name wrapping
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="SoFi Stadium" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Intuit Dome" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Kia Forum" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Dignity Health Sports Park" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rose Bowl Stadium" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Crypto.com Arena" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="L.A. Memorial Coliseum" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="LA Convention Center" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Dodger Stadium" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Hollywood Bowl" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Past Events" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SoFi Stadium" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intuit Dome" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kia Forum" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dignity Health Sports Park" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rose Bowl Stadium" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto.com Arena" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L.A. Memorial Coliseum" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LA Convention Center" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dodger Stadium" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hollywood Bowl" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Past Events" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11289,14 +11289,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="56" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11329,930 +11329,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3888?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270112</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>01/13/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3889?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270113</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>01/16/2026</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3890?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270116</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>01/17/2026</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3891?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270117</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>01/20/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3913?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270120</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>01/21/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3914?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270121</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>01/24/2026</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3915?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270124</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>01/25/2026</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3916?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270125</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>01/28/2026</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3917?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270128</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>01/29/2026</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Olivia Rodrigo</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3918?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270129</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>02/26/2026</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>MORAT</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3967?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=morat_270226</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>06/13/2026</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>7:30 PM</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3671?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260613</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>06/14/2026</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>7:30 PM</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3672?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260614</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>06/20/2026</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>12:30 PM</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>BIG3</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3898?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=big3_260620</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>07/11/2026</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>6:30 PM</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>JOJI: SOLARIS</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3506?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260711</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>07/12/2026</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>6:30 PM</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>JOJI: SOLARIS</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3513?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260712</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>07/17/2026</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Forrest Frank</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3285?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=forrest_frank_260717</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>07/27/2026</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>4:30 PM</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>WWE Monday Night RAW</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3937?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=wwe_monday_night_raw_260727</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Grupo Frontera</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3520?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=grupo_frontera_260807</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>7:30 PM</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Lionel Richie and Earth, Wind &amp; Fire</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3449?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=lionel_richie_earth_wind_fire_260809</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>08/15/2026</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Yeat</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3699?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=yeat_260815</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>08/21/2026</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Ne-Yo &amp; Akon</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3454?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=ne-yo_akon_260821</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>09/03/2026</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>J. Cole</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3492?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>09/04/2026</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>J. Cole</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3498?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>World of Warcraft®: 20 Years of Music</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3683?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=world_of_warcraft_260910</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>09/18/2026</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>8:30 PM</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Maná</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260918</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>09/19/2026</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>8:30 PM</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Maná</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260919</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>09/24/2026</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>6:30 PM</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Kehlani</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/4033?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=kehlani_260924</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>10/03/2026</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>aespa LIVE TOUR – SYNK : COMPLæXITY – in Los Angeles</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3850?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=aespa_live_tour_261003</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>10/10/2026</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>7:30 PM</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>TLC and Salt-N-Pepa</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3613?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=tlc_salt-n-pepa_261010</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>10/17/2026</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Young Miko</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3707?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=young_miko_261017</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>10/24/2026</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>7:30 PM</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Pokémon Night Out</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3674?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=pokemon_night_out_261024</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>11/22/2026</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Three Days Grace</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.intuitdome.com/events/event-schedule/3149?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=three_days_grace_261122</t>
+          <t>No events found</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12263,14 +11344,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12303,1602 +11384,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>06/07/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>RUSH – Fifty Something</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rush/</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>06/09/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>RUSH – Fifty Something</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rush-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>06/11/2026</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>RUSH – Fifty Something</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rush-3/</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>06/13/2026</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>RUSH – Fifty Something</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rush-4/</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>06/17/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/ariana-grande-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>06/19/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/ariana-grande/</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>06/20/2026</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/ariana-grande-3/</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>06/24/2026</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>MADISON BEER – the locket tour</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/madison-beer/</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>06/26/2026</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>PALOMAZO NORTEÑO – CLASE MAESTRA TOUR</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/palomazo-norteno/</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>06/27/2026</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>A$AP ROCKY – Don't Be Dumb World Tour</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/aap-rocky/</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>06/29/2026</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>ROSALÍA – LUX TOUR 2026</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rosalia/</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>07/01/2026</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>ROSALÍA – LUX TOUR 2026</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rosalia-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>07/08/2026</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>HILARY DUFF – the lucky me tour</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/hilary-duff/</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>07/09/2026</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>HILARY DUFF – the lucky me tour</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/hilary-duff-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>07/11/2026</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>5 SECONDS OF SUMMER – EVERYONE’S A STAR! World Tour</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/5-seconds-of-summer/</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>07/17/2026</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>YOUNG THE GIANT – Victory Garden Tour</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/young-the-giant/</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>07/18/2026</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>EVANESCENCE</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/evanescence/</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>07/31/2026</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>MOTIONLESS IN WHITE – The Sweat and Blood Tour</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/motionless-in-white/</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>08/01/2026</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>IVE – WORLD TOUR [SHOW WHAT I AM] IN LOS ANGELES</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/ive/</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>08/06/2026</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>RÜFÜS DU SOL</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol/</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>RÜFÜS DU SOL</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol-3/</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>08/11/2026</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>RÜFÜS DU SOL</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>08/12/2026</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>RÜFÜS DU SOL</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol-4/</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>08/13/2026</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>RÜFÜS DU SOL – with Ben Böhmer</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rufus-du-sol-5/</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>08/14/2026</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>MELANIE MARTINEZ – HADES: THE SACRIFICE</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/melanie-martinez/</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>08/21/2026</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>OMAR COURTZ – POR SI MAÑANA NO ESTOY USA TOUR</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/omar-courtz/</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>09/06/2026</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>CHICAGO &amp; STYX – The Windy Cities Tour - All The Hits... Your Kind of Tour</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/chicago-styx/</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>09/11/2026</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>JOHNNY BLUE SKIES &amp; THE DARK CLOUDS – Mutiny for the Masses 2026 Tour</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/johnny-blue-skies-the-dark-clouds/</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>09/12/2026</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>SODA STEREO – ECOS TOUR</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/soda-stereo/</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>09/23/2026</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>ROBYN – The Sexistential Tour</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/robyn/</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>09/24/2026</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>ROBYN – The Sexistential Tour</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/robyn-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>09/25/2026</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>LILY ALLEN – Lily Allen Performs West End Girl</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/lily-allen/</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>09/26/2026</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>BILLY STRINGS</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/billy-strings-3/</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>09/30/2026</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>DISNEY DESCENDANTS, ZOMBIES &amp; CAMP ROCK: WORLDS COLLIDE CONCERT TOUR</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/worlds-collide-concert-tour/</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>10/03/2026</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>KLANGKUENSTLER – OUTWORLD – Klangkuenstler All Night Long</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/klangkuenstler/</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>10/06/2026</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/mumford-sons/</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>10/07/2026</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/mumford-sons-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>10/09/2026</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/the-neighbourhood/</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>10/10/2026</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>SOMBR – You Are The Reason Tour</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/sombr/</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>10/16/2026</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>JUANES</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/juanes/</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>10/20/2026</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>MONSTA X – 2026 MONSTA X WORLD TOUR [THE X : NEXUS] IN LOS ANGELES</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/monsta-x/</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>10/22/2026</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>DOJA CAT – Tour Ma Vie World Tour</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/doja-cat/</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>10/24/2026</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>GORILLAZ – The Mountain Tour</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/gorillaz-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>11/06/2026</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>DON OMAR – The Last King World Tour</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/don-omar/</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>11/07/2026</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>MON LAFERTE – Femme Fatale Tour</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/mon-laferte/</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>11/12/2026</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>THE SMASHING PUMPKINS – The Rats In A Cage Tour</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/the-smashing-pumpkins/</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>11/13/2026</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>SLAYER – Reign in Blood 40th Anniversary</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/slayer/</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>11/14/2026</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>SLAYER – Reign in Blood 40th Anniversary</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/slayer-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>11/15/2026</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>RAWAYANA – ¿Dónde es el after? World Tour</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/rawayana/</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>11/18/2026</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>TEDDY SWIMS – The UGLY Tour</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/teddy-swims/</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/the-neighbourhood-2/</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>12/05/2026</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/the-neighbourhood-3/</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>12/14/2026</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>GRACIE ABRAMS – The Look at My Life Tour</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/gracie-abrams-5/</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>12/18/2026</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>GRACIE ABRAMS – The Look at My Life Tour</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/gracie-abrams-6/</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>12/19/2026</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>GRACIE ABRAMS – The Look at My Life Tour</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/gracie-abrams-4/</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>12/20/2026</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>GRACIE ABRAMS – The Look at My Life Tour</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/gracie-abrams-3/</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>05/22/2027</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>NIALL HORAN – Dinner Party Live On Tour</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>https://thekiaforum.com/event/niall-horan/</t>
+          <t>No events found</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId57"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13909,14 +11399,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="39" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13949,174 +11439,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>07/17/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>LA Galaxy vs LAFC</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-lafc</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>07/22/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>LA Galaxy vs St. Louis CITY SC</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-st-louis-city-sc</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>07/25/2026</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Campeón de Campeones 2026</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/campeon-de-campeones-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>08/01/2026</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>LA Galaxy vs FC Dallas</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-fc-dallas</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>08/19/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>LA Galaxy vs San Jose Earthquakes</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-san-jose-earthquakes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>09/05/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>LA Galaxy vs New England Revolution</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-new-england-revolution</t>
+          <t>No events found</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15017,14 +12344,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -15057,90 +12384,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>06/02/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Los Angeles Sparks vs Las Vegas Aces – Commissioner's Cup</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.cryptoarena.com/events/detail/sparksaces060226</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Los Angeles Sparks vs Dallas Wings – Commissioner's Cup</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.cryptoarena.com/events/detail/sparkswings060526</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>06/06/2026</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>7:30 PM</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Alex Warren: Finding Family on the Road – With special guests Nat &amp; Alex Wolff</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.cryptoarena.com/events/detail/alexwarren060626</t>
+          <t>No events found</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15151,14 +12399,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -15191,258 +12439,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>06/11/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>FIFA Fan Festival™ Los Angeles</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/fifa-fan-festival-los-angeles/</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>07/04/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>America250 July 4 Concert</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/america250-july-4-concert/</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>08/29/2026</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>San Jose State vs USC</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/sanjosestate-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>09/04/2026</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Fresno State vs USC</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/fresno-state-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>09/12/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Louisiana vs USC</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/louisiana-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>09/26/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Oregon vs USC</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/oregon-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>10/03/2026</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Washington vs USC</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/washington-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>10/31/2026</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Ohio State vs USC</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/ohio-state-vs-usc-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>11/21/2026</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Maryland vs USC</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lacoliseum.com/events/maryland-vs-usc-2026/</t>
+          <t>No events found</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16651,14 +13652,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16691,1490 +13692,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>05/29/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>7:15 PM</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>vs. Philadelphia Phillies</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823946</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>05/30/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>vs. Philadelphia Phillies</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823945</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>05/31/2026</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1:10 PM</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>vs. Philadelphia Phillies</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823944</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>06/05/2026</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>vs. Los Angeles Angels</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823943</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>06/06/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>vs. Los Angeles Angels</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823942</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>06/07/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1:10 PM</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>vs. Los Angeles Angels</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823941</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>06/15/2026</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>vs. Tampa Bay Rays</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823938</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>06/16/2026</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>vs. Tampa Bay Rays</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823939</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>06/17/2026</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>12:10 PM</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>vs. Tampa Bay Rays</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823940</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>06/19/2026</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>vs. Baltimore Orioles</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823936</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>06/20/2026</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>vs. Baltimore Orioles</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823937</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>06/21/2026</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1:10 PM</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>vs. Baltimore Orioles</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823934</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>07/02/2026</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>vs. San Diego Padres</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823935</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>07/03/2026</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>vs. San Diego Padres</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823933</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>07/04/2026</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>vs. San Diego Padres</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823932</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>4:20 PM</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>vs. San Diego Padres</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823931</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>07/06/2026</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>vs. Colorado Rockies</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823930</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>07/07/2026</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>vs. Colorado Rockies</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823929</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>07/08/2026</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>vs. Colorado Rockies</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823928</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>07/10/2026</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>vs. Arizona Diamondbacks</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823927</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>07/11/2026</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>6:10 PM</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>vs. Arizona Diamondbacks</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823926</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>07/12/2026</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1:10 PM</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>vs. Arizona Diamondbacks</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823925</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>07/28/2026</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>vs. Seattle Mariners</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823923</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>07/29/2026</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>vs. Seattle Mariners</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823924</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>07/30/2026</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>vs. Seattle Mariners</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823921</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>07/31/2026</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>vs. Boston Red Sox</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823922</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>08/01/2026</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>6:10 PM</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>vs. Boston Red Sox</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823920</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>08/02/2026</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>4:20 PM</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>vs. Boston Red Sox</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823919</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>08/10/2026</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>vs. Kansas City Royals</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823918</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>08/11/2026</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>vs. Kansas City Royals</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823917</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>08/12/2026</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>vs. Kansas City Royals</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823916</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>08/13/2026</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>vs. Milwaukee Brewers</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823915</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>08/14/2026</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>vs. Milwaukee Brewers</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823913</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>08/15/2026</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>4:15 PM</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>vs. Milwaukee Brewers</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823914</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>08/16/2026</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>1:10 PM</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>vs. Milwaukee Brewers</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823912</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>08/21/2026</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>vs. Pittsburgh Pirates</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823911</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>08/22/2026</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>6:10 PM</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>vs. Pittsburgh Pirates</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823910</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>08/23/2026</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>1:10 PM</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>vs. Pittsburgh Pirates</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823909</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>09/01/2026</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>vs. St. Louis Cardinals</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823908</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>09/02/2026</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>vs. St. Louis Cardinals</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823906</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>09/03/2026</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>vs. St. Louis Cardinals</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823907</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>09/04/2026</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>vs. Washington Nationals</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823905</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>09/05/2026</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>6:10 PM</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>vs. Washington Nationals</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823904</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>09/06/2026</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>vs. Washington Nationals</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823903</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>6:10 PM</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>vs. Cincinnati Reds</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823902</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>09/08/2026</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>vs. Cincinnati Reds</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823901</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>vs. Cincinnati Reds</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823900</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>09/18/2026</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>vs. San Francisco Giants</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823898</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>09/19/2026</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>6:10 PM</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>vs. San Francisco Giants</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823899</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>09/20/2026</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>1:10 PM</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>vs. San Francisco Giants</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823896</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>09/22/2026</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>vs. San Diego Padres</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823897</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>09/23/2026</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>vs. San Diego Padres</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823894</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>09/24/2026</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>7:10 PM</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>vs. San Diego Padres</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mlb.com/gameday/823895</t>
+          <t>No events found</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update events: 2026-05-29 22:32 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SoFi Stadium" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intuit Dome" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kia Forum" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dignity Health Sports Park" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rose Bowl Stadium" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto.com Arena" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L.A. Memorial Coliseum" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LA Convention Center" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dodger Stadium" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hollywood Bowl" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Past Events" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="SoFi Stadium" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Intuit Dome" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Kia Forum" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dignity Health Sports Park" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Rose Bowl Stadium" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Crypto.com Arena" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="L.A. Memorial Coliseum" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="LA Convention Center" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Dodger Stadium" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Hollywood Bowl" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Past Events" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11289,14 +11289,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11329,11 +11329,930 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>01/12/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3888?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270112</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>01/13/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3889?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270113</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>01/16/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3890?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270116</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>01/17/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3891?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270117</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>01/20/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3913?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270120</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>01/21/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3914?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270121</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>01/24/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3915?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270124</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>01/25/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3916?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270125</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>01/28/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3917?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270128</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>01/29/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Olivia Rodrigo</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3918?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=olivia_rodrigo_270129</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>02/26/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MORAT</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3967?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=morat_270226</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06/13/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3671?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260613</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06/14/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>SHAKIRA: Las Mujeres Ya No Lloran World Tour 2026</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3672?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=shakira_260614</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06/20/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>12:30 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>BIG3</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3898?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=big3_260620</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>JOJI: SOLARIS</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3506?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260711</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07/12/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>JOJI: SOLARIS</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3513?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=joji_260712</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Forrest Frank</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3285?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=forrest_frank_260717</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07/27/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>4:30 PM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>WWE Monday Night RAW</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3937?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=wwe_monday_night_raw_260727</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Grupo Frontera</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3520?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=grupo_frontera_260807</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Lionel Richie and Earth, Wind &amp; Fire</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3449?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=lionel_richie_earth_wind_fire_260809</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08/15/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Yeat</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3699?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=yeat_260815</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08/21/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ne-Yo &amp; Akon</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3454?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=ne-yo_akon_260821</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>09/03/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>J. Cole</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3492?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>J. Cole</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3498?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=j_cole_260903</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>World of Warcraft®: 20 Years of Music</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3683?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=world_of_warcraft_260910</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>09/18/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>8:30 PM</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Maná</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260918</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>09/19/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>8:30 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Maná</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://intuitdome.com/events/mana?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=mana_260919</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09/24/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Kehlani</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/4033?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=kehlani_260924</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>aespa LIVE TOUR – SYNK : COMPLæXITY – in Los Angeles</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3850?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=aespa_live_tour_261003</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>TLC and Salt-N-Pepa</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3613?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=tlc_salt-n-pepa_261010</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>10/17/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Young Miko</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3707?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=young_miko_261017</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Pokémon Night Out</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3674?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=pokemon_night_out_261024</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>11/22/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Three Days Grace</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intuitdome.com/events/event-schedule/3149?utm_source=IDwebsite&amp;utm_medium=eventschedule&amp;utm_campaign=IDevents26&amp;utm_content=three_days_grace_261122</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11344,14 +12263,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11384,11 +12303,1602 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>06/09/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>06/13/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>RUSH – Fifty Something</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rush-4/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06/17/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ariana-grande-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06/19/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ariana-grande/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06/20/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ARIANA GRANDE – The Eternal Sunshine Tour</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ariana-grande-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06/24/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>MADISON BEER – the locket tour</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/madison-beer/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06/26/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PALOMAZO NORTEÑO – CLASE MAESTRA TOUR</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/palomazo-norteno/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06/27/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>A$AP ROCKY – Don't Be Dumb World Tour</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/aap-rocky/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06/29/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ROSALÍA – LUX TOUR 2026</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rosalia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ROSALÍA – LUX TOUR 2026</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rosalia-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>HILARY DUFF – the lucky me tour</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/hilary-duff/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>HILARY DUFF – the lucky me tour</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/hilary-duff-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>5 SECONDS OF SUMMER – EVERYONE’S A STAR! World Tour</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/5-seconds-of-summer/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>YOUNG THE GIANT – Victory Garden Tour</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/young-the-giant/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07/18/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>EVANESCENCE</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/evanescence/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07/31/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MOTIONLESS IN WHITE – The Sweat and Blood Tour</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/motionless-in-white/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>IVE – WORLD TOUR [SHOW WHAT I AM] IN LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/ive/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>08/12/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-4/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>08/13/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL – with Ben Böhmer</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rufus-du-sol-5/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>08/14/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>MELANIE MARTINEZ – HADES: THE SACRIFICE</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/melanie-martinez/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>08/21/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>OMAR COURTZ – POR SI MAÑANA NO ESTOY USA TOUR</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/omar-courtz/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>09/06/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CHICAGO &amp; STYX – The Windy Cities Tour - All The Hits... Your Kind of Tour</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/chicago-styx/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09/11/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>JOHNNY BLUE SKIES &amp; THE DARK CLOUDS – Mutiny for the Masses 2026 Tour</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/johnny-blue-skies-the-dark-clouds/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>09/12/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SODA STEREO – ECOS TOUR</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/soda-stereo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>09/23/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>ROBYN – The Sexistential Tour</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/robyn/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>09/24/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>ROBYN – The Sexistential Tour</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/robyn-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>09/25/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>LILY ALLEN – Lily Allen Performs West End Girl</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/lily-allen/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>09/26/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>BILLY STRINGS</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/billy-strings-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>09/30/2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>DISNEY DESCENDANTS, ZOMBIES &amp; CAMP ROCK: WORLDS COLLIDE CONCERT TOUR</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/worlds-collide-concert-tour/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>KLANGKUENSTLER – OUTWORLD – Klangkuenstler All Night Long</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/klangkuenstler/</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/mumford-sons/</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>MUMFORD &amp; SONS – Prizefighter Tour</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/mumford-sons-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>SOMBR – You Are The Reason Tour</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/sombr/</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>10/16/2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>JUANES</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/juanes/</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>10/20/2026</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>MONSTA X – 2026 MONSTA X WORLD TOUR [THE X : NEXUS] IN LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/monsta-x/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>10/22/2026</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>DOJA CAT – Tour Ma Vie World Tour</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/doja-cat/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>GORILLAZ – The Mountain Tour</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/gorillaz-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>11/06/2026</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>DON OMAR – The Last King World Tour</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/don-omar/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>11/07/2026</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>MON LAFERTE – Femme Fatale Tour</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/mon-laferte/</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>11/12/2026</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>THE SMASHING PUMPKINS – The Rats In A Cage Tour</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-smashing-pumpkins/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>11/13/2026</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>SLAYER – Reign in Blood 40th Anniversary</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/slayer/</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>11/14/2026</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>SLAYER – Reign in Blood 40th Anniversary</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/slayer-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>11/15/2026</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>RAWAYANA – ¿Dónde es el after? World Tour</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/rawayana/</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>11/18/2026</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>TEDDY SWIMS – The UGLY Tour</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/teddy-swims/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>12/05/2026</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>THE NEIGHBOURHOOD – THE WOURLD TOUR</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/the-neighbourhood-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>12/14/2026</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>GRACIE ABRAMS – The Look at My Life Tour</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/gracie-abrams-5/</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>12/18/2026</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>GRACIE ABRAMS – The Look at My Life Tour</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/gracie-abrams-6/</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>12/19/2026</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>GRACIE ABRAMS – The Look at My Life Tour</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/gracie-abrams-4/</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>12/20/2026</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>GRACIE ABRAMS – The Look at My Life Tour</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/gracie-abrams-3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>05/22/2027</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>NIALL HORAN – Dinner Party Live On Tour</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>https://thekiaforum.com/event/niall-horan/</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId57"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11399,14 +13909,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11439,11 +13949,174 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs LAFC</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-lafc</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>07/22/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs St. Louis CITY SC</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-st-louis-city-sc</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>07/25/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Campeón de Campeones 2026</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/campeon-de-campeones-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs FC Dallas</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-fc-dallas</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>08/19/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs San Jose Earthquakes</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-san-jose-earthquakes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs New England Revolution</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-new-england-revolution</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12344,14 +15017,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12384,11 +15057,90 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/02/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Las Vegas Aces – Commissioner's Cup</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksaces060226</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Dallas Wings – Commissioner's Cup</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparkswings060526</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Alex Warren: Finding Family on the Road – With special guests Nat &amp; Alex Wolff</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/alexwarren060626</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12399,14 +15151,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12439,11 +15191,258 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FIFA Fan Festival™ Los Angeles</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/fifa-fan-festival-los-angeles/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>America250 July 4 Concert</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/america250-july-4-concert/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>08/29/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>San Jose State vs USC</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/sanjosestate-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Fresno State vs USC</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/fresno-state-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>09/12/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Louisiana vs USC</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/louisiana-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>09/26/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Oregon vs USC</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/oregon-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Washington vs USC</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/washington-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10/31/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ohio State vs USC</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/ohio-state-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>11/21/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Maryland vs USC</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/maryland-vs-usc-2026/</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13652,14 +16651,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13692,11 +16691,1490 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>05/29/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7:15 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>vs. Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823946</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>05/30/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>vs. Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823945</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>05/31/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1:10 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>vs. Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823944</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>vs. Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823943</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>vs. Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823942</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1:10 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>vs. Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823941</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06/15/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>vs. Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823938</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06/16/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>vs. Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823939</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06/17/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>12:10 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>vs. Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823940</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06/19/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>vs. Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823936</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06/20/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>vs. Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823937</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06/21/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1:10 PM</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>vs. Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823934</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>07/02/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>vs. San Diego Padres</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823935</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>vs. San Diego Padres</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823933</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>vs. San Diego Padres</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823932</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>4:20 PM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>vs. San Diego Padres</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823931</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07/06/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>vs. Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823930</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07/07/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>vs. Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823929</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>vs. Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823928</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>vs. Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823927</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>07/11/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>6:10 PM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>vs. Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823926</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>07/12/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1:10 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>vs. Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823925</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>07/28/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>vs. Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823923</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>07/29/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>vs. Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823924</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>07/30/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>vs. Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823921</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>07/31/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>vs. Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823922</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>6:10 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>vs. Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823920</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>08/02/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>4:20 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>vs. Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823919</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>vs. Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823918</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>vs. Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823917</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>08/12/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>vs. Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823916</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>08/13/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>vs. Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823915</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>08/14/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>vs. Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823913</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>08/15/2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>4:15 PM</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>vs. Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823914</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>08/16/2026</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1:10 PM</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>vs. Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>08/21/2026</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>vs. Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823911</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>08/22/2026</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>6:10 PM</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>vs. Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823910</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>08/23/2026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1:10 PM</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>vs. Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823909</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>vs. St. Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823908</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>09/02/2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>vs. St. Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823906</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>09/03/2026</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>vs. St. Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823907</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>vs. Washington Nationals</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823905</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>6:10 PM</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>vs. Washington Nationals</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823904</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>09/06/2026</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>vs. Washington Nationals</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823903</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>09/07/2026</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>6:10 PM</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>vs. Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823902</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>09/08/2026</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>vs. Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823901</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>vs. Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823900</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>09/18/2026</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>vs. San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823898</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>09/19/2026</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>6:10 PM</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>vs. San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823899</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>09/20/2026</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>1:10 PM</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>vs. San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823896</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>09/22/2026</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>vs. San Diego Padres</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823897</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>09/23/2026</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>vs. San Diego Padres</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823894</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>09/24/2026</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>7:10 PM</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>vs. San Diego Padres</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlb.com/gameday/823895</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update events: 2026-05-29 22:55 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -15017,12 +15017,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
@@ -15135,11 +15135,1103 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>4:00 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Portland Fire – Commissioner's Cup</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksfire060726</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06/11/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Louis Tomlinson – How Did We Get Here? World Tour 2026 with Guests The Aces</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/louistomlinson061126</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06/13/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Ariana Grande – The Eternal Sunshine Tour</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/arianagrande26</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06/17/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Minnesota Lynx – Commissioner's Cup</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparkslynx061726</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06/18/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Diljit Dosanjh – Aura North American Tour 2026</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/diljitdosanjh061826</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06/21/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>5:00 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs New York Liberty</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksliberty062126</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06/25/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Summer Walker – Still Finally Over It Tour</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/summerwalker062526</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06/26/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Kid Cudi Presents: The Rebel Ragers Tour 2026 – With Big Boi, Dot Da Genius, and Chip Tha Ripper</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/kidkudi062626</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06/28/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Don Toliver – Octane Tour with SahBabii, SoFaygo, and Chase B</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/dontoliver062926</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>07/02/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>J-POP SOUND CAPSULE 2026 – ALI | Roselia | SPYAIR | Yoko Kanno | Yoko Takahashi</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/j-pop-sound-capsule-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07/06/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Seattle Storm</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksstorm070626</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Indiana Fever</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksfever070826</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Chicago Sky</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparkssky071026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07/14/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Olivia Dean – The Art of Living - Live 2026</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/oliviadean26</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Monster Jam</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/monsterjam26</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07/22/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Phoenix Mercury</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksmercury072226</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07/28/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs New York Liberty</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksliberty072826</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Megan Moroney – The Cloud 9 Tour with JP Saxe and Solon Holt</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/megan-moroney-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>4:00 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Golden State Valkyries</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksvalkyries080926</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Benson Boone – Wanted Man Tour 2026</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/bensonboone26</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>08/14/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>KCON LA 2026 M Countdown</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/kcon26</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>08/20/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Atlanta Dream</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksdream082026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>08/22/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Connecticut Sun</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparkssun082226</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>08/24/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Atlanta Dream</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksdream082426</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>08/25/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>MAMAMOO – 2026 USA TOUR</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/mamamoo082526</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>08/28/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Washington Mystics</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksmystics082826</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>09/12/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Journey – FINAL FRONTIER TOUR</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/journey091226</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>09/16/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2026 LE SSERAFIM TOUR 'PUREFLOW' IN LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/lesserafim26</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>09/20/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>4:00 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Portland Fire</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksfire092026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>09/24/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks vs Golden State Valkyries</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/sparksvalkyries092426</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>09/25/2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Yandel – SINFÓNICO USA TOUR 2026</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/yandel092526</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>09/28/2026</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Disney Descendants, ZOMBIES &amp; Camp Rock: Worlds Collide Concert Tour – Malachi Barton, Liamani Segura, Dara Reneé, Mekonnen Knife, Hudson Stone, Swayam Bhatia, Kiara Romero, Alexandro Byrd</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/disneydescendants092826</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>JUNGLE – World Tour 2026 with RIO KOSTA</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/jungle101026</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>10/18/2026</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Kacey Musgraves – Middle of Nowhere Tour with Gabriella Rose and Estevie</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/kaceymusgraves26</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Weezer: The Gathering – With special guests The Shins &amp; Silversun Pickups</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/weezer102426</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>11/05/2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>XG WORLD TOUR: THE CORE IN LOS ANGELES</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/xg-110526</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>11/21/2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>KATSEYE – The WILDWORLD Tour</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/katseye26</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>J. Cole – The Fall-Off World Tour</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/jcole090126</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>NCAA West Regional</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cryptoarena.com/events/detail/ncaawestregional2027</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update events: 2026-05-29 23:02 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -13909,7 +13909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -14108,6 +14108,168 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>09/12/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs Seattle Sounders</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-seattle-sounders</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>09/19/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SuperMotocross Playoff Round 2</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/supermotocross</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>09/26/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs Colorado Rapids</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-colorado-rapids</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10/14/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs Portland Timbers FC</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-portland-timbers</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10/17/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs San Diego FC</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-san-diego-fc</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>10/31/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs Austin FC</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-austin-fc</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
@@ -14116,6 +14278,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update events: 2026-06-04 21:17 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -2371,7 +2371,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Salsa Spectacular: Nathy Peluso &amp; Grupo Niche</t>
+          <t>Salsa Spectacular: Nathy Peluso &amp; Grupo Niche – El Marchante</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -14625,7 +14625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14697,34 +14697,34 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>06/27/2026</t>
+          <t>06/20/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>10:30 AM</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Demo Days</t>
+          <t>Picture on the Pitch</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/649/demo-days</t>
+          <t>https://www.rosebowlstadium.com/events/details/652/picture-on-the-pitch</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06/28/2026</t>
+          <t>06/27/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -14739,51 +14739,51 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/650/demo-days</t>
+          <t>https://www.rosebowlstadium.com/events/details/649/demo-days</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>06/28/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3:00 PM</t>
+          <t>10:00 AM</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Foodieland</t>
+          <t>Demo Days</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/637/foodieland</t>
+          <t>https://www.rosebowlstadium.com/events/details/650/demo-days</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>3:00 PM</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -14793,19 +14793,19 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/638/foodieland</t>
+          <t>https://www.rosebowlstadium.com/events/details/637/foodieland</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -14820,142 +14820,142 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/639/foodieland</t>
+          <t>https://www.rosebowlstadium.com/events/details/638/foodieland</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>07/11/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>5:15 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DRUM CORPS AT THE ROSE BOWL</t>
+          <t>Foodieland</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/644/drum-corps-at-the-rose-bowl</t>
+          <t>https://www.rosebowlstadium.com/events/details/639/foodieland</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>07/12/2026</t>
+          <t>07/11/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>5:15 PM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>DRUM CORPS AT THE ROSE BOWL</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/602/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/644/drum-corps-at-the-rose-bowl</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>08/08/2026</t>
+          <t>07/12/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Head in the Clouds</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/642/head-in-the-clouds</t>
+          <t>https://www.rosebowlstadium.com/events/details/602/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>08/08/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>Head in the Clouds</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/603/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/642/head-in-the-clouds</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>08/15/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>6:30 PM</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NOAH KAHAN - THE GREAT DIVIDE TOUR</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/633/noah-kahan-the-great-divide-tour</t>
+          <t>https://www.rosebowlstadium.com/events/details/603/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
@@ -14967,22 +14967,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>08/22/2026</t>
+          <t>08/15/2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>6:30 PM</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Just Like Heaven</t>
+          <t>NOAH KAHAN - THE GREAT DIVIDE TOUR</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/640/just-like-heaven</t>
+          <t>https://www.rosebowlstadium.com/events/details/633/noah-kahan-the-great-divide-tour</t>
         </is>
       </c>
     </row>
@@ -14994,7 +14994,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>08/22/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -15004,12 +15004,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>GUNS N’ ROSES</t>
+          <t>Just Like Heaven</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/579/guns-n'-roses</t>
+          <t>https://www.rosebowlstadium.com/events/details/640/just-like-heaven</t>
         </is>
       </c>
     </row>
@@ -15021,130 +15021,130 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>09/12/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4:15 PM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>SAN DIEGO STATE VS UCLA</t>
+          <t>GUNS N’ ROSES</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/594/san-diego-state-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/579/guns-n'-roses</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>09/13/2026</t>
+          <t>09/12/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>4:15 PM</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>SAN DIEGO STATE VS UCLA</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/604/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/594/san-diego-state-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>09/19/2026</t>
+          <t>09/13/2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>PURDUE VS UCLA</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/595/purdue-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/604/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10/11/2026</t>
+          <t>09/19/2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>PURDUE VS UCLA</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/605/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/595/purdue-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10/17/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>WISCONSIN VS UCLA</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/627/wisconsin-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/605/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
@@ -15156,7 +15156,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10/24/2026</t>
+          <t>10/17/2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -15166,12 +15166,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>MICHIGAN STATE VS UCLA</t>
+          <t>WISCONSIN VS UCLA</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/628/michigan-state-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/627/wisconsin-vs-ucla</t>
         </is>
       </c>
     </row>
@@ -15183,7 +15183,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10/31/2026</t>
+          <t>10/24/2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -15193,159 +15193,159 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>NEVADA VS UCLA</t>
+          <t>MICHIGAN STATE VS UCLA</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/629/nevada-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/628/michigan-state-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>11/08/2026</t>
+          <t>10/31/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>NEVADA VS UCLA</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/606/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/629/nevada-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>11/13/2026</t>
+          <t>11/08/2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ILLINOIS VS UCLA</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/630/illinois-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/606/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>11/28/2026</t>
+          <t>11/13/2026</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>6:00 PM</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>USC VS UCLA</t>
+          <t>ILLINOIS VS UCLA</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/630/illinois-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>12/13/2026</t>
+          <t>11/28/2026</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>USC VS UCLA</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>12/26/2026</t>
+          <t>12/13/2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>HOLIDAY TOURS</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>12/27/2026</t>
+          <t>12/26/2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -15360,19 +15360,19 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>12/28/2026</t>
+          <t>12/27/2026</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -15387,19 +15387,19 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>01/02/2027</t>
+          <t>12/28/2026</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -15414,7 +15414,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
         </is>
       </c>
     </row>
@@ -15436,37 +15436,64 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>HOLIDAY TOURS (duplicate)</t>
+          <t>HOLIDAY TOURS</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/647/holiday-tours-(duplicate)</t>
+          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>01/02/2027</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>HOLIDAY TOURS (duplicate)</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/647/holiday-tours-(duplicate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>01/17/2027</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Rose Bowl Half Marathon &amp; 5K</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>https://www.rosebowlstadium.com/events/details/626/rose-bowl-half-marathon-and-5k</t>
         </is>
@@ -15504,6 +15531,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update events: 2026-06-09 21:26 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -440,14 +440,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -480,1238 +480,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>06/12/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>USA vs. Paraguay – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-usa-paraguay</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>06/15/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>IR Iran vs. New Zealand – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-iran-new-zealand</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>06/18/2026</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Switzerland vs. Bosnia and Herzegovina – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-switzerland-vs-bosnia-and-herzegovina</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>06/21/2026</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Belgium vs. IR Iran – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-belgium-iran</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>06/25/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Türkiye vs. USA – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-turkiye-vs-usa</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>06/28/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Round of 32: TBD vs. TBD – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-roundof32-june28</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>07/02/2026</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Round of 32: TBD vs. TBD – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-roundof32-july2</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>07/10/2026</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Quarterfinals: TBD vs. TBD – FIFA World Cup 26™</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/fifa-world-cup-quarterfinal-july10</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>08/08/2026</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>5:30 PM</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Ed Sheeran – With Myles Smith, Sigrid, Aaron Rowe</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/ed-sheeran-august-8-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>08/14/2026</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>KAROL G - VIAJANDO POR EL MUNDO TROPITOUR</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/karol-g-august-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>08/15/2026</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>KAROL G - VIAJANDO POR EL MUNDO TROPITOUR</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/karol-g-august-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>08/16/2026</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>KAROL G - VIAJANDO POR EL MUNDO TROPITOUR</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/karol-g-august-16</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>08/20/2026</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Chargers vs 49ers – Preseason</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-49ers-preseason-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>08/22/2026</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1:00 PM</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Rams vs. Saints – Preseason</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-saints-preseason-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>08/27/2026</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Chargers vs Rams – Preseason</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-rams-preseason-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>09/01/2026</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>BTS – BTS WORLD TOUR ‘ARIRANG’ IN LOS ANGELES</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/bts-september-1-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>09/02/2026</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>BTS – BTS WORLD TOUR ‘ARIRANG’ IN LOS ANGELES</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/bts-september-2-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>09/05/2026</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>BTS – BTS WORLD TOUR ‘ARIRANG’ IN LOS ANGELES</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/bts-september-5-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>09/06/2026</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>BTS – BTS WORLD TOUR ‘ARIRANG’ IN LOS ANGELES</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/bts-september-6-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>09/13/2026</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>1:25 PM</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Chargers vs. Cardinals – Week 1</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-cardinals-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>09/20/2026</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>1:05 PM</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Chargers vs. Raiders – Week 2</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-raiders-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>09/21/2026</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>5:15 PM</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Rams vs. Giants – Week 2</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-giants-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>09/25/2026</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>09/26/2026</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>09/30/2026</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-september-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>10/02/2026</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>10/03/2026</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>10/06/2026</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-6</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>10/07/2026</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-7</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>10/11/2026</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>1:05 PM</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Chargers vs. Broncos – Week 5</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-broncos-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>10/12/2026</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>5:15 PM</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Rams vs. Bills – Week 5</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-bills-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>10/18/2026</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>1:05 PM</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Rams vs. Cardinals – Week 6</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-cardinals-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>11/01/2026</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>1:05 PM</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Rams vs. Chargers – Week 8</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-chargers-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>11/08/2026</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>1:05 PM</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Chargers vs. Texans – Week 9</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-texans-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>11/15/2026</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-november-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>11/22/2026</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>1:05 PM</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Chargers vs. Jets – Week 11</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-jets-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Wednesday</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>11/25/2026</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Rams vs. Packers – Week 12</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-packers-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>11/29/2026</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>5:20 PM</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Chargers vs. Patriots – Week 12</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-patriots-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>12/03/2026</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>5:15 PM</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Rams vs. Chiefs – Week 13</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-chiefs-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>12/17/2026</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>5:15 PM</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Chargers vs. 49ers – Week 15</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-49ers-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>12/20/2026</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>1:25 PM</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Rams vs. Cowboys – Week 15</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-cowboys-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Chargers vs. Chiefs – Week 17</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-chiefs-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Rams vs. Seahawks – Week 18</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-seahawks-2027</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>02/14/2027</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Super Bowl LXI</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/super-bowl-lxi</t>
+          <t>No events found</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2290,7 +1063,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Salsa Spectacular: Nathy Peluso &amp; Grupo Niche – El Marchante</t>
+          <t>Salsa Spectacular: Nathy Peluso &amp; Grupo Niche – El Marchante with Willy Calderon</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -14983,7 +13756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15077,39 +13850,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06/27/2026</t>
+          <t>06/26/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>5:00 PM</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Demo Days</t>
+          <t>626 ELITE YOUTH FOOTBALL CAMP</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/649/demo-days</t>
+          <t>https://www.rosebowlstadium.com/events/details/661/626-elite-youth-football-camp</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06/28/2026</t>
+          <t>06/27/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -15124,51 +13897,51 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/650/demo-days</t>
+          <t>https://www.rosebowlstadium.com/events/details/649/demo-days</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>06/28/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3:00 PM</t>
+          <t>10:00 AM</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Foodieland</t>
+          <t>Demo Days</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/637/foodieland</t>
+          <t>https://www.rosebowlstadium.com/events/details/650/demo-days</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1:00 PM</t>
+          <t>3:00 PM</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -15178,19 +13951,19 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/638/foodieland</t>
+          <t>https://www.rosebowlstadium.com/events/details/637/foodieland</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -15205,142 +13978,142 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/639/foodieland</t>
+          <t>https://www.rosebowlstadium.com/events/details/638/foodieland</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>07/11/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>5:15 PM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>DRUM CORPS AT THE ROSE BOWL</t>
+          <t>Foodieland</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/644/drum-corps-at-the-rose-bowl</t>
+          <t>https://www.rosebowlstadium.com/events/details/639/foodieland</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>07/12/2026</t>
+          <t>07/11/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>5:15 PM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>DRUM CORPS AT THE ROSE BOWL</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/602/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/644/drum-corps-at-the-rose-bowl</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>08/08/2026</t>
+          <t>07/12/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Head in the Clouds</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/642/head-in-the-clouds</t>
+          <t>https://www.rosebowlstadium.com/events/details/602/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>08/08/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>Head in the Clouds</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/603/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/642/head-in-the-clouds</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>08/15/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>6:30 PM</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>NOAH KAHAN - THE GREAT DIVIDE TOUR</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/633/noah-kahan-the-great-divide-tour</t>
+          <t>https://www.rosebowlstadium.com/events/details/603/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
@@ -15352,22 +14125,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>08/22/2026</t>
+          <t>08/15/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>6:30 PM</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Just Like Heaven</t>
+          <t>NOAH KAHAN - THE GREAT DIVIDE TOUR</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/640/just-like-heaven</t>
+          <t>https://www.rosebowlstadium.com/events/details/633/noah-kahan-the-great-divide-tour</t>
         </is>
       </c>
     </row>
@@ -15379,7 +14152,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>08/22/2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -15389,12 +14162,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>GUNS N’ ROSES</t>
+          <t>Just Like Heaven</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/579/guns-n'-roses</t>
+          <t>https://www.rosebowlstadium.com/events/details/640/just-like-heaven</t>
         </is>
       </c>
     </row>
@@ -15406,130 +14179,130 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>09/12/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>4:15 PM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>SAN DIEGO STATE VS UCLA</t>
+          <t>GUNS N’ ROSES</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/594/san-diego-state-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/579/guns-n'-roses</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>09/13/2026</t>
+          <t>09/12/2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>4:15 PM</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>SAN DIEGO STATE VS UCLA</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/604/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/594/san-diego-state-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>09/19/2026</t>
+          <t>09/13/2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>PURDUE VS UCLA</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/595/purdue-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/604/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10/11/2026</t>
+          <t>09/19/2026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>PURDUE VS UCLA</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/605/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/595/purdue-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10/17/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>WISCONSIN VS UCLA</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/627/wisconsin-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/605/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
@@ -15541,7 +14314,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10/24/2026</t>
+          <t>10/17/2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -15551,12 +14324,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MICHIGAN STATE VS UCLA</t>
+          <t>WISCONSIN VS UCLA</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/628/michigan-state-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/627/wisconsin-vs-ucla</t>
         </is>
       </c>
     </row>
@@ -15568,7 +14341,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10/31/2026</t>
+          <t>10/24/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -15578,159 +14351,159 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>NEVADA VS UCLA</t>
+          <t>MICHIGAN STATE VS UCLA</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/629/nevada-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/628/michigan-state-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>11/08/2026</t>
+          <t>10/31/2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>NEVADA VS UCLA</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/606/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/629/nevada-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>11/13/2026</t>
+          <t>11/08/2026</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ILLINOIS VS UCLA</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/630/illinois-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/606/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>11/28/2026</t>
+          <t>11/13/2026</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>6:00 PM</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>USC VS UCLA</t>
+          <t>ILLINOIS VS UCLA</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/630/illinois-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>12/13/2026</t>
+          <t>11/28/2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>USC VS UCLA</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>12/26/2026</t>
+          <t>12/13/2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>HOLIDAY TOURS</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>12/27/2026</t>
+          <t>12/26/2026</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -15745,19 +14518,19 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>12/28/2026</t>
+          <t>12/27/2026</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -15772,19 +14545,19 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>01/02/2027</t>
+          <t>12/28/2026</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -15799,7 +14572,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
         </is>
       </c>
     </row>
@@ -15821,37 +14594,64 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>HOLIDAY TOURS (duplicate)</t>
+          <t>HOLIDAY TOURS</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/647/holiday-tours-(duplicate)</t>
+          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>01/02/2027</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>HOLIDAY TOURS (duplicate)</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/647/holiday-tours-(duplicate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>01/17/2027</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Rose Bowl Half Marathon &amp; 5K</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>https://www.rosebowlstadium.com/events/details/626/rose-bowl-half-marathon-and-5k</t>
         </is>
@@ -15890,6 +14690,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update events: 2026-06-23 17:21 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -16244,7 +16244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16299,7 +16299,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>PASADENA ELITE YOUTH FOOTBALL CAMP</t>
+          <t>Pasadena Elite Youth Football Camp</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -17067,52 +17067,25 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>01/02/2027</t>
+          <t>01/17/2027</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>HOLIDAY TOURS (duplicate)</t>
+          <t>Rose Bowl Half Marathon &amp; 5K</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rosebowlstadium.com/events/details/647/holiday-tours-(duplicate)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>01/17/2027</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Rose Bowl Half Marathon &amp; 5K</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>https://www.rosebowlstadium.com/events/details/626/rose-bowl-half-marathon-and-5k</t>
         </is>
@@ -17150,7 +17123,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update events: 2026-06-24 17:10 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -16244,7 +16244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16500,81 +16500,81 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>08/08/2026</t>
+          <t>08/02/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>10:00 AM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Head in the Clouds</t>
+          <t>Dena Community Backpack Giveaway</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/642/head-in-the-clouds</t>
+          <t>https://www.rosebowlstadium.com/events/details/663/dena-community-backpack-giveaway</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>08/08/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>Head in the Clouds</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/603/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/642/head-in-the-clouds</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>08/15/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>6:30 PM</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NOAH KAHAN - THE GREAT DIVIDE TOUR</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/633/noah-kahan-the-great-divide-tour</t>
+          <t>https://www.rosebowlstadium.com/events/details/603/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
@@ -16586,22 +16586,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>08/22/2026</t>
+          <t>08/15/2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>6:30 PM</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Just Like Heaven</t>
+          <t>NOAH KAHAN - THE GREAT DIVIDE TOUR</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/640/just-like-heaven</t>
+          <t>https://www.rosebowlstadium.com/events/details/633/noah-kahan-the-great-divide-tour</t>
         </is>
       </c>
     </row>
@@ -16613,7 +16613,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>08/22/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -16623,12 +16623,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>GUNS N’ ROSES</t>
+          <t>Just Like Heaven</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/579/guns-n'-roses</t>
+          <t>https://www.rosebowlstadium.com/events/details/640/just-like-heaven</t>
         </is>
       </c>
     </row>
@@ -16640,157 +16640,157 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>09/12/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4:15 PM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>SAN DIEGO STATE VS UCLA</t>
+          <t>GUNS N’ ROSES</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/594/san-diego-state-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/579/guns-n'-roses</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>09/13/2026</t>
+          <t>09/12/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>4:15 PM</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>SAN DIEGO STATE VS UCLA</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/604/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/594/san-diego-state-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>09/19/2026</t>
+          <t>09/13/2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>PURDUE VS UCLA</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/595/purdue-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/604/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>09/19/2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>5:00 PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Next Rung - Battle for Mental Health</t>
+          <t>PURDUE VS UCLA</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/662/next-rung-battle-for-mental-health</t>
+          <t>https://www.rosebowlstadium.com/events/details/595/purdue-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10/11/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>5:00 PM</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>Next Rung - Battle for Mental Health</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/605/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/662/next-rung-battle-for-mental-health</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10/17/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>WISCONSIN VS UCLA</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/627/wisconsin-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/605/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
@@ -16802,7 +16802,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10/24/2026</t>
+          <t>10/17/2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -16812,12 +16812,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MICHIGAN STATE VS UCLA</t>
+          <t>WISCONSIN VS UCLA</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/628/michigan-state-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/627/wisconsin-vs-ucla</t>
         </is>
       </c>
     </row>
@@ -16829,7 +16829,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10/31/2026</t>
+          <t>10/24/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -16839,159 +16839,159 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>NEVADA VS UCLA</t>
+          <t>MICHIGAN STATE VS UCLA</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/629/nevada-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/628/michigan-state-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>11/08/2026</t>
+          <t>10/31/2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>NEVADA VS UCLA</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/606/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/629/nevada-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>11/13/2026</t>
+          <t>11/08/2026</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ILLINOIS VS UCLA</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/630/illinois-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/606/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>11/28/2026</t>
+          <t>11/13/2026</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>6:00 PM</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>USC VS UCLA</t>
+          <t>ILLINOIS VS UCLA</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/630/illinois-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>12/13/2026</t>
+          <t>11/28/2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>USC VS UCLA</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>12/26/2026</t>
+          <t>12/13/2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>HOLIDAY TOURS</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>12/27/2026</t>
+          <t>12/26/2026</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -17006,19 +17006,19 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>12/28/2026</t>
+          <t>12/27/2026</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -17033,19 +17033,19 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>01/02/2027</t>
+          <t>12/28/2026</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -17060,32 +17060,59 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>01/02/2027</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>HOLIDAY TOURS</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>01/17/2027</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Rose Bowl Half Marathon &amp; 5K</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>https://www.rosebowlstadium.com/events/details/626/rose-bowl-half-marathon-and-5k</t>
         </is>
@@ -17123,6 +17150,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update events: 2026-07-14 16:21 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -17689,13 +17689,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -17972,108 +17972,108 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>5:00 PM</t>
+          <t>8:45 AM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Next Rung - Battle for Mental Health</t>
+          <t>2026 Los Angeles Heart and Stroke Walk</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/662/next-rung-battle-for-mental-health</t>
+          <t>https://www.rosebowlstadium.com/events/details/665/2026-los-angeles-heart-and-stroke-walk</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>7:00 AM</t>
+          <t>5:00 PM</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Race For The Rescues</t>
+          <t>Next Rung - Battle for Mental Health</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/664/race-for-the-rescues</t>
+          <t>https://www.rosebowlstadium.com/events/details/662/next-rung-battle-for-mental-health</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10/11/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>7:00 AM</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>Race For The Rescues</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/605/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/664/race-for-the-rescues</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10/17/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>WISCONSIN VS UCLA</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/627/wisconsin-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/605/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
@@ -18085,7 +18085,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10/24/2026</t>
+          <t>10/17/2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -18095,12 +18095,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MICHIGAN STATE VS UCLA</t>
+          <t>WISCONSIN VS UCLA</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/628/michigan-state-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/627/wisconsin-vs-ucla</t>
         </is>
       </c>
     </row>
@@ -18112,7 +18112,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10/31/2026</t>
+          <t>10/24/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -18122,159 +18122,159 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>NEVADA VS UCLA</t>
+          <t>MICHIGAN STATE VS UCLA</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/629/nevada-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/628/michigan-state-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>11/08/2026</t>
+          <t>10/31/2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>NEVADA VS UCLA</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/606/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/629/nevada-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11/13/2026</t>
+          <t>11/08/2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>ILLINOIS VS UCLA</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/630/illinois-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/606/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>11/28/2026</t>
+          <t>11/13/2026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>6:00 PM</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>USC VS UCLA</t>
+          <t>ILLINOIS VS UCLA</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/630/illinois-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>12/13/2026</t>
+          <t>11/28/2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>USC VS UCLA</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>12/26/2026</t>
+          <t>12/13/2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>HOLIDAY TOURS</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>12/27/2026</t>
+          <t>12/26/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -18289,19 +18289,19 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>12/28/2026</t>
+          <t>12/27/2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -18316,19 +18316,19 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>01/02/2027</t>
+          <t>12/28/2026</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -18343,32 +18343,59 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>01/02/2027</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>HOLIDAY TOURS</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>01/17/2027</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Rose Bowl Half Marathon &amp; 5K</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>https://www.rosebowlstadium.com/events/details/626/rose-bowl-half-marathon-and-5k</t>
         </is>
@@ -18400,6 +18427,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update events: 2026-08-21 19:35 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -669,27 +669,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>09/12/2026</t>
+          <t>09/13/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>1:25 PM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Sip &amp; Stroll at SoFi Stadium – Curated selection of wines, delicious bites &amp; behind-the-scenes tour!</t>
+          <t>Chargers vs. Cardinals – Week 1</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/sofi-tour-sip-wine-stroll-september-12</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-cardinals-2026</t>
         </is>
       </c>
     </row>
@@ -701,88 +701,88 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>09/13/2026</t>
+          <t>09/20/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1:25 PM</t>
+          <t>1:05 PM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Chargers vs. Cardinals – Week 1</t>
+          <t>Chargers vs. Raiders – Week 2</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-cardinals-2026</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-raiders-2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>09/20/2026</t>
+          <t>09/21/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1:05 PM</t>
+          <t>5:15 PM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Chargers vs. Raiders – Week 2</t>
+          <t>Rams vs. Giants – Week 2</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-raiders-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-giants-2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>09/21/2026</t>
+          <t>09/25/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>5:15 PM</t>
+          <t>7:30 PM</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Rams vs. Giants – Week 2</t>
+          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-giants-2026</t>
+          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-25</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>09/25/2026</t>
+          <t>09/26/2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -797,46 +797,46 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-25</t>
+          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-26</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>09/26/2026</t>
+          <t>09/30/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
+          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-26</t>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-september-30</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>09/30/2026</t>
+          <t>10/02/2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -846,24 +846,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee</t>
+          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-september-30</t>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10/02/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -878,19 +878,19 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-2</t>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-3</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -905,19 +905,19 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-3</t>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-6</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10/06/2026</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -932,127 +932,127 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-6</t>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-7</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>1:05 PM</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
+          <t>Chargers vs. Broncos – Week 5</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-7</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-broncos-2026</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10/11/2026</t>
+          <t>10/12/2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1:05 PM</t>
+          <t>5:15 PM</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Chargers vs. Broncos – Week 5</t>
+          <t>Rams vs. Bills – Week 5</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-broncos-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-bills-2026</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10/12/2026</t>
+          <t>10/18/2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>5:15 PM</t>
+          <t>1:05 PM</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Rams vs. Bills – Week 5</t>
+          <t>Rams vs. Cardinals – Week 6</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-bills-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-cardinals-2026</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10/18/2026</t>
+          <t>10/23/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1:05 PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Rams vs. Cardinals – Week 6</t>
+          <t>JAŸ-Z 30</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-cardinals-2026</t>
+          <t>https://www.sofistadium.com/events/detail/jay-z-october-23-2026</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10/23/2026</t>
+          <t>10/24/2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1067,34 +1067,34 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/jay-z-october-23-2026</t>
+          <t>https://www.sofistadium.com/events/detail/jay-z-october-24-2026</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10/24/2026</t>
+          <t>11/01/2026</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>1:05 PM</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>JAŸ-Z 30</t>
+          <t>Rams vs. Chargers – Week 8</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/jay-z-october-24-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-chargers-2026</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>11/01/2026</t>
+          <t>11/08/2026</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1116,12 +1116,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Rams vs. Chargers – Week 8</t>
+          <t>Chargers vs. Texans – Week 9</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-chargers-2026</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-texans-2026</t>
         </is>
       </c>
     </row>
@@ -1133,34 +1133,34 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>11/08/2026</t>
+          <t>11/15/2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1:05 PM</t>
+          <t>7:30 PM</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Chargers vs. Texans – Week 9</t>
+          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-texans-2026</t>
+          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-november-15</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>11/15/2026</t>
+          <t>11/16/2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1175,115 +1175,115 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-november-15</t>
+          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-november-16</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>11/16/2026</t>
+          <t>11/22/2026</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>1:05 PM</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
+          <t>Chargers vs. Jets – Week 11</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-november-16</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-jets-2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>11/22/2026</t>
+          <t>11/25/2026</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1:05 PM</t>
+          <t>5:00 PM</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Chargers vs. Jets – Week 11</t>
+          <t>Rams vs. Packers – Week 12</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-jets-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-packers-2026</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>11/25/2026</t>
+          <t>11/29/2026</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>5:00 PM</t>
+          <t>5:20 PM</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Rams vs. Packers – Week 12</t>
+          <t>Chargers vs. Patriots – Week 12</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-packers-2026</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-patriots-2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>11/29/2026</t>
+          <t>12/03/2026</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>5:20 PM</t>
+          <t>5:15 PM</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Chargers vs. Patriots – Week 12</t>
+          <t>Rams vs. Chiefs – Week 13</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-patriots-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-chiefs-2026</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>12/03/2026</t>
+          <t>12/17/2026</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1305,66 +1305,66 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Rams vs. Chiefs – Week 13</t>
+          <t>Chargers vs. 49ers – Week 15</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-chiefs-2026</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-49ers-2026</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>12/17/2026</t>
+          <t>12/20/2026</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>5:15 PM</t>
+          <t>1:25 PM</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Chargers vs. 49ers – Week 15</t>
+          <t>Rams vs. Cowboys – Week 15</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-49ers-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-cowboys-2026</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>12/20/2026</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1:25 PM</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Rams vs. Cowboys – Week 15</t>
+          <t>Chargers vs. Chiefs – Week 17</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-cowboys-2026</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-chiefs-2026</t>
         </is>
       </c>
     </row>
@@ -1386,64 +1386,37 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Chargers vs. Chiefs – Week 17</t>
+          <t>Rams vs. Seahawks – Week 18</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-chiefs-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-seahawks-2027</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>02/14/2027</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
           <t>TBA</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Rams vs. Seahawks – Week 18</t>
+          <t>Super Bowl LXI</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-seahawks-2027</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>02/14/2027</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Super Bowl LXI</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>https://www.sofistadium.com/events/detail/super-bowl-lxi</t>
         </is>
@@ -1486,7 +1459,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21232,7 +21204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -21407,189 +21379,189 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>09/19/2026</t>
+          <t>09/17/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>12:00 PM</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>PURDUE VS UCLA</t>
+          <t>Rose Bowl Quarterbacks Club</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/595/purdue-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/671/rose-bowl-quarterbacks-club</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>09/27/2026</t>
+          <t>09/19/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>8:30 AM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026 Bimbo Global Race</t>
+          <t>PURDUE VS UCLA</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/669/2026-bimbo-global-race</t>
+          <t>https://www.rosebowlstadium.com/events/details/595/purdue-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>09/27/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>8:45 AM</t>
+          <t>8:30 AM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026 Los Angeles Heart and Stroke Walk</t>
+          <t>2026 Bimbo Global Race</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/665/2026-los-angeles-heart-and-stroke-walk</t>
+          <t>https://www.rosebowlstadium.com/events/details/669/2026-bimbo-global-race</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>5:00 PM</t>
+          <t>8:45 AM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Next Rung - Battle for Mental Health</t>
+          <t>2026 Los Angeles Heart and Stroke Walk</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/662/next-rung-battle-for-mental-health</t>
+          <t>https://www.rosebowlstadium.com/events/details/665/2026-los-angeles-heart-and-stroke-walk</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>7:00 AM</t>
+          <t>5:00 PM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Race For The Rescues</t>
+          <t>Next Rung - Battle for Mental Health</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/664/race-for-the-rescues</t>
+          <t>https://www.rosebowlstadium.com/events/details/662/next-rung-battle-for-mental-health</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10/11/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>7:00 AM</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>Race For The Rescues</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/605/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/664/race-for-the-rescues</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10/17/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>WISCONSIN VS UCLA</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/627/wisconsin-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/605/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
@@ -21601,7 +21573,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10/24/2026</t>
+          <t>10/17/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -21611,12 +21583,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MICHIGAN STATE VS UCLA</t>
+          <t>WISCONSIN VS UCLA</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/628/michigan-state-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/627/wisconsin-vs-ucla</t>
         </is>
       </c>
     </row>
@@ -21628,7 +21600,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10/31/2026</t>
+          <t>10/24/2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -21638,159 +21610,159 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>NEVADA VS UCLA</t>
+          <t>MICHIGAN STATE VS UCLA</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/629/nevada-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/628/michigan-state-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>11/08/2026</t>
+          <t>10/31/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>NEVADA VS UCLA</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/606/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/629/nevada-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>11/13/2026</t>
+          <t>11/08/2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ILLINOIS VS UCLA</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/630/illinois-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/606/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11/28/2026</t>
+          <t>11/13/2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>6:00 PM</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>USC VS UCLA</t>
+          <t>ILLINOIS VS UCLA</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/630/illinois-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>12/13/2026</t>
+          <t>11/28/2026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>USC VS UCLA</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>12/26/2026</t>
+          <t>12/13/2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>HOLIDAY TOURS</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>12/27/2026</t>
+          <t>12/26/2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -21805,19 +21777,19 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>12/28/2026</t>
+          <t>12/27/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -21832,61 +21804,61 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>01/01/2027</t>
+          <t>12/28/2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Rose Bowl Game</t>
+          <t>HOLIDAY TOURS</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/667/rose-bowl-game</t>
+          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>01/02/2027</t>
+          <t>01/01/2027</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>HOLIDAY TOURS</t>
+          <t>Rose Bowl Game</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/667/rose-bowl-game</t>
         </is>
       </c>
     </row>
@@ -21903,42 +21875,69 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>10:00 PM</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>HOLIDAY HUDDLE</t>
+          <t>HOLIDAY TOURS</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/668/holiday-huddle</t>
+          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>01/02/2027</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>10:00 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>HOLIDAY HUDDLE</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/668/holiday-huddle</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>01/17/2027</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Rose Bowl Half Marathon &amp; 5K</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>https://www.rosebowlstadium.com/events/details/626/rose-bowl-half-marathon-and-5k</t>
         </is>
@@ -21971,6 +21970,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update events: 2026-08-21 20:16 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -17,7 +17,8 @@
     <sheet name="LA Convention Center" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Dodger Stadium" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Hollywood Bowl" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Past Events" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Hollywood Palladium" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Past Events" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2859,6 +2860,1064 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Event Name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>08/21/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Maddix</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/maddix-hollywood-california-08-21-2026/event/09006452F92BBD18</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>08/22/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Goldfinger w/ The Vandals, The Suicide Machines, Pulley &amp; Sullvn</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/goldfinger-w-the-vandals-the-suicide-hollywood-california-08-22-2026/event/0900643EDCF7E666</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>08/24/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>The Breeders</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/the-breeders-hollywood-california-08-24-2026/event/09006429E509D273</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>08/25/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Right After You Left ft Andrew Santino, Josh Johnson &amp; Special Guests</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/right-after-you-left-ft-andrew-hollywood-california-08-25-2026/event/09006513CF99C753</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>08/28/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ian Asher</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/ian-asher-hollywood-california-08-28-2026/event/090064B4D6CF7477</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>08/29/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Courtney Barnett - Creature of Habit Tour</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/courtney-barnett-creature-of-habit-tour-hollywood-california-08-29-2026/event/0900642DC297B2B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Morgan Jay - Right After You Left - Vinyl Room @ the Palladium</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/morgan-jay-right-after-you-left-hollywood-california-09-01-2026/event/09006513CFA1C765</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>09/02/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>The Garden</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/the-garden-hollywood-california-09-02-2026/event/090064CCAF8AD996</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>The Charlatans UK - North American Tour 2026</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/the-charlatans-uk-north-american-tour-hollywood-california-09-04-2026/event/09006490B9D99051</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>William Black</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/william-black-hollywood-california-09-05-2026/event/090064DA849B4543</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09/06/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Stephen Wilson Jr. - Gary The Torch Tour</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/stephen-wilson-jr-gary-the-torch-hollywood-california-09-06-2026/event/0900646DE9B21460</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ArtDontSleep &amp; KCRW Presents Cortex</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/artdontsleep-kcrw-presents-cortex-hollywood-california-09-09-2026/event/090064E688CB3319</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Polyphia Tour MMXXVI</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/polyphia-tour-mmxxvi-hollywood-california-09-10-2026/event/090064CAF59921C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>09/11/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>San Holo presents TRUE LOVE IN A MADE UP WORLD</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/san-holo-presents-true-love-in-hollywood-california-09-11-2026/event/0900647EA88187AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09/14/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Jack Harlow - Monica Tour</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/jack-harlow-monica-tour-hollywood-california-09-14-2026/event/09006471809E4335</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>09/16/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Starbomb featuring DJ Commander Meouch - Probably The Only Tour Ever</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/starbomb-featuring-dj-commander-meouch-probably-hollywood-california-09-16-2026/event/090064B02490A2FE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>09/17/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Citizen</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/citizen-hollywood-california-09-17-2026/event/09006495AE13A478</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>09/18/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Gravedgr</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/gravedgr-hollywood-california-09-18-2026/event/090064CCD2313334</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>09/19/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Peter Hook &amp; The Light - North American Tour 2026</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/peter-hook-the-light-north-american-hollywood-california-09-19-2026/event/09006312976815C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>09/20/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Chance The Rapper - Coloring Book 10 Year Anniversary Tour</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/chance-the-rapper-coloring-book-10-hollywood-california-09-20-2026/event/090064D2E6C0EEDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>09/25/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Overmono - Pure Devotion World Tour</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/overmono-pure-devotion-world-tour-hollywood-california-09-25-2026/event/090064B0F998CD8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>09/26/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Dexter and The Moonrocks</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/dexter-and-the-moonrocks-hollywood-california-09-26-2026/event/090064C49BC79F9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>09/28/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>JACK WHITE LIVE 2026</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/jack-white-live-2026-hollywood-california-09-28-2026/event/090064878E2C68FC</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>09/29/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>JACK WHITE LIVE 2026</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/jack-white-live-2026-hollywood-california-09-29-2026/event/090064878E416938</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>09/30/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>SUGAR - Love You Even Still 2026 World Tour</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/sugar-love-you-even-still-2026-hollywood-california-09-30-2026/event/09006434A1B88DDD</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>10/01/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Social Distortion</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/social-distortion-hollywood-california-10-01-2026/event/09006455A7CEBF3A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>10/02/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Social Distortion</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/social-distortion-hollywood-california-10-02-2026/event/09006455A7E2BF66</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>EsDeeKid - Council House Rat Tour</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/esdeekid-council-house-rat-tour-hollywood-california-10-07-2026/event/090064F0F51C470D</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SCHOOLBOY Q - 10 Years of Blank Face LP</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/schoolboy-q-10-years-of-blank-hollywood-california-10-09-2026/event/090064ED8E51464F</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Mastodon</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/mastodon-hollywood-california-10-10-2026/event/090064BD4B3E8A67</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>10/11/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Loathe: A Stranger to You</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/loathe-a-stranger-to-you-hollywood-california-10-11-2026/event/090064987F5E5CAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>10/15/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Iration</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/iration-hollywood-california-10-15-2026/event/090064DA83834398</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>10/16/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Boy Harsher</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/boy-harsher-hollywood-california-10-16-2026/event/090064C325F30F8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>10/18/2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>SEX PISTOLS (Steve Jones, Paul Cook, Glen Matlock) feat. Frank Carter</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/sex-pistols-steve-jones-paul-cook-hollywood-california-10-18-2026/event/0900627AEA50512B</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>10/20/2026</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Modest Mouse</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/modest-mouse-hollywood-california-10-20-2026/event/0900648FCF4AA265</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>10/21/2026</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>fakemink: a Terrible Beauty. - The Tour. part 2</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/fakemink-a-terrible-beauty-the-tour-hollywood-california-10-21-2026/event/09006513D701D1D2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Update events: 2026-08-21 20:57 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -2865,7 +2865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3871,6 +3871,600 @@
       <c r="E37" s="2" t="inlineStr">
         <is>
           <t>https://www.ticketmaster.com/fakemink-a-terrible-beauty-the-tour-hollywood-california-10-21-2026/event/09006513D701D1D2</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>10/23/2026</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Two Friends</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/two-friends-hollywood-california-10-23-2026/event/090064A4ABA1D8E9</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>10/24/2026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Two Friends</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/two-friends-hollywood-california-10-24-2026/event/090064A4AC83DB33</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>10/25/2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>XAVIER WULF - THE COOL WORLD TOUR</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/xavier-wulf-the-cool-world-tour-hollywood-california-10-25-2026/event/090064F4D3499ECC</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>11/03/2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>10 Years of 6LACK Tour</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/10-years-of-6lack-tour-hollywood-california-11-03-2026/event/090064B61A982EB0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>11/06/2026</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Carl Cox</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/carl-cox-hollywood-california-11-06-2026/event/09006503777A2802</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>11/07/2026</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>TINASHE - ONE NIGHT WITH A POPSTAR</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/tinashe-one-night-with-a-popstar-hollywood-california-11-07-2026/event/090064F499E14E53</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>11/11/2026</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Turnover - Down On Earth Tour</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/turnover-down-on-earth-tour-hollywood-california-11-11-2026/event/090064D2BD80BA7E</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>11/12/2026</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Sabaton: Legends on Tour</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/sabaton-legends-on-tour-hollywood-california-11-12-2026/event/09006455C0F6592F</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>11/13/2026</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Underoath - Define the Great Line 20th Anniversary Tour</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/underoath-define-the-great-line-20th-hollywood-california-11-13-2026/event/090064F50081FBAA</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>11/14/2026</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Insomniac presents Valentino Khan</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/insomniac-presents-valentino-khan-hollywood-california-11-14-2026/event/090064BDA75FB781</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>11/15/2026</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>LIL PEEP 30TH BIRTHDAY CELEBRATION</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/lil-peep-30th-birthday-celebration-hollywood-california-11-15-2026/event/090065068E7555BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>11/19/2026</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>BOLO</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/bolo-hollywood-california-11-19-2026/event/0900650CAE378D35</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>11/20/2026</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Rhye</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/rhye-hollywood-california-11-20-2026/event/090064C32762134F</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>11/21/2026</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>BOLO</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/bolo-hollywood-california-11-21-2026/event/09006506891F4B69</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>11/22/2026</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>BOLO</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/bolo-hollywood-california-11-22-2026/event/0900650CD725EBE0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>11/27/2026</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Insomniac presents DEVAULT</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/insomniac-presents-devault-hollywood-california-11-27-2026/event/090064CD1DD77F50</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Fetty Wap: Nostalgia Tour</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/fetty-wap-nostalgia-tour-hollywood-california-12-04-2026/event/090064AB3B0AFD8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>12/05/2026</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Thundercat: Distracted AF Tour</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/thundercat-distracted-af-tour-hollywood-california-12-05-2026/event/090064E88ABF42B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>12/11/2026</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>BASSRUSH presents Virtual Riot &amp; Blanke - Far From Home Tour</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/bassrush-presents-virtual-riot-blanke-far-hollywood-california-12-11-2026/event/090064D6B46E7E1D</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>12/18/2026</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Beartooth: Pure Ecstasy World Tour</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/beartooth-pure-ecstasy-world-tour-hollywood-california-12-18-2026/event/090064AB1333BE7A</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>12/19/2026</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Earl Sweatshirt &amp; MIKE Home on the Range Tour 2026</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/earl-sweatshirt-mike-home-on-the-hollywood-california-12-19-2026/event/09006466BA1DF6D7</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>04/04/2027</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Nothing But Thieves: The Stray Dogs World Tour</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticketmaster.com/nothing-but-thieves-the-stray-dogs-hollywood-california-04-04-2027/event/090064B61FAB46C9</t>
         </is>
       </c>
     </row>
@@ -3912,6 +4506,28 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId58"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update events: 2026-08-21 23:35 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -27589,14 +27589,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -27629,11 +27629,258 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No events found</t>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>08/29/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>San Jose State vs USC</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/sanjosestate-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Fresno State vs USC</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/fresno-state-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>09/12/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Louisiana vs USC</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/louisiana-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>09/26/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Oregon vs USC</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/oregon-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Washington vs USC</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/washington-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>MEXTOUR: Mexico vs. Chile</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/mextour-mexico-vs-chile/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10/31/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Ohio State vs USC</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/ohio-state-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>11/21/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Maryland vs USC</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/maryland-vs-usc-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>12/12/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>JOHN SUMMIT – CTRL ESCAPE TOUR</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lacoliseum.com/events/john-summit-ctrl-escape-tour/</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update events: 2026-08-28 23:59 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -481,39 +481,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>08/27/2026</t>
+          <t>09/01/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Chargers vs Rams – Preseason</t>
+          <t>BTS – BTS WORLD TOUR ‘ARIRANG’ IN LOS ANGELES</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-rams-preseason-2026</t>
+          <t>https://www.sofistadium.com/events/detail/bts-september-1-2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>09/01/2026</t>
+          <t>09/02/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -528,19 +528,19 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/bts-september-1-2026</t>
+          <t>https://www.sofistadium.com/events/detail/bts-september-2-2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>09/02/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,19 +555,19 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/bts-september-2-2026</t>
+          <t>https://www.sofistadium.com/events/detail/bts-september-5-2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/bts-september-5-2026</t>
+          <t>https://www.sofistadium.com/events/detail/bts-september-6-2026</t>
         </is>
       </c>
     </row>
@@ -594,22 +594,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>09/06/2026</t>
+          <t>09/13/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>1:25 PM</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>BTS – BTS WORLD TOUR ‘ARIRANG’ IN LOS ANGELES</t>
+          <t>Chargers vs. Cardinals – Week 1</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/bts-september-6-2026</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-cardinals-2026</t>
         </is>
       </c>
     </row>
@@ -621,88 +621,88 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>09/13/2026</t>
+          <t>09/20/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1:25 PM</t>
+          <t>1:05 PM</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Chargers vs. Cardinals – Week 1</t>
+          <t>Chargers vs. Raiders – Week 2</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-cardinals-2026</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-raiders-2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>09/20/2026</t>
+          <t>09/21/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1:05 PM</t>
+          <t>5:15 PM</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Chargers vs. Raiders – Week 2</t>
+          <t>Rams vs. Giants – Week 2</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-raiders-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-giants-2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>09/21/2026</t>
+          <t>09/25/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>5:15 PM</t>
+          <t>7:30 PM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Rams vs. Giants – Week 2</t>
+          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-giants-2026</t>
+          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-25</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>09/25/2026</t>
+          <t>09/26/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -717,46 +717,46 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-25</t>
+          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-26</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>09/26/2026</t>
+          <t>09/30/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
+          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-september-26</t>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-september-30</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>09/30/2026</t>
+          <t>10/02/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -766,24 +766,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee</t>
+          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-september-30</t>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10/02/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -798,19 +798,19 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-2</t>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-3</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -825,19 +825,19 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-3</t>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-6</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10/06/2026</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -852,127 +852,127 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-6</t>
+          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-7</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>1:05 PM</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bruno Mars – The Romantic Tour with Anderson.Paak as DJ Pee.Wee and Raye</t>
+          <t>Chargers vs. Broncos – Week 5</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/bruno-mars-october-7</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-broncos-2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10/11/2026</t>
+          <t>10/12/2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1:05 PM</t>
+          <t>5:15 PM</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Chargers vs. Broncos – Week 5</t>
+          <t>Rams vs. Bills – Week 5</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-broncos-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-bills-2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10/12/2026</t>
+          <t>10/18/2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>5:15 PM</t>
+          <t>1:05 PM</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Rams vs. Bills – Week 5</t>
+          <t>Rams vs. Cardinals – Week 6</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-bills-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-cardinals-2026</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10/18/2026</t>
+          <t>10/23/2026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1:05 PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Rams vs. Cardinals – Week 6</t>
+          <t>JAŸ-Z 30</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-cardinals-2026</t>
+          <t>https://www.sofistadium.com/events/detail/jay-z-october-23-2026</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10/23/2026</t>
+          <t>10/24/2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -987,34 +987,34 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/jay-z-october-23-2026</t>
+          <t>https://www.sofistadium.com/events/detail/jay-z-october-24-2026</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10/24/2026</t>
+          <t>11/01/2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>1:05 PM</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>JAŸ-Z 30</t>
+          <t>Rams vs. Chargers – Week 8</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/jay-z-october-24-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-chargers-2026</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>11/01/2026</t>
+          <t>11/08/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1036,12 +1036,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Rams vs. Chargers – Week 8</t>
+          <t>Chargers vs. Texans – Week 9</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-chargers-2026</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-texans-2026</t>
         </is>
       </c>
     </row>
@@ -1053,34 +1053,34 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>11/08/2026</t>
+          <t>11/15/2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1:05 PM</t>
+          <t>7:30 PM</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Chargers vs. Texans – Week 9</t>
+          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-texans-2026</t>
+          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-november-15</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>11/15/2026</t>
+          <t>11/16/2026</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1095,115 +1095,115 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-november-15</t>
+          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-november-16</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>11/16/2026</t>
+          <t>11/22/2026</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>1:05 PM</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>The R&amp;B Tour - Starring Usher Raymond &amp; Chris Brown</t>
+          <t>Chargers vs. Jets – Week 11</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chris-brown-usher-november-16</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-jets-2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>11/22/2026</t>
+          <t>11/25/2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1:05 PM</t>
+          <t>5:00 PM</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Chargers vs. Jets – Week 11</t>
+          <t>Rams vs. Packers – Week 12</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-jets-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-packers-2026</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>11/25/2026</t>
+          <t>11/29/2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>5:00 PM</t>
+          <t>5:20 PM</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Rams vs. Packers – Week 12</t>
+          <t>Chargers vs. Patriots – Week 12</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-packers-2026</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-patriots-2026</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>11/29/2026</t>
+          <t>12/03/2026</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>5:20 PM</t>
+          <t>5:15 PM</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Chargers vs. Patriots – Week 12</t>
+          <t>Rams vs. Chiefs – Week 13</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-patriots-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-chiefs-2026</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>12/03/2026</t>
+          <t>12/17/2026</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1225,66 +1225,66 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Rams vs. Chiefs – Week 13</t>
+          <t>Chargers vs. 49ers – Week 15</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-chiefs-2026</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-49ers-2026</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>12/17/2026</t>
+          <t>12/20/2026</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>5:15 PM</t>
+          <t>1:25 PM</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Chargers vs. 49ers – Week 15</t>
+          <t>Rams vs. Cowboys – Week 15</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-49ers-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-cowboys-2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>12/20/2026</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1:25 PM</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Rams vs. Cowboys – Week 15</t>
+          <t>Chargers vs. Chiefs – Week 17</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/rams-cowboys-2026</t>
+          <t>https://www.sofistadium.com/events/detail/chargers-chiefs-2026</t>
         </is>
       </c>
     </row>
@@ -1306,64 +1306,37 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Chargers vs. Chiefs – Week 17</t>
+          <t>Rams vs. Seahawks – Week 18</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://www.sofistadium.com/events/detail/chargers-chiefs-2026</t>
+          <t>https://www.sofistadium.com/events/detail/rams-seahawks-2027</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>02/14/2027</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
           <t>TBA</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Rams vs. Seahawks – Week 18</t>
+          <t>Super Bowl LXI</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sofistadium.com/events/detail/rams-seahawks-2027</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Sunday</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>02/14/2027</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Super Bowl LXI</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>https://www.sofistadium.com/events/detail/super-bowl-lxi</t>
         </is>
@@ -1403,7 +1376,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1415,7 +1387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1455,12 +1427,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>08/27/2026</t>
+          <t>08/28/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1470,24 +1442,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Rachmaninoff &amp; Adams</t>
+          <t>David Byrne: Who is the Sky?</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4327/2026-08-27/rachmaninoff-adams</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4328/2026-08-28/david-byrne-who-is-the-sky</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>08/28/2026</t>
+          <t>08/29/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1502,100 +1474,100 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4328/2026-08-28/david-byrne-who-is-the-sky</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4329/2026-08-29/david-byrne-who-is-the-sky</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>08/29/2026</t>
+          <t>08/30/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>6:30 PM</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>David Byrne: Who is the Sky?</t>
+          <t>Smooth Summer Jazz – The Commodores • Boney James, Sheila E.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4329/2026-08-29/david-byrne-who-is-the-sky</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4252/2026-08-30/smooth-summer-jazz</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>08/30/2026</t>
+          <t>08/31/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>6:30 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Smooth Summer Jazz – The Commodores • Boney James, Sheila E.</t>
+          <t>MUSE – Portugal. The Man, The Temper Trap</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4252/2026-08-30/smooth-summer-jazz</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4837/2026-08-31/muse</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>08/31/2026</t>
+          <t>09/01/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MUSE – Portugal. The Man, The Temper Trap</t>
+          <t>Dvořák &amp; Bruch</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4837/2026-08-31/muse</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4331/2026-09-01/dvorak-bruch</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>09/01/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1605,24 +1577,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Dvořák &amp; Bruch</t>
+          <t>Amadeusin Concert</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4331/2026-09-01/dvorak-bruch</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4332/2026-09-03/amadeus-in-concert</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1632,24 +1604,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Amadeusin Concert</t>
+          <t>Maestro of the Movies:A Tribute to John Williams</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4332/2026-09-03/amadeus-in-concert</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4333/2026-09-04/maestro-of-the-movies-a-tribute-to-john-williams</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1664,24 +1636,24 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4333/2026-09-04/maestro-of-the-movies-a-tribute-to-john-williams</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4334/2026-09-05/maestro-of-the-movies-a-tribute-to-john-williams</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>7:30 PM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1691,46 +1663,46 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4334/2026-09-05/maestro-of-the-movies-a-tribute-to-john-williams</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4335/2026-09-06/maestro-of-the-movies-a-tribute-to-john-williams</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>09/06/2026</t>
+          <t>09/08/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Maestro of the Movies:A Tribute to John Williams</t>
+          <t>Los Angeles Ballet at the Bowl</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4335/2026-09-06/maestro-of-the-movies-a-tribute-to-john-williams</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4336/2026-09-08/los-angeles-ballet-at-the-bowl</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>09/08/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1740,24 +1712,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Los Angeles Ballet at the Bowl</t>
+          <t>Buddy Guy 90 – with Special Guests Christone “Kingfish” Ingram and his Delta Jam</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4336/2026-09-08/los-angeles-ballet-at-the-bowl</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4337/2026-09-09/buddy-guy-90</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1767,24 +1739,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Buddy Guy 90 – with Special Guests Christone “Kingfish” Ingram and his Delta Jam</t>
+          <t>Ravel, Debussy &amp; Saint-Saëns</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4337/2026-09-09/buddy-guy-90</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4338/2026-09-10/ravel-debussy-saint-saens</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>09/11/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1794,24 +1766,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Ravel, Debussy &amp; Saint-Saëns</t>
+          <t>Fireworks Finale:OneRepublic</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4338/2026-09-10/ravel-debussy-saint-saens</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4339/2026-09-11/fireworks-finale-onerepublic</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>09/11/2026</t>
+          <t>09/12/2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1826,73 +1798,73 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4339/2026-09-11/fireworks-finale-onerepublic</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4340/2026-09-12/fireworks-finale-onerepublic</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>09/12/2026</t>
+          <t>09/13/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Fireworks Finale:OneRepublic</t>
+          <t>Lucy Dacus with the Hollywood Bowl Orchestra – Cat Power performing, The Greatest, KCRW Festival</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4340/2026-09-12/fireworks-finale-onerepublic</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4341/2026-09-13/lucy-dacus-with-the-hollywood-bowl-orchestra</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>09/13/2026</t>
+          <t>09/15/2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Lucy Dacus with the Hollywood Bowl Orchestra – Cat Power performing, The Greatest, KCRW Festival</t>
+          <t>Andrea Bocelli</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4341/2026-09-13/lucy-dacus-with-the-hollywood-bowl-orchestra</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4356/2026-09-15/andrea-bocelli</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>09/15/2026</t>
+          <t>09/16/2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1907,19 +1879,19 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4356/2026-09-15/andrea-bocelli</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4357/2026-09-16/andrea-bocelli</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>09/16/2026</t>
+          <t>09/18/2026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1929,24 +1901,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Andrea Bocelli</t>
+          <t>Orville Peck – Lucius, Deloyd Elze</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4357/2026-09-16/andrea-bocelli</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4355/2026-09-18/orville-peck</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>09/18/2026</t>
+          <t>09/19/2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1956,78 +1928,78 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Orville Peck – Lucius, Deloyd Elze</t>
+          <t>Squeeze – with special guest ADAM ANT, and The English Beat</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4355/2026-09-18/orville-peck</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4343/2026-09-19/squeeze</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>09/19/2026</t>
+          <t>09/20/2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>7:30 PM</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Squeeze – with special guest ADAM ANT, and The English Beat</t>
+          <t>Gregory Alan Isakov with the Hollywood Bowl Orchestra – José González</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4343/2026-09-19/squeeze</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4344/2026-09-20/gregory-alan-isakov-with-the-hollywood-bowl-orchestra</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>09/20/2026</t>
+          <t>09/23/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Gregory Alan Isakov with the Hollywood Bowl Orchestra – José González</t>
+          <t>Jazz at Lincoln Center Orchestra with Wynton Marsalis – John Coltrane 100th Celebration with Lakecia Benjamin</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4344/2026-09-20/gregory-alan-isakov-with-the-hollywood-bowl-orchestra</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4345/2026-09-23/jazz-at-lincoln-center-orchestra-with-wynton-marsalis</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>09/23/2026</t>
+          <t>09/24/2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2037,24 +2009,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Jazz at Lincoln Center Orchestra with Wynton Marsalis – John Coltrane 100th Celebration with Lakecia Benjamin</t>
+          <t>Jon Bellion</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4345/2026-09-23/jazz-at-lincoln-center-orchestra-with-wynton-marsalis</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4509/2026-09-24/jon-bellion</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>09/24/2026</t>
+          <t>09/25/2026</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2064,51 +2036,51 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Jon Bellion</t>
+          <t>The Concert:A Tribute to ABBA – MenAlive</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4509/2026-09-24/jon-bellion</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4254/2026-09-25/the-concert-a-tribute-to-abba</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>09/25/2026</t>
+          <t>09/26/2026</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>7:30 PM</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>The Concert:A Tribute to ABBA – MenAlive</t>
+          <t>Rodgers &amp; Hammerstein’s The Sound of Music Sing-A-Long</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4254/2026-09-25/the-concert-a-tribute-to-abba</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4342/2026-09-26/rodgers-hammersteins-the-sound-of-music-sing-a-long</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>09/26/2026</t>
+          <t>09/27/2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2118,51 +2090,51 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Rodgers &amp; Hammerstein’s The Sound of Music Sing-A-Long</t>
+          <t>Jon Batiste</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4342/2026-09-26/rodgers-hammersteins-the-sound-of-music-sing-a-long</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4346/2026-09-27/jon-batiste</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>09/27/2026</t>
+          <t>09/29/2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Jon Batiste</t>
+          <t>Lauren Halsey'semajendatErykah Badu and The Alchemist – with DJ Pee .Wee (Anderson .Paak), Flea, Charles Gaines Collective with Black Nile and Devin Daniels</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4346/2026-09-27/jon-batiste</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4843/2026-09-29/lauren-halseys-emajendat-erykah-badu-and-the-alchemist</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>09/29/2026</t>
+          <t>09/30/2026</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2172,51 +2144,51 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Lauren Halsey'semajendatErykah Badu and The Alchemist – with DJ Pee .Wee (Anderson .Paak), Flea, Charles Gaines Collective with Black Nile and Devin Daniels</t>
+          <t>Rubén Blades &amp; Roberto Delgado Big Band: Fotografías Tour – Silvana Estrada</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4843/2026-09-29/lauren-halseys-emajendat-erykah-badu-and-the-alchemist</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4347/2026-09-30/ruben-blades-roberto-delgado-big-band-fotografias-tour</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>09/30/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Rubén Blades &amp; Roberto Delgado Big Band: Fotografías Tour – Silvana Estrada</t>
+          <t>“The Hayley Williams Show”</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4347/2026-09-30/ruben-blades-roberto-delgado-big-band-fotografias-tour</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4885/2026-10-05/the-hayley-williams-show</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10/05/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2231,105 +2203,105 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4885/2026-10-05/the-hayley-williams-show</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4888/2026-10-06/the-hayley-williams-show</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10/06/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>7:30 PM</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>“The Hayley Williams Show”</t>
+          <t>Empire of the Sun – Polo &amp; Pan, Midnight Gen</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4888/2026-10-06/the-hayley-williams-show</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4537/2026-10-08/empire-of-the-sun</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>10/08/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Empire of the Sun – Polo &amp; Pan, Midnight Gen</t>
+          <t>Mac DeMarco</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4537/2026-10-08/empire-of-the-sun</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4363/2026-10-09/mac-demarco</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>7:30 PM</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Mac DeMarco</t>
+          <t>Jack Johnson – Hermanos Gutiérrez</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4363/2026-10-09/mac-demarco</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4256/2026-10-10/jack-johnson</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2339,46 +2311,46 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4256/2026-10-10/jack-johnson</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4257/2026-10-11/jack-johnson</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>10/11/2026</t>
+          <t>10/15/2026</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>7:30 PM</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Jack Johnson – Hermanos Gutiérrez</t>
+          <t>Cynthia Erivo</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4257/2026-10-11/jack-johnson</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4891/2026-10-15/cynthia-erivo</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>10/15/2026</t>
+          <t>10/17/2026</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2388,51 +2360,51 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Cynthia Erivo</t>
+          <t>SmartLess Live with Jason Bateman, Sean Hayes, &amp; Will Arnett</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4891/2026-10-15/cynthia-erivo</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4841/2026-10-17/smartless-live-with-jason-bateman-sean-hayes-will-arnett</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>10/17/2026</t>
+          <t>10/21/2026</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>SmartLess Live with Jason Bateman, Sean Hayes, &amp; Will Arnett</t>
+          <t>My Chemical Romance</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4841/2026-10-17/smartless-live-with-jason-bateman-sean-hayes-will-arnett</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4231/2026-10-21/my-chemical-romance</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>10/21/2026</t>
+          <t>10/23/2026</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2447,19 +2419,19 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4231/2026-10-21/my-chemical-romance</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4232/2026-10-23/my-chemical-romance</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>10/23/2026</t>
+          <t>10/24/2026</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2474,46 +2446,46 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4232/2026-10-23/my-chemical-romance</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4233/2026-10-24/my-chemical-romance</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>10/24/2026</t>
+          <t>10/30/2026</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>My Chemical Romance</t>
+          <t>My Chemical Romance – The Used</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4233/2026-10-24/my-chemical-romance</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4263/2026-10-30/my-chemical-romance</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>10/30/2026</t>
+          <t>10/31/2026</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2523,12 +2495,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>My Chemical Romance – The Used</t>
+          <t>My Chemical Romance – Thrice</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4263/2026-10-30/my-chemical-romance</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4264/2026-10-31/my-chemical-romance</t>
         </is>
       </c>
     </row>
@@ -2540,7 +2512,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>10/31/2026</t>
+          <t>11/07/2026</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2550,51 +2522,51 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>My Chemical Romance – Thrice</t>
+          <t>Jimmy Eat WorldThe Format – The Linda Lindas</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4264/2026-10-31/my-chemical-romance</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4898/2026-11-07/jimmy-eat-world-the-format</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>11/07/2026</t>
+          <t>11/08/2026</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>7:30 PM</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Jimmy Eat WorldThe Format – The Linda Lindas</t>
+          <t>Ms. Lauryn Hill &amp; Wyclef Jean</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4898/2026-11-07/jimmy-eat-world-the-format</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4899/2026-11-08/ms-lauryn-hill-wyclef-jean</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>11/08/2026</t>
+          <t>11/18/2026</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2604,24 +2576,24 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Ms. Lauryn Hill &amp; Wyclef Jean</t>
+          <t>Jonas Brothers – All Time Low, Magnus Ferrell</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4899/2026-11-08/ms-lauryn-hill-wyclef-jean</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4902/2026-11-18/jonas-brothers</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>11/18/2026</t>
+          <t>11/19/2026</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2636,59 +2608,32 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4902/2026-11-18/jonas-brothers</t>
+          <t>https://www.hollywoodbowl.com/events/performances/4904/2026-11-19/jonas-brothers</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>11/19/2026</t>
+          <t>11/21/2026</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>7:30 PM</t>
+          <t>8:00 PM</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Jonas Brothers – All Time Low, Magnus Ferrell</t>
+          <t>Steve Lacy</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>https://www.hollywoodbowl.com/events/performances/4904/2026-11-19/jonas-brothers</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>11/21/2026</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>8:00 PM</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Steve Lacy</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>https://www.hollywoodbowl.com/events/performances/4900/2026-11-21/steve-lacy</t>
         </is>
@@ -2741,7 +2686,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -26737,13 +26681,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -26777,12 +26721,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>09/02/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -26792,12 +26736,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>LA Galaxy vs New England Revolution</t>
+          <t>Leagues Cup: Club América vs. C.F. Monterrey</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-new-england-revolution</t>
+          <t>https://www.dignityhealthsportspark.com/events/detail/leagues-cup-club-america-vs-c</t>
         </is>
       </c>
     </row>
@@ -26809,7 +26753,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>09/12/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -26819,12 +26763,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>LA Galaxy vs Seattle Sounders</t>
+          <t>LA Galaxy vs New England Revolution</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-seattle-sounders</t>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-new-england-revolution</t>
         </is>
       </c>
     </row>
@@ -26836,7 +26780,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>09/19/2026</t>
+          <t>09/12/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -26846,12 +26790,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SuperMotocross Playoff Round 2</t>
+          <t>LA Galaxy vs Seattle Sounders</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/supermotocross</t>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-seattle-sounders</t>
         </is>
       </c>
     </row>
@@ -26863,7 +26807,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>09/26/2026</t>
+          <t>09/19/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -26873,24 +26817,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>LA Galaxy vs Colorado Rapids</t>
+          <t>SuperMotocross Playoff Round 2</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-colorado-rapids</t>
+          <t>https://www.dignityhealthsportspark.com/events/detail/supermotocross</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10/14/2026</t>
+          <t>09/26/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -26900,24 +26844,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>LA Galaxy vs Portland Timbers FC</t>
+          <t>LA Galaxy vs Colorado Rapids</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-portland-timbers</t>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-colorado-rapids</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10/17/2026</t>
+          <t>10/14/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -26927,12 +26871,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>LA Galaxy vs San Diego FC</t>
+          <t>LA Galaxy vs Portland Timbers FC</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-san-diego-fc</t>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-portland-timbers</t>
         </is>
       </c>
     </row>
@@ -26944,7 +26888,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>10/31/2026</t>
+          <t>10/17/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -26954,37 +26898,64 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>LA Galaxy vs Austin FC</t>
+          <t>LA Galaxy vs San Diego FC</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-austin-fc</t>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-san-diego-fc</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10/31/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>LA Galaxy vs Austin FC</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dignityhealthsportspark.com/events/detail/la-galaxy-vs-austin-fc</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>11/01/2026</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>TBA</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Angel City FC vs Boston Legacy FC</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>https://www.dignityhealthsportspark.com/events/detail/angel-city-fc-vs-boston-legacy-fc</t>
         </is>
@@ -27000,6 +26971,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>